<commit_message>
Penn and Stanford S&W: assume 35% fringe benefit rate; keep CDS student count for Northeastern
S&W = audited combined salaries and benefits / 1.35 for Penn and Stanford (Penn $278K, Stanford $463K per
student, flagged est.). The fringe rate is a single input cell in the backup workbook with sensitivity to the
Form 990 share and the original 72.8%. Northeastern student count stays on the Common Data Set (39,774).

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCNX7EgSWHMHv9UtVBoXog
</commit_message>
<xml_diff>
--- a/nu-peer-slides/NU_peer_slides_backup.xlsx
+++ b/nu-peer-slides/NU_peer_slides_backup.xlsx
@@ -109,7 +109,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="28">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -132,6 +132,7 @@
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="1" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="9" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="3" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="2" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -615,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -671,7 +672,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Download 'fy25 Harvard Financial Report' from finance.harvard.edu (Financial Reports) in a browser and upload; I will add Harvard to the chart.</t>
+          <t>Download the FY25 Harvard Financial Report from finance.harvard.edu (Financial Reports) in a browser and upload; I will add Harvard to the chart.</t>
         </is>
       </c>
     </row>
@@ -683,17 +684,17 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Northeastern official student count for FY25 analysis</t>
+          <t>Penn and Stanford salaries and wages (optional)</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>CDS 39,774 vs IPEDS-style 32,553 vs Facts and Figures 48,812 (S&amp;W per student $26K / $32K / $21K).</t>
+          <t>Estimated at combined salaries+benefits / 1.35 (35% fringe rate, per Northeastern). Audited statements combine the two lines; Form 990s cover a narrower scope.</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>Confirm with University Decision Support which count leadership uses; I will relabel.</t>
+          <t>If either finance office can supply consolidated S&amp;W, replace the grey estimate.</t>
         </is>
       </c>
     </row>
@@ -705,17 +706,17 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Penn and Stanford salaries and wages</t>
+          <t>Princeton Common Data Set 2024-25 (optional)</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>Audited statements combine salaries and benefits; Form 990s cover a narrower scope than the consolidated statements.</t>
+          <t>ir.princeton.edu is behind a bot challenge; the Treasurer's report count (9,050) is used.</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
-          <t>If Penn / Stanford finance offices can supply consolidated S&amp;W, replace the grey estimates.</t>
+          <t>Upload the CDS PDF if you want the same instrument as the other schools.</t>
         </is>
       </c>
     </row>
@@ -727,39 +728,17 @@
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Princeton Common Data Set 2024-25</t>
+          <t>IPEDS fall 2024 enrollment and FY24 finance files</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>ir.princeton.edu is behind a bot challenge; the Treasurer's report count (9,050) is used.</t>
+          <t>Not yet posted on the IPEDS data center.</t>
         </is>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
-          <t>Optional: upload the CDS PDF.</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>IPEDS fall 2024 enrollment and FY24 finance files</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>Not yet posted on the IPEDS data center.</t>
-        </is>
-      </c>
-      <c r="D8" s="4" t="inlineStr">
-        <is>
-          <t>Re-check when posted; IPEDS fall enrollment would give one government-standard definition.</t>
+          <t>Re-check when posted.</t>
         </is>
       </c>
     </row>
@@ -68957,7 +68936,22 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Core operating expenses = total operating expenses - depreciation - amortization - interest. S&amp;W basis: audited line, Form 990 / MD&amp;A chart, or ESTIMATE (Penn, Stanford). Students = fall 2024 total enrollment.</t>
+          <t>Core operating expenses = total operating expenses - depreciation - amortization - interest. S&amp;W basis: audited line, Form 990 / MD&amp;A chart, or ESTIMATE (Penn, Stanford: 35% assumed fringe rate). Students = fall 2024 total enrollment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Assumed fringe benefit rate (benefits / S&amp;W) for Penn and Stanford</t>
+        </is>
+      </c>
+      <c r="E3" s="18" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="F3" s="17" t="inlineStr">
+        <is>
+          <t>&lt;- input: S&amp;W = combined salaries + benefits / (1 + rate). Change it and the estimates, slide-3 inputs and sensitivities update here.</t>
         </is>
       </c>
     </row>
@@ -69069,7 +69063,7 @@
           <t>June 30, 2025</t>
         </is>
       </c>
-      <c r="C5" s="18" t="n">
+      <c r="C5" s="19" t="n">
         <v>515800000</v>
       </c>
       <c r="D5" s="9" t="inlineStr">
@@ -69077,24 +69071,24 @@
           <t>audited line</t>
         </is>
       </c>
-      <c r="E5" s="18">
+      <c r="E5" s="19">
         <f>C5+123330000</f>
         <v/>
       </c>
-      <c r="H5" s="18" t="n">
+      <c r="H5" s="19" t="n">
         <v>1087937000</v>
       </c>
-      <c r="I5" s="18" t="n">
+      <c r="I5" s="19" t="n">
         <v>82255000</v>
       </c>
-      <c r="K5" s="18" t="n">
+      <c r="K5" s="19" t="n">
         <v>45396000</v>
       </c>
-      <c r="L5" s="18">
+      <c r="L5" s="19">
         <f>H5-I5-J5-K5</f>
         <v/>
       </c>
-      <c r="M5" s="18" t="n">
+      <c r="M5" s="19" t="n">
         <v>8961</v>
       </c>
       <c r="N5" s="11">
@@ -69105,11 +69099,11 @@
         <f>L5/M5</f>
         <v/>
       </c>
-      <c r="P5" s="19">
+      <c r="P5" s="20">
         <f>C5/L5</f>
         <v/>
       </c>
-      <c r="Q5" s="20">
+      <c r="Q5" s="21">
         <f>O5*P5-N5</f>
         <v/>
       </c>
@@ -69135,7 +69129,7 @@
           <t>June 30, 2025</t>
         </is>
       </c>
-      <c r="C6" s="18" t="n">
+      <c r="C6" s="19" t="n">
         <v>804000000</v>
       </c>
       <c r="D6" s="9" t="inlineStr">
@@ -69143,23 +69137,23 @@
           <t>MD&amp;A expense chart</t>
         </is>
       </c>
-      <c r="E6" s="18" t="n">
+      <c r="E6" s="19" t="n">
         <v>976417000</v>
       </c>
-      <c r="H6" s="18" t="n">
+      <c r="H6" s="19" t="n">
         <v>1799663000</v>
       </c>
-      <c r="I6" s="18" t="n">
+      <c r="I6" s="19" t="n">
         <v>116913000</v>
       </c>
-      <c r="K6" s="18" t="n">
+      <c r="K6" s="19" t="n">
         <v>30063000</v>
       </c>
-      <c r="L6" s="18">
+      <c r="L6" s="19">
         <f>H6-I6-J6-K6</f>
         <v/>
       </c>
-      <c r="M6" s="18" t="n">
+      <c r="M6" s="19" t="n">
         <v>13575</v>
       </c>
       <c r="N6" s="11">
@@ -69170,11 +69164,11 @@
         <f>L6/M6</f>
         <v/>
       </c>
-      <c r="P6" s="19">
+      <c r="P6" s="20">
         <f>C6/L6</f>
         <v/>
       </c>
-      <c r="Q6" s="20">
+      <c r="Q6" s="21">
         <f>O6*P6-N6</f>
         <v/>
       </c>
@@ -69200,7 +69194,7 @@
           <t>August 31, 2025</t>
         </is>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="19">
         <f>F7</f>
         <v/>
       </c>
@@ -69209,29 +69203,29 @@
           <t>Form 990 (ties to audited)</t>
         </is>
       </c>
-      <c r="E7" s="18" t="n">
+      <c r="E7" s="19" t="n">
         <v>1997951000</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="19" t="n">
         <v>1556522638</v>
       </c>
-      <c r="G7" s="18" t="n">
+      <c r="G7" s="19" t="n">
         <v>1997950859</v>
       </c>
-      <c r="H7" s="18" t="n">
+      <c r="H7" s="19" t="n">
         <v>3607255000</v>
       </c>
-      <c r="I7" s="18" t="n">
+      <c r="I7" s="19" t="n">
         <v>216713000</v>
       </c>
-      <c r="K7" s="18" t="n">
+      <c r="K7" s="19" t="n">
         <v>99478000</v>
       </c>
-      <c r="L7" s="18">
+      <c r="L7" s="19">
         <f>H7-I7-J7-K7</f>
         <v/>
       </c>
-      <c r="M7" s="18" t="n">
+      <c r="M7" s="19" t="n">
         <v>23431</v>
       </c>
       <c r="N7" s="11">
@@ -69242,11 +69236,11 @@
         <f>L7/M7</f>
         <v/>
       </c>
-      <c r="P7" s="19">
+      <c r="P7" s="20">
         <f>C7/L7</f>
         <v/>
       </c>
-      <c r="Q7" s="20">
+      <c r="Q7" s="21">
         <f>O7*P7-N7</f>
         <v/>
       </c>
@@ -69272,7 +69266,7 @@
           <t>June 30, 2025</t>
         </is>
       </c>
-      <c r="C8" s="18" t="n">
+      <c r="C8" s="19" t="n">
         <v>1162823000</v>
       </c>
       <c r="D8" s="9" t="inlineStr">
@@ -69280,24 +69274,24 @@
           <t>audited line</t>
         </is>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="19">
         <f>C8+351760000</f>
         <v/>
       </c>
-      <c r="H8" s="18" t="n">
+      <c r="H8" s="19" t="n">
         <v>2744548000</v>
       </c>
-      <c r="I8" s="18" t="n">
+      <c r="I8" s="19" t="n">
         <v>231467000</v>
       </c>
-      <c r="K8" s="18" t="n">
+      <c r="K8" s="19" t="n">
         <v>221826000</v>
       </c>
-      <c r="L8" s="18">
+      <c r="L8" s="19">
         <f>H8-I8-J8-K8</f>
         <v/>
       </c>
-      <c r="M8" s="18" t="n">
+      <c r="M8" s="19" t="n">
         <v>9050</v>
       </c>
       <c r="N8" s="11">
@@ -69308,11 +69302,11 @@
         <f>L8/M8</f>
         <v/>
       </c>
-      <c r="P8" s="19">
+      <c r="P8" s="20">
         <f>C8/L8</f>
         <v/>
       </c>
-      <c r="Q8" s="20">
+      <c r="Q8" s="21">
         <f>O8*P8-N8</f>
         <v/>
       </c>
@@ -69343,7 +69337,7 @@
           <t>pending</t>
         </is>
       </c>
-      <c r="M9" s="18" t="n">
+      <c r="M9" s="19" t="n">
         <v>21189</v>
       </c>
       <c r="S9" s="4" t="inlineStr">
@@ -69363,7 +69357,7 @@
           <t>June 30, 2025</t>
         </is>
       </c>
-      <c r="C10" s="18" t="n">
+      <c r="C10" s="19" t="n">
         <v>2737371000</v>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -69371,21 +69365,21 @@
           <t>audited line</t>
         </is>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="19">
         <f>C10+861635000</f>
         <v/>
       </c>
-      <c r="H10" s="18" t="n">
+      <c r="H10" s="19" t="n">
         <v>5807911000</v>
       </c>
-      <c r="I10" s="18" t="n">
+      <c r="I10" s="19" t="n">
         <v>504923000</v>
       </c>
-      <c r="L10" s="18">
+      <c r="L10" s="19">
         <f>H10-I10-J10-K10</f>
         <v/>
       </c>
-      <c r="M10" s="18" t="n">
+      <c r="M10" s="19" t="n">
         <v>15564</v>
       </c>
       <c r="N10" s="11">
@@ -69396,11 +69390,11 @@
         <f>L10/M10</f>
         <v/>
       </c>
-      <c r="P10" s="19">
+      <c r="P10" s="20">
         <f>C10/L10</f>
         <v/>
       </c>
-      <c r="Q10" s="20">
+      <c r="Q10" s="21">
         <f>O10*P10-N10</f>
         <v/>
       </c>
@@ -69426,7 +69420,7 @@
           <t>June 30, 2025</t>
         </is>
       </c>
-      <c r="C11" s="18" t="n">
+      <c r="C11" s="19" t="n">
         <v>3678678000</v>
       </c>
       <c r="D11" s="9" t="inlineStr">
@@ -69434,23 +69428,23 @@
           <t>audited line</t>
         </is>
       </c>
-      <c r="E11" s="18" t="n">
+      <c r="E11" s="19" t="n">
         <v>4517817000</v>
       </c>
-      <c r="H11" s="18" t="n">
+      <c r="H11" s="19" t="n">
         <v>8283042000</v>
       </c>
-      <c r="I11" s="18" t="n">
+      <c r="I11" s="19" t="n">
         <v>401386000</v>
       </c>
-      <c r="K11" s="18" t="n">
+      <c r="K11" s="19" t="n">
         <v>215170000</v>
       </c>
-      <c r="L11" s="18">
+      <c r="L11" s="19">
         <f>H11-I11-J11-K11</f>
         <v/>
       </c>
-      <c r="M11" s="18" t="n">
+      <c r="M11" s="19" t="n">
         <v>16221</v>
       </c>
       <c r="N11" s="11">
@@ -69461,11 +69455,11 @@
         <f>L11/M11</f>
         <v/>
       </c>
-      <c r="P11" s="19">
+      <c r="P11" s="20">
         <f>C11/L11</f>
         <v/>
       </c>
-      <c r="Q11" s="20">
+      <c r="Q11" s="21">
         <f>O11*P11-N11</f>
         <v/>
       </c>
@@ -69491,7 +69485,7 @@
           <t>June 30, 2025</t>
         </is>
       </c>
-      <c r="C12" s="18" t="n">
+      <c r="C12" s="19" t="n">
         <v>5041664000</v>
       </c>
       <c r="D12" s="9" t="inlineStr">
@@ -69499,23 +69493,23 @@
           <t>audited line</t>
         </is>
       </c>
-      <c r="E12" s="18" t="n">
+      <c r="E12" s="19" t="n">
         <v>6230712000</v>
       </c>
-      <c r="H12" s="18" t="n">
+      <c r="H12" s="19" t="n">
         <v>10953208000</v>
       </c>
-      <c r="I12" s="18" t="n">
+      <c r="I12" s="19" t="n">
         <v>471677000</v>
       </c>
-      <c r="K12" s="18" t="n">
+      <c r="K12" s="19" t="n">
         <v>161512000</v>
       </c>
-      <c r="L12" s="18">
+      <c r="L12" s="19">
         <f>H12-I12-J12-K12</f>
         <v/>
       </c>
-      <c r="M12" s="18" t="n">
+      <c r="M12" s="19" t="n">
         <v>17499</v>
       </c>
       <c r="N12" s="11">
@@ -69526,11 +69520,11 @@
         <f>L12/M12</f>
         <v/>
       </c>
-      <c r="P12" s="19">
+      <c r="P12" s="20">
         <f>C12/L12</f>
         <v/>
       </c>
-      <c r="Q12" s="20">
+      <c r="Q12" s="21">
         <f>O12*P12-N12</f>
         <v/>
       </c>
@@ -69556,7 +69550,7 @@
           <t>August 31, 2025</t>
         </is>
       </c>
-      <c r="C13" s="18" t="n">
+      <c r="C13" s="19" t="n">
         <v>5265449000</v>
       </c>
       <c r="D13" s="9" t="inlineStr">
@@ -69564,24 +69558,24 @@
           <t>audited line</t>
         </is>
       </c>
-      <c r="E13" s="18">
+      <c r="E13" s="19">
         <f>C13+1259151000</f>
         <v/>
       </c>
-      <c r="H13" s="18" t="n">
+      <c r="H13" s="19" t="n">
         <v>10577959000</v>
       </c>
-      <c r="I13" s="18" t="n">
+      <c r="I13" s="19" t="n">
         <v>379158000</v>
       </c>
-      <c r="K13" s="18" t="n">
+      <c r="K13" s="19" t="n">
         <v>113892000</v>
       </c>
-      <c r="L13" s="18">
+      <c r="L13" s="19">
         <f>H13-I13-J13-K13</f>
         <v/>
       </c>
-      <c r="M13" s="18" t="n">
+      <c r="M13" s="19" t="n">
         <v>15179</v>
       </c>
       <c r="N13" s="11">
@@ -69592,11 +69586,11 @@
         <f>L13/M13</f>
         <v/>
       </c>
-      <c r="P13" s="19">
+      <c r="P13" s="20">
         <f>C13/L13</f>
         <v/>
       </c>
-      <c r="Q13" s="20">
+      <c r="Q13" s="21">
         <f>O13*P13-N13</f>
         <v/>
       </c>
@@ -69622,38 +69616,38 @@
           <t>June 30, 2025</t>
         </is>
       </c>
-      <c r="C14" s="18">
-        <f>E14*F14/G14</f>
-        <v/>
-      </c>
-      <c r="D14" s="21" t="inlineStr">
-        <is>
-          <t>ESTIMATE (990 share x audited combined)</t>
-        </is>
-      </c>
-      <c r="E14" s="18" t="n">
+      <c r="C14" s="19">
+        <f>E14/(1+$E$3)</f>
+        <v/>
+      </c>
+      <c r="D14" s="22" t="inlineStr">
+        <is>
+          <t>ESTIMATE (combined / (1 + fringe rate))</t>
+        </is>
+      </c>
+      <c r="E14" s="19" t="n">
         <v>9019270000</v>
       </c>
-      <c r="F14" s="18" t="n">
+      <c r="F14" s="19" t="n">
         <v>4515553000</v>
       </c>
-      <c r="G14" s="18" t="n">
+      <c r="G14" s="19" t="n">
         <v>5886033000</v>
       </c>
-      <c r="H14" s="18" t="n">
+      <c r="H14" s="19" t="n">
         <v>16445321000</v>
       </c>
-      <c r="I14" s="18" t="n">
+      <c r="I14" s="19" t="n">
         <v>686510000</v>
       </c>
-      <c r="K14" s="18" t="n">
+      <c r="K14" s="19" t="n">
         <v>133923000</v>
       </c>
-      <c r="L14" s="18">
+      <c r="L14" s="19">
         <f>H14-I14-J14-K14</f>
         <v/>
       </c>
-      <c r="M14" s="18" t="n">
+      <c r="M14" s="19" t="n">
         <v>24023</v>
       </c>
       <c r="N14" s="11">
@@ -69664,11 +69658,11 @@
         <f>L14/M14</f>
         <v/>
       </c>
-      <c r="P14" s="19">
+      <c r="P14" s="20">
         <f>C14/L14</f>
         <v/>
       </c>
-      <c r="Q14" s="20">
+      <c r="Q14" s="21">
         <f>O14*P14-N14</f>
         <v/>
       </c>
@@ -69679,7 +69673,7 @@
       </c>
       <c r="S14" s="4" t="inlineStr">
         <is>
-          <t>Statements show 'compensation and benefits' combined only. S&amp;W ESTIMATED = combined x Form 990 S&amp;W share (990 covers a narrower scope than the consolidated statements). D&amp;A one line.</t>
+          <t>Statements show 'compensation and benefits' combined only. S&amp;W ESTIMATED = combined / (1 + 35% assumed fringe rate), per Northeastern. Columns F-G (Form 990, narrower scope) are shown for reference only. D&amp;A one line.</t>
         </is>
       </c>
     </row>
@@ -69694,38 +69688,38 @@
           <t>August 31, 2025</t>
         </is>
       </c>
-      <c r="C15" s="18">
-        <f>E15*F15/G15</f>
-        <v/>
-      </c>
-      <c r="D15" s="21" t="inlineStr">
-        <is>
-          <t>ESTIMATE (990 share x audited combined)</t>
-        </is>
-      </c>
-      <c r="E15" s="18" t="n">
+      <c r="C15" s="19">
+        <f>E15/(1+$E$3)</f>
+        <v/>
+      </c>
+      <c r="D15" s="22" t="inlineStr">
+        <is>
+          <t>ESTIMATE (combined / (1 + fringe rate))</t>
+        </is>
+      </c>
+      <c r="E15" s="19" t="n">
         <v>11647045000</v>
       </c>
-      <c r="F15" s="18" t="n">
+      <c r="F15" s="19" t="n">
         <v>4781181437</v>
       </c>
-      <c r="G15" s="18" t="n">
+      <c r="G15" s="19" t="n">
         <v>5963697901</v>
       </c>
-      <c r="H15" s="18" t="n">
+      <c r="H15" s="19" t="n">
         <v>18935447000</v>
       </c>
-      <c r="I15" s="18" t="n">
+      <c r="I15" s="19" t="n">
         <v>930917000</v>
       </c>
-      <c r="K15" s="18" t="n">
+      <c r="K15" s="19" t="n">
         <v>278763000</v>
       </c>
-      <c r="L15" s="18">
+      <c r="L15" s="19">
         <f>H15-I15-J15-K15</f>
         <v/>
       </c>
-      <c r="M15" s="18" t="n">
+      <c r="M15" s="19" t="n">
         <v>18625</v>
       </c>
       <c r="N15" s="11">
@@ -69736,11 +69730,11 @@
         <f>L15/M15</f>
         <v/>
       </c>
-      <c r="P15" s="19">
+      <c r="P15" s="20">
         <f>C15/L15</f>
         <v/>
       </c>
-      <c r="Q15" s="20">
+      <c r="Q15" s="21">
         <f>O15*P15-N15</f>
         <v/>
       </c>
@@ -69751,7 +69745,7 @@
       </c>
       <c r="S15" s="4" t="inlineStr">
         <is>
-          <t>Statements show salaries and benefits combined only. S&amp;W ESTIMATED = combined x Form 990 S&amp;W share. Interest is net and embedded in other operating expenses. Includes SLAC and the hospitals.</t>
+          <t>Statements show salaries and benefits combined only. S&amp;W ESTIMATED = combined / (1 + 35% assumed fringe rate), per Northeastern. Columns F-G (Form 990, narrower scope) are reference only. Interest is net and embedded in other operating expenses. Includes SLAC and the hospitals.</t>
         </is>
       </c>
     </row>
@@ -69766,7 +69760,7 @@
           <t>June 30, 2025</t>
         </is>
       </c>
-      <c r="C16" s="18">
+      <c r="C16" s="19">
         <f>F16</f>
         <v/>
       </c>
@@ -69775,29 +69769,29 @@
           <t>Form 990 (96.8% of audited combined)</t>
         </is>
       </c>
-      <c r="E16" s="18" t="n">
+      <c r="E16" s="19" t="n">
         <v>1341049000</v>
       </c>
-      <c r="F16" s="18" t="n">
+      <c r="F16" s="19" t="n">
         <v>1045135178</v>
       </c>
-      <c r="G16" s="18" t="n">
+      <c r="G16" s="19" t="n">
         <v>1297581752</v>
       </c>
-      <c r="H16" s="18" t="n">
+      <c r="H16" s="19" t="n">
         <v>2388249000</v>
       </c>
-      <c r="I16" s="18" t="n">
+      <c r="I16" s="19" t="n">
         <v>151250000</v>
       </c>
-      <c r="K16" s="18" t="n">
+      <c r="K16" s="19" t="n">
         <v>49862000</v>
       </c>
-      <c r="L16" s="18">
+      <c r="L16" s="19">
         <f>H16-I16-J16-K16</f>
         <v/>
       </c>
-      <c r="M16" s="18" t="n">
+      <c r="M16" s="19" t="n">
         <v>39774</v>
       </c>
       <c r="N16" s="11">
@@ -69808,11 +69802,11 @@
         <f>L16/M16</f>
         <v/>
       </c>
-      <c r="P16" s="19">
+      <c r="P16" s="20">
         <f>C16/L16</f>
         <v/>
       </c>
-      <c r="Q16" s="20">
+      <c r="Q16" s="21">
         <f>O16*P16-N16</f>
         <v/>
       </c>
@@ -69838,7 +69832,7 @@
           <t>June 30, 2025</t>
         </is>
       </c>
-      <c r="C17" s="18" t="n">
+      <c r="C17" s="19" t="n">
         <v>1238476000</v>
       </c>
       <c r="D17" s="9" t="inlineStr">
@@ -69846,24 +69840,24 @@
           <t>audited line</t>
         </is>
       </c>
-      <c r="E17" s="18">
+      <c r="E17" s="19">
         <f>C17+389796000</f>
         <v/>
       </c>
-      <c r="H17" s="18" t="n">
+      <c r="H17" s="19" t="n">
         <v>2719848000</v>
       </c>
-      <c r="I17" s="18" t="n">
+      <c r="I17" s="19" t="n">
         <v>160697000</v>
       </c>
-      <c r="K17" s="18" t="n">
+      <c r="K17" s="19" t="n">
         <v>81689000</v>
       </c>
-      <c r="L17" s="18">
+      <c r="L17" s="19">
         <f>H17-I17-J17-K17</f>
         <v/>
       </c>
-      <c r="M17" s="18" t="n">
+      <c r="M17" s="19" t="n">
         <v>37737</v>
       </c>
       <c r="N17" s="11">
@@ -69874,11 +69868,11 @@
         <f>L17/M17</f>
         <v/>
       </c>
-      <c r="P17" s="19">
+      <c r="P17" s="20">
         <f>C17/L17</f>
         <v/>
       </c>
-      <c r="Q17" s="20">
+      <c r="Q17" s="21">
         <f>O17*P17-N17</f>
         <v/>
       </c>
@@ -69904,7 +69898,7 @@
           <t>June 30, 2025</t>
         </is>
       </c>
-      <c r="C18" s="18" t="n">
+      <c r="C18" s="19" t="n">
         <v>2090862000</v>
       </c>
       <c r="D18" s="9" t="inlineStr">
@@ -69912,23 +69906,23 @@
           <t>audited line</t>
         </is>
       </c>
-      <c r="E18" s="18" t="n">
+      <c r="E18" s="19" t="n">
         <v>2796822000</v>
       </c>
-      <c r="H18" s="18" t="n">
+      <c r="H18" s="19" t="n">
         <v>5117184000</v>
       </c>
-      <c r="I18" s="18" t="n">
+      <c r="I18" s="19" t="n">
         <v>289575000</v>
       </c>
-      <c r="K18" s="18" t="n">
+      <c r="K18" s="19" t="n">
         <v>170489000</v>
       </c>
-      <c r="L18" s="18">
+      <c r="L18" s="19">
         <f>H18-I18-J18-K18</f>
         <v/>
       </c>
-      <c r="M18" s="18" t="n">
+      <c r="M18" s="19" t="n">
         <v>11886</v>
       </c>
       <c r="N18" s="11">
@@ -69939,11 +69933,11 @@
         <f>L18/M18</f>
         <v/>
       </c>
-      <c r="P18" s="19">
+      <c r="P18" s="20">
         <f>C18/L18</f>
         <v/>
       </c>
-      <c r="Q18" s="20">
+      <c r="Q18" s="21">
         <f>O18*P18-N18</f>
         <v/>
       </c>
@@ -69972,7 +69966,7 @@
         <f>MEDIAN(O5:O18)</f>
         <v/>
       </c>
-      <c r="P20" s="22">
+      <c r="P20" s="23">
         <f>MEDIAN(P5:P18)</f>
         <v/>
       </c>
@@ -69994,7 +69988,7 @@
           <t>Northeastern S&amp;W per student as % of peer median</t>
         </is>
       </c>
-      <c r="N22" s="23">
+      <c r="N22" s="24">
         <f>N16/N20</f>
         <v/>
       </c>
@@ -70010,7 +70004,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H32"/>
+  <dimension ref="A1:J43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -70074,7 +70068,7 @@
           <t>Common Data Set 2024-25 (used on slide)</t>
         </is>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="19" t="n">
         <v>39774</v>
       </c>
       <c r="C6" s="11">
@@ -70097,7 +70091,7 @@
           <t>IPEDS-style headcount (College Navigator fall 2024)</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="19" t="n">
         <v>32553</v>
       </c>
       <c r="C7" s="11">
@@ -70120,7 +70114,7 @@
           <t>Northeastern Facts and Figures fall 2024</t>
         </is>
       </c>
-      <c r="B8" s="18" t="n">
+      <c r="B8" s="19" t="n">
         <v>48812</v>
       </c>
       <c r="C8" s="11">
@@ -70192,11 +70186,11 @@
           <t>Rice</t>
         </is>
       </c>
-      <c r="B12" s="18">
+      <c r="B12" s="19">
         <f>S3_FY25!M5</f>
         <v/>
       </c>
-      <c r="C12" s="18" t="n">
+      <c r="C12" s="19" t="n">
         <v>8556</v>
       </c>
       <c r="D12" s="11">
@@ -70215,7 +70209,7 @@
         <f>RANK(E12,E$12:E$24,1)</f>
         <v/>
       </c>
-      <c r="H12" s="24">
+      <c r="H12" s="25">
         <f>(C12/B12-1)*100</f>
         <v/>
       </c>
@@ -70226,11 +70220,11 @@
           <t>Vanderbilt</t>
         </is>
       </c>
-      <c r="B13" s="18">
+      <c r="B13" s="19">
         <f>S3_FY25!M6</f>
         <v/>
       </c>
-      <c r="C13" s="18" t="n">
+      <c r="C13" s="19" t="n">
         <v>13456</v>
       </c>
       <c r="D13" s="11">
@@ -70249,7 +70243,7 @@
         <f>RANK(E13,E$12:E$24,1)</f>
         <v/>
       </c>
-      <c r="H13" s="24">
+      <c r="H13" s="25">
         <f>(C13/B13-1)*100</f>
         <v/>
       </c>
@@ -70260,11 +70254,11 @@
           <t>Northwestern</t>
         </is>
       </c>
-      <c r="B14" s="18">
+      <c r="B14" s="19">
         <f>S3_FY25!M7</f>
         <v/>
       </c>
-      <c r="C14" s="18" t="n">
+      <c r="C14" s="19" t="n">
         <v>23203</v>
       </c>
       <c r="D14" s="11">
@@ -70283,7 +70277,7 @@
         <f>RANK(E14,E$12:E$24,1)</f>
         <v/>
       </c>
-      <c r="H14" s="24">
+      <c r="H14" s="25">
         <f>(C14/B14-1)*100</f>
         <v/>
       </c>
@@ -70294,11 +70288,11 @@
           <t>Princeton</t>
         </is>
       </c>
-      <c r="B15" s="18">
+      <c r="B15" s="19">
         <f>S3_FY25!M8</f>
         <v/>
       </c>
-      <c r="C15" s="18" t="n">
+      <c r="C15" s="19" t="n">
         <v>8922</v>
       </c>
       <c r="D15" s="11">
@@ -70317,7 +70311,7 @@
         <f>RANK(E15,E$12:E$24,1)</f>
         <v/>
       </c>
-      <c r="H15" s="24">
+      <c r="H15" s="25">
         <f>(C15/B15-1)*100</f>
         <v/>
       </c>
@@ -70328,11 +70322,11 @@
           <t>Yale</t>
         </is>
       </c>
-      <c r="B16" s="18">
+      <c r="B16" s="19">
         <f>S3_FY25!M10</f>
         <v/>
       </c>
-      <c r="C16" s="18" t="n">
+      <c r="C16" s="19" t="n">
         <v>15081</v>
       </c>
       <c r="D16" s="11">
@@ -70351,7 +70345,7 @@
         <f>RANK(E16,E$12:E$24,1)</f>
         <v/>
       </c>
-      <c r="H16" s="24">
+      <c r="H16" s="25">
         <f>(C16/B16-1)*100</f>
         <v/>
       </c>
@@ -70362,11 +70356,11 @@
           <t>Chicago</t>
         </is>
       </c>
-      <c r="B17" s="18">
+      <c r="B17" s="19">
         <f>S3_FY25!M11</f>
         <v/>
       </c>
-      <c r="C17" s="18" t="n">
+      <c r="C17" s="19" t="n">
         <v>18339</v>
       </c>
       <c r="D17" s="11">
@@ -70385,7 +70379,7 @@
         <f>RANK(E17,E$12:E$24,1)</f>
         <v/>
       </c>
-      <c r="H17" s="24">
+      <c r="H17" s="25">
         <f>(C17/B17-1)*100</f>
         <v/>
       </c>
@@ -70396,11 +70390,11 @@
           <t>Duke</t>
         </is>
       </c>
-      <c r="B18" s="18">
+      <c r="B18" s="19">
         <f>S3_FY25!M12</f>
         <v/>
       </c>
-      <c r="C18" s="18" t="n">
+      <c r="C18" s="19" t="n">
         <v>17112</v>
       </c>
       <c r="D18" s="11">
@@ -70419,7 +70413,7 @@
         <f>RANK(E18,E$12:E$24,1)</f>
         <v/>
       </c>
-      <c r="H18" s="24">
+      <c r="H18" s="25">
         <f>(C18/B18-1)*100</f>
         <v/>
       </c>
@@ -70430,11 +70424,11 @@
           <t>Emory</t>
         </is>
       </c>
-      <c r="B19" s="18">
+      <c r="B19" s="19">
         <f>S3_FY25!M13</f>
         <v/>
       </c>
-      <c r="C19" s="18" t="n">
+      <c r="C19" s="19" t="n">
         <v>15046</v>
       </c>
       <c r="D19" s="11">
@@ -70453,7 +70447,7 @@
         <f>RANK(E19,E$12:E$24,1)</f>
         <v/>
       </c>
-      <c r="H19" s="24">
+      <c r="H19" s="25">
         <f>(C19/B19-1)*100</f>
         <v/>
       </c>
@@ -70464,11 +70458,11 @@
           <t>Penn</t>
         </is>
       </c>
-      <c r="B20" s="18">
+      <c r="B20" s="19">
         <f>S3_FY25!M14</f>
         <v/>
       </c>
-      <c r="C20" s="18" t="n">
+      <c r="C20" s="19" t="n">
         <v>28711</v>
       </c>
       <c r="D20" s="11">
@@ -70487,7 +70481,7 @@
         <f>RANK(E20,E$12:E$24,1)</f>
         <v/>
       </c>
-      <c r="H20" s="24">
+      <c r="H20" s="25">
         <f>(C20/B20-1)*100</f>
         <v/>
       </c>
@@ -70498,11 +70492,11 @@
           <t>Stanford</t>
         </is>
       </c>
-      <c r="B21" s="18">
+      <c r="B21" s="19">
         <f>S3_FY25!M15</f>
         <v/>
       </c>
-      <c r="C21" s="18" t="n">
+      <c r="C21" s="19" t="n">
         <v>18446</v>
       </c>
       <c r="D21" s="11">
@@ -70521,7 +70515,7 @@
         <f>RANK(E21,E$12:E$24,1)</f>
         <v/>
       </c>
-      <c r="H21" s="24">
+      <c r="H21" s="25">
         <f>(C21/B21-1)*100</f>
         <v/>
       </c>
@@ -70532,11 +70526,11 @@
           <t>Northeastern</t>
         </is>
       </c>
-      <c r="B22" s="18">
+      <c r="B22" s="19">
         <f>S3_FY25!M16</f>
         <v/>
       </c>
-      <c r="C22" s="18" t="n">
+      <c r="C22" s="19" t="n">
         <v>31159</v>
       </c>
       <c r="D22" s="11">
@@ -70555,7 +70549,7 @@
         <f>RANK(E22,E$12:E$24,1)</f>
         <v/>
       </c>
-      <c r="H22" s="24">
+      <c r="H22" s="25">
         <f>(C22/B22-1)*100</f>
         <v/>
       </c>
@@ -70566,11 +70560,11 @@
           <t>Boston University</t>
         </is>
       </c>
-      <c r="B23" s="18">
+      <c r="B23" s="19">
         <f>S3_FY25!M17</f>
         <v/>
       </c>
-      <c r="C23" s="18" t="n">
+      <c r="C23" s="19" t="n">
         <v>36624</v>
       </c>
       <c r="D23" s="11">
@@ -70589,7 +70583,7 @@
         <f>RANK(E23,E$12:E$24,1)</f>
         <v/>
       </c>
-      <c r="H23" s="24">
+      <c r="H23" s="25">
         <f>(C23/B23-1)*100</f>
         <v/>
       </c>
@@ -70600,11 +70594,11 @@
           <t>MIT</t>
         </is>
       </c>
-      <c r="B24" s="18">
+      <c r="B24" s="19">
         <f>S3_FY25!M18</f>
         <v/>
       </c>
-      <c r="C24" s="18" t="n">
+      <c r="C24" s="19" t="n">
         <v>11920</v>
       </c>
       <c r="D24" s="11">
@@ -70623,7 +70617,7 @@
         <f>RANK(E24,E$12:E$24,1)</f>
         <v/>
       </c>
-      <c r="H24" s="24">
+      <c r="H24" s="25">
         <f>(C24/B24-1)*100</f>
         <v/>
       </c>
@@ -70631,7 +70625,7 @@
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>C. Penn and Stanford estimated S&amp;W under alternative S&amp;W shares of salaries + benefits</t>
+          <t>C. Penn and Stanford estimated S&amp;W under alternative assumptions</t>
         </is>
       </c>
     </row>
@@ -70648,32 +70642,42 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>S&amp;W share used (Form 990)</t>
+          <t>Fringe rate used (input on S3_FY25)</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>S&amp;W per student, share used</t>
+          <t>S&amp;W per student, used</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t>Peer-median share (hospital schools)</t>
+          <t>Alt 1: own Form 990 S&amp;W share</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t>S&amp;W per student, peer share</t>
+          <t>S&amp;W per student, Alt 1</t>
         </is>
       </c>
       <c r="G28" s="5" t="inlineStr">
         <is>
-          <t>Original slide assumption (72.8%)</t>
+          <t>Alt 1 vs used (%)</t>
         </is>
       </c>
       <c r="H28" s="5" t="inlineStr">
         <is>
-          <t>S&amp;W per student, 72.8%</t>
+          <t>Alt 2: original slide 72.8%</t>
+        </is>
+      </c>
+      <c r="I28" s="5" t="inlineStr">
+        <is>
+          <t>S&amp;W per student, Alt 2</t>
+        </is>
+      </c>
+      <c r="J28" s="5" t="inlineStr">
+        <is>
+          <t>Alt 2 vs used (%)</t>
         </is>
       </c>
     </row>
@@ -70683,31 +70687,39 @@
           <t>Penn</t>
         </is>
       </c>
-      <c r="B29" s="18">
+      <c r="B29" s="19">
         <f>S3_FY25!E14</f>
         <v/>
       </c>
-      <c r="C29" s="19">
+      <c r="C29" s="15">
+        <f>S3_FY25!E3</f>
+        <v/>
+      </c>
+      <c r="D29" s="11">
+        <f>B29/(1+C29)/S3_FY25!M14</f>
+        <v/>
+      </c>
+      <c r="E29" s="20">
         <f>S3_FY25!F14/S3_FY25!G14</f>
-        <v/>
-      </c>
-      <c r="D29" s="11">
-        <f>B29*C29/S3_FY25!M14</f>
-        <v/>
-      </c>
-      <c r="E29" s="19">
-        <f>MEDIAN(S3_FY25!C11/S3_FY25!E11,S3_FY25!C12/S3_FY25!E12,S3_FY25!C13/S3_FY25!E13)</f>
         <v/>
       </c>
       <c r="F29" s="11">
         <f>B29*E29/S3_FY25!M14</f>
         <v/>
       </c>
-      <c r="G29" s="19" t="n">
+      <c r="G29" s="25">
+        <f>(F29/D29-1)*100</f>
+        <v/>
+      </c>
+      <c r="H29" s="20" t="n">
         <v>0.728</v>
       </c>
-      <c r="H29" s="11">
-        <f>B29*G29/S3_FY25!M14</f>
+      <c r="I29" s="11">
+        <f>B29*H29/S3_FY25!M14</f>
+        <v/>
+      </c>
+      <c r="J29" s="25">
+        <f>(I29/D29-1)*100</f>
         <v/>
       </c>
     </row>
@@ -70717,38 +70729,246 @@
           <t>Stanford</t>
         </is>
       </c>
-      <c r="B30" s="18">
+      <c r="B30" s="19">
         <f>S3_FY25!E15</f>
         <v/>
       </c>
-      <c r="C30" s="19">
+      <c r="C30" s="15">
+        <f>S3_FY25!E3</f>
+        <v/>
+      </c>
+      <c r="D30" s="11">
+        <f>B30/(1+C30)/S3_FY25!M15</f>
+        <v/>
+      </c>
+      <c r="E30" s="20">
         <f>S3_FY25!F15/S3_FY25!G15</f>
-        <v/>
-      </c>
-      <c r="D30" s="11">
-        <f>B30*C30/S3_FY25!M15</f>
-        <v/>
-      </c>
-      <c r="E30" s="19">
-        <f>MEDIAN(S3_FY25!C11/S3_FY25!E11,S3_FY25!C12/S3_FY25!E12,S3_FY25!C13/S3_FY25!E13)</f>
         <v/>
       </c>
       <c r="F30" s="11">
         <f>B30*E30/S3_FY25!M15</f>
         <v/>
       </c>
-      <c r="G30" s="19" t="n">
+      <c r="G30" s="25">
+        <f>(F30/D30-1)*100</f>
+        <v/>
+      </c>
+      <c r="H30" s="20" t="n">
         <v>0.728</v>
       </c>
-      <c r="H30" s="11">
-        <f>B30*G30/S3_FY25!M15</f>
+      <c r="I30" s="11">
+        <f>B30*H30/S3_FY25!M15</f>
+        <v/>
+      </c>
+      <c r="J30" s="25">
+        <f>(I30/D30-1)*100</f>
         <v/>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="17" t="inlineStr">
-        <is>
-          <t>Peer-median share = median of Chicago, Duke and Emory (the hospital-consolidated schools whose audited statements report S&amp;W and benefits separately).</t>
+      <c r="A32" s="3" t="inlineStr">
+        <is>
+          <t>D. Fringe benefit rates (benefits / S&amp;W) observed where audited statements report both lines</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="5" t="inlineStr">
+        <is>
+          <t>Institution</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>S&amp;W ($)</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Benefits ($)</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>Fringe rate</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="9" t="inlineStr">
+        <is>
+          <t>Rice</t>
+        </is>
+      </c>
+      <c r="B34" s="19">
+        <f>S3_FY25!C5</f>
+        <v/>
+      </c>
+      <c r="C34" s="19">
+        <f>S3_FY25!E5-S3_FY25!C5</f>
+        <v/>
+      </c>
+      <c r="D34" s="20">
+        <f>C34/B34</f>
+        <v/>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="9" t="inlineStr">
+        <is>
+          <t>Princeton</t>
+        </is>
+      </c>
+      <c r="B35" s="19">
+        <f>S3_FY25!C8</f>
+        <v/>
+      </c>
+      <c r="C35" s="19">
+        <f>S3_FY25!E8-S3_FY25!C8</f>
+        <v/>
+      </c>
+      <c r="D35" s="20">
+        <f>C35/B35</f>
+        <v/>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="9" t="inlineStr">
+        <is>
+          <t>Yale</t>
+        </is>
+      </c>
+      <c r="B36" s="19">
+        <f>S3_FY25!C10</f>
+        <v/>
+      </c>
+      <c r="C36" s="19">
+        <f>S3_FY25!E10-S3_FY25!C10</f>
+        <v/>
+      </c>
+      <c r="D36" s="20">
+        <f>C36/B36</f>
+        <v/>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="9" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="B37" s="19">
+        <f>S3_FY25!C11</f>
+        <v/>
+      </c>
+      <c r="C37" s="19">
+        <f>S3_FY25!E11-S3_FY25!C11</f>
+        <v/>
+      </c>
+      <c r="D37" s="20">
+        <f>C37/B37</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="9" t="inlineStr">
+        <is>
+          <t>Duke</t>
+        </is>
+      </c>
+      <c r="B38" s="19">
+        <f>S3_FY25!C12</f>
+        <v/>
+      </c>
+      <c r="C38" s="19">
+        <f>S3_FY25!E12-S3_FY25!C12</f>
+        <v/>
+      </c>
+      <c r="D38" s="20">
+        <f>C38/B38</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="9" t="inlineStr">
+        <is>
+          <t>Emory</t>
+        </is>
+      </c>
+      <c r="B39" s="19">
+        <f>S3_FY25!C13</f>
+        <v/>
+      </c>
+      <c r="C39" s="19">
+        <f>S3_FY25!E13-S3_FY25!C13</f>
+        <v/>
+      </c>
+      <c r="D39" s="20">
+        <f>C39/B39</f>
+        <v/>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="9" t="inlineStr">
+        <is>
+          <t>Boston University</t>
+        </is>
+      </c>
+      <c r="B40" s="19">
+        <f>S3_FY25!C17</f>
+        <v/>
+      </c>
+      <c r="C40" s="19">
+        <f>S3_FY25!E17-S3_FY25!C17</f>
+        <v/>
+      </c>
+      <c r="D40" s="20">
+        <f>C40/B40</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="9" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="B41" s="19">
+        <f>S3_FY25!C18</f>
+        <v/>
+      </c>
+      <c r="C41" s="19">
+        <f>S3_FY25!E18-S3_FY25!C18</f>
+        <v/>
+      </c>
+      <c r="D41" s="20">
+        <f>C41/B41</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="3" t="inlineStr">
+        <is>
+          <t>Minimum / median / maximum</t>
+        </is>
+      </c>
+      <c r="B42" s="23">
+        <f>MIN(D34:D41)</f>
+        <v/>
+      </c>
+      <c r="C42" s="23">
+        <f>MEDIAN(D34:D41)</f>
+        <v/>
+      </c>
+      <c r="D42" s="23">
+        <f>MAX(D34:D41)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="17" t="inlineStr">
+        <is>
+          <t>The 35% assumption sits above every observed rate, so the Penn and Stanford estimates lean low relative to peers (Alt 1 gives higher S&amp;W per student).</t>
         </is>
       </c>
     </row>
@@ -70874,41 +71094,41 @@
           <t>Rice</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n">
+      <c r="B5" s="19" t="n">
         <v>421781000</v>
       </c>
-      <c r="C5" s="18" t="n">
+      <c r="C5" s="19" t="n">
         <v>959377000</v>
       </c>
-      <c r="D5" s="18" t="n">
+      <c r="D5" s="19" t="n">
         <v>421781000</v>
       </c>
-      <c r="E5" s="18" t="n">
+      <c r="E5" s="19" t="n">
         <v>959377000</v>
       </c>
-      <c r="F5" s="18" t="n">
+      <c r="F5" s="19" t="n">
         <v>118187000</v>
       </c>
-      <c r="G5" s="18">
+      <c r="G5" s="19">
         <f>E5-F5</f>
         <v/>
       </c>
-      <c r="H5" s="24">
+      <c r="H5" s="25">
         <f>(C5/E5-1)*100</f>
         <v/>
       </c>
-      <c r="I5" s="24">
+      <c r="I5" s="25">
         <f>(C5/G5-1)*100</f>
         <v/>
       </c>
-      <c r="J5" s="24">
+      <c r="J5" s="25">
         <f>(B5/D5-1)*100</f>
         <v/>
       </c>
-      <c r="M5" s="18" t="n">
+      <c r="M5" s="19" t="n">
         <v>959377000</v>
       </c>
-      <c r="N5" s="18" t="n">
+      <c r="N5" s="19" t="n">
         <v>421781000</v>
       </c>
     </row>
@@ -70918,48 +71138,48 @@
           <t>Vanderbilt</t>
         </is>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="19" t="n">
         <v>699234000</v>
       </c>
-      <c r="C6" s="18" t="n">
+      <c r="C6" s="19" t="n">
         <v>1615854000</v>
       </c>
-      <c r="D6" s="18" t="n">
+      <c r="D6" s="19" t="n">
         <v>700000000</v>
       </c>
-      <c r="E6" s="18" t="n">
+      <c r="E6" s="19" t="n">
         <v>1615854000</v>
       </c>
-      <c r="F6" s="18" t="n">
+      <c r="F6" s="19" t="n">
         <v>122175000</v>
       </c>
-      <c r="G6" s="18">
+      <c r="G6" s="19">
         <f>E6-F6</f>
         <v/>
       </c>
-      <c r="H6" s="24">
+      <c r="H6" s="25">
         <f>(C6/E6-1)*100</f>
         <v/>
       </c>
-      <c r="I6" s="24">
+      <c r="I6" s="25">
         <f>(C6/G6-1)*100</f>
         <v/>
       </c>
-      <c r="J6" s="24">
+      <c r="J6" s="25">
         <f>(B6/D6-1)*100</f>
         <v/>
       </c>
-      <c r="K6" s="18" t="n">
+      <c r="K6" s="19" t="n">
         <v>832612000</v>
       </c>
-      <c r="L6" s="25">
+      <c r="L6" s="26">
         <f>B6/K6</f>
         <v/>
       </c>
-      <c r="M6" s="18" t="n">
+      <c r="M6" s="19" t="n">
         <v>1615854013</v>
       </c>
-      <c r="N6" s="18" t="n">
+      <c r="N6" s="19" t="n">
         <v>699234852</v>
       </c>
     </row>
@@ -70969,42 +71189,42 @@
           <t>Northwestern</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="19" t="n">
         <v>1219645336</v>
       </c>
-      <c r="C7" s="18" t="n">
+      <c r="C7" s="19" t="n">
         <v>3038060000</v>
       </c>
-      <c r="D7" s="18" t="n"/>
-      <c r="E7" s="18" t="n">
+      <c r="D7" s="19" t="n"/>
+      <c r="E7" s="19" t="n">
         <v>3038060000</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="19" t="n">
         <v>303553000</v>
       </c>
-      <c r="G7" s="18">
+      <c r="G7" s="19">
         <f>E7-F7</f>
         <v/>
       </c>
-      <c r="H7" s="24">
+      <c r="H7" s="25">
         <f>(C7/E7-1)*100</f>
         <v/>
       </c>
-      <c r="I7" s="24">
+      <c r="I7" s="25">
         <f>(C7/G7-1)*100</f>
         <v/>
       </c>
-      <c r="K7" s="18" t="n">
+      <c r="K7" s="19" t="n">
         <v>1675337000</v>
       </c>
-      <c r="L7" s="25">
+      <c r="L7" s="26">
         <f>B7/K7</f>
         <v/>
       </c>
-      <c r="M7" s="18" t="n">
+      <c r="M7" s="19" t="n">
         <v>3038060000</v>
       </c>
-      <c r="N7" s="18" t="n">
+      <c r="N7" s="19" t="n">
         <v>1334540000</v>
       </c>
     </row>
@@ -71014,41 +71234,41 @@
           <t>Princeton</t>
         </is>
       </c>
-      <c r="B8" s="18" t="n">
+      <c r="B8" s="19" t="n">
         <v>969089000</v>
       </c>
-      <c r="C8" s="18" t="n">
+      <c r="C8" s="19" t="n">
         <v>2263259000</v>
       </c>
-      <c r="D8" s="18" t="n">
+      <c r="D8" s="19" t="n">
         <v>969089000</v>
       </c>
-      <c r="E8" s="18" t="n">
+      <c r="E8" s="19" t="n">
         <v>2263259000</v>
       </c>
-      <c r="F8" s="18" t="n">
+      <c r="F8" s="19" t="n">
         <v>349162000</v>
       </c>
-      <c r="G8" s="18">
+      <c r="G8" s="19">
         <f>E8-F8</f>
         <v/>
       </c>
-      <c r="H8" s="24">
+      <c r="H8" s="25">
         <f>(C8/E8-1)*100</f>
         <v/>
       </c>
-      <c r="I8" s="24">
+      <c r="I8" s="25">
         <f>(C8/G8-1)*100</f>
         <v/>
       </c>
-      <c r="J8" s="24">
+      <c r="J8" s="25">
         <f>(B8/D8-1)*100</f>
         <v/>
       </c>
-      <c r="M8" s="18" t="n">
+      <c r="M8" s="19" t="n">
         <v>2263259000</v>
       </c>
-      <c r="N8" s="18" t="n">
+      <c r="N8" s="19" t="n">
         <v>886833000</v>
       </c>
     </row>
@@ -71058,21 +71278,21 @@
           <t>Harvard</t>
         </is>
       </c>
-      <c r="B9" s="18" t="n">
+      <c r="B9" s="19" t="n">
         <v>2421076000</v>
       </c>
-      <c r="C9" s="18" t="n">
+      <c r="C9" s="19" t="n">
         <v>5911797000</v>
       </c>
-      <c r="D9" s="21" t="inlineStr">
+      <c r="D9" s="22" t="inlineStr">
         <is>
           <t>Harvard FY23 report not reached</t>
         </is>
       </c>
-      <c r="M9" s="18" t="n">
+      <c r="M9" s="19" t="n">
         <v>5911797000</v>
       </c>
-      <c r="N9" s="18" t="n">
+      <c r="N9" s="19" t="n">
         <v>2421074000</v>
       </c>
     </row>
@@ -71082,41 +71302,41 @@
           <t>Yale</t>
         </is>
       </c>
-      <c r="B10" s="18" t="n">
+      <c r="B10" s="19" t="n">
         <v>2328136000</v>
       </c>
-      <c r="C10" s="18" t="n">
+      <c r="C10" s="19" t="n">
         <v>4936268000</v>
       </c>
-      <c r="D10" s="18" t="n">
+      <c r="D10" s="19" t="n">
         <v>2328136000</v>
       </c>
-      <c r="E10" s="18" t="n">
+      <c r="E10" s="19" t="n">
         <v>4936268000</v>
       </c>
-      <c r="F10" s="18" t="n">
+      <c r="F10" s="19" t="n">
         <v>441202000</v>
       </c>
-      <c r="G10" s="18">
+      <c r="G10" s="19">
         <f>E10-F10</f>
         <v/>
       </c>
-      <c r="H10" s="24">
+      <c r="H10" s="25">
         <f>(C10/E10-1)*100</f>
         <v/>
       </c>
-      <c r="I10" s="24">
+      <c r="I10" s="25">
         <f>(C10/G10-1)*100</f>
         <v/>
       </c>
-      <c r="J10" s="24">
+      <c r="J10" s="25">
         <f>(B10/D10-1)*100</f>
         <v/>
       </c>
-      <c r="M10" s="18" t="n">
+      <c r="M10" s="19" t="n">
         <v>4873675887</v>
       </c>
-      <c r="N10" s="18" t="n">
+      <c r="N10" s="19" t="n">
         <v>2202260626</v>
       </c>
     </row>
@@ -71126,48 +71346,48 @@
           <t>Chicago</t>
         </is>
       </c>
-      <c r="B11" s="18" t="n">
+      <c r="B11" s="19" t="n">
         <v>3033100000</v>
       </c>
-      <c r="C11" s="18" t="n">
+      <c r="C11" s="19" t="n">
         <v>6779655000</v>
       </c>
-      <c r="D11" s="18" t="n">
+      <c r="D11" s="19" t="n">
         <v>3033100000</v>
       </c>
-      <c r="E11" s="18" t="n">
+      <c r="E11" s="19" t="n">
         <v>6779655000</v>
       </c>
-      <c r="F11" s="18" t="n">
+      <c r="F11" s="19" t="n">
         <v>563830000</v>
       </c>
-      <c r="G11" s="18">
+      <c r="G11" s="19">
         <f>E11-F11</f>
         <v/>
       </c>
-      <c r="H11" s="24">
+      <c r="H11" s="25">
         <f>(C11/E11-1)*100</f>
         <v/>
       </c>
-      <c r="I11" s="24">
+      <c r="I11" s="25">
         <f>(C11/G11-1)*100</f>
         <v/>
       </c>
-      <c r="J11" s="24">
+      <c r="J11" s="25">
         <f>(B11/D11-1)*100</f>
         <v/>
       </c>
-      <c r="K11" s="18" t="n">
+      <c r="K11" s="19" t="n">
         <v>3662513000</v>
       </c>
-      <c r="L11" s="25">
+      <c r="L11" s="26">
         <f>B11/K11</f>
         <v/>
       </c>
-      <c r="M11" s="18" t="n">
+      <c r="M11" s="19" t="n">
         <v>5084463771</v>
       </c>
-      <c r="N11" s="18" t="n">
+      <c r="N11" s="19" t="n">
         <v>1604106945</v>
       </c>
     </row>
@@ -71177,48 +71397,48 @@
           <t>Duke</t>
         </is>
       </c>
-      <c r="B12" s="18" t="n">
+      <c r="B12" s="19" t="n">
         <v>3676675000</v>
       </c>
-      <c r="C12" s="18" t="n">
+      <c r="C12" s="19" t="n">
         <v>8431382000</v>
       </c>
-      <c r="D12" s="18" t="n">
+      <c r="D12" s="19" t="n">
         <v>3676675000</v>
       </c>
-      <c r="E12" s="18" t="n">
+      <c r="E12" s="19" t="n">
         <v>8431382000</v>
       </c>
-      <c r="F12" s="18" t="n">
+      <c r="F12" s="19" t="n">
         <v>635501000</v>
       </c>
-      <c r="G12" s="18">
+      <c r="G12" s="19">
         <f>E12-F12</f>
         <v/>
       </c>
-      <c r="H12" s="24">
+      <c r="H12" s="25">
         <f>(C12/E12-1)*100</f>
         <v/>
       </c>
-      <c r="I12" s="24">
+      <c r="I12" s="25">
         <f>(C12/G12-1)*100</f>
         <v/>
       </c>
-      <c r="J12" s="24">
+      <c r="J12" s="25">
         <f>(B12/D12-1)*100</f>
         <v/>
       </c>
-      <c r="K12" s="18" t="n">
+      <c r="K12" s="19" t="n">
         <v>4568399000</v>
       </c>
-      <c r="L12" s="25">
+      <c r="L12" s="26">
         <f>B12/K12</f>
         <v/>
       </c>
-      <c r="M12" s="18" t="n">
+      <c r="M12" s="19" t="n">
         <v>8431382000</v>
       </c>
-      <c r="N12" s="18" t="n">
+      <c r="N12" s="19" t="n">
         <v>3609077000</v>
       </c>
     </row>
@@ -71228,41 +71448,41 @@
           <t>Emory</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
         <v>4313737000</v>
       </c>
-      <c r="C13" s="18" t="n">
+      <c r="C13" s="19" t="n">
         <v>8570621000</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="D13" s="19" t="n">
         <v>4313737000</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="E13" s="19" t="n">
         <v>8570621000</v>
       </c>
-      <c r="F13" s="18" t="n">
+      <c r="F13" s="19" t="n">
         <v>452316000</v>
       </c>
-      <c r="G13" s="18">
+      <c r="G13" s="19">
         <f>E13-F13</f>
         <v/>
       </c>
-      <c r="H13" s="24">
+      <c r="H13" s="25">
         <f>(C13/E13-1)*100</f>
         <v/>
       </c>
-      <c r="I13" s="24">
+      <c r="I13" s="25">
         <f>(C13/G13-1)*100</f>
         <v/>
       </c>
-      <c r="J13" s="24">
+      <c r="J13" s="25">
         <f>(B13/D13-1)*100</f>
         <v/>
       </c>
-      <c r="M13" s="18" t="n">
+      <c r="M13" s="19" t="n">
         <v>8514754000</v>
       </c>
-      <c r="N13" s="18" t="n">
+      <c r="N13" s="19" t="n">
         <v>4252849000</v>
       </c>
     </row>
@@ -71272,42 +71492,42 @@
           <t>Penn</t>
         </is>
       </c>
-      <c r="B14" s="18" t="n">
+      <c r="B14" s="19" t="n">
         <v>5636695792</v>
       </c>
-      <c r="C14" s="18" t="n">
+      <c r="C14" s="19" t="n">
         <v>13857148000</v>
       </c>
-      <c r="D14" s="18" t="n"/>
-      <c r="E14" s="18" t="n">
+      <c r="D14" s="19" t="n"/>
+      <c r="E14" s="19" t="n">
         <v>13857148000</v>
       </c>
-      <c r="F14" s="18" t="n">
+      <c r="F14" s="19" t="n">
         <v>789992000</v>
       </c>
-      <c r="G14" s="18">
+      <c r="G14" s="19">
         <f>E14-F14</f>
         <v/>
       </c>
-      <c r="H14" s="24">
+      <c r="H14" s="25">
         <f>(C14/E14-1)*100</f>
         <v/>
       </c>
-      <c r="I14" s="24">
+      <c r="I14" s="25">
         <f>(C14/G14-1)*100</f>
         <v/>
       </c>
-      <c r="K14" s="18" t="n">
+      <c r="K14" s="19" t="n">
         <v>7742714000</v>
       </c>
-      <c r="L14" s="25">
+      <c r="L14" s="26">
         <f>B14/K14</f>
         <v/>
       </c>
-      <c r="M14" s="18" t="n">
+      <c r="M14" s="19" t="n">
         <v>13857148000</v>
       </c>
-      <c r="N14" s="18" t="n">
+      <c r="N14" s="19" t="n">
         <v>6045218000</v>
       </c>
     </row>
@@ -71317,42 +71537,42 @@
           <t>Stanford</t>
         </is>
       </c>
-      <c r="B15" s="18" t="n">
+      <c r="B15" s="19" t="n">
         <v>7106067696</v>
       </c>
-      <c r="C15" s="18" t="n">
+      <c r="C15" s="19" t="n">
         <v>16053362000</v>
       </c>
-      <c r="D15" s="18" t="n"/>
-      <c r="E15" s="18" t="n">
+      <c r="D15" s="19" t="n"/>
+      <c r="E15" s="19" t="n">
         <v>16053362000</v>
       </c>
-      <c r="F15" s="18" t="n">
+      <c r="F15" s="19" t="n">
         <v>1116974000</v>
       </c>
-      <c r="G15" s="18">
+      <c r="G15" s="19">
         <f>E15-F15</f>
         <v/>
       </c>
-      <c r="H15" s="24">
+      <c r="H15" s="25">
         <f>(C15/E15-1)*100</f>
         <v/>
       </c>
-      <c r="I15" s="24">
+      <c r="I15" s="25">
         <f>(C15/G15-1)*100</f>
         <v/>
       </c>
-      <c r="K15" s="18" t="n">
+      <c r="K15" s="19" t="n">
         <v>9761082000</v>
       </c>
-      <c r="L15" s="25">
+      <c r="L15" s="26">
         <f>B15/K15</f>
         <v/>
       </c>
-      <c r="M15" s="18" t="n">
+      <c r="M15" s="19" t="n">
         <v>7659884000</v>
       </c>
-      <c r="N15" s="18" t="n">
+      <c r="N15" s="19" t="n">
         <v>3467999000</v>
       </c>
     </row>
@@ -71461,29 +71681,29 @@
           <t>Rice</t>
         </is>
       </c>
-      <c r="B5" s="18" t="n">
+      <c r="B5" s="19" t="n">
         <v>8961</v>
       </c>
-      <c r="C5" s="18" t="n">
+      <c r="C5" s="19" t="n">
         <v>8556</v>
       </c>
-      <c r="D5" s="18" t="n">
+      <c r="D5" s="19" t="n">
         <v>8672</v>
       </c>
-      <c r="E5" s="18" t="n">
+      <c r="E5" s="19" t="n">
         <v>8556</v>
       </c>
-      <c r="F5" s="18" t="n">
+      <c r="F5" s="19" t="n">
         <v>8672</v>
       </c>
-      <c r="G5" s="18" t="n">
+      <c r="G5" s="19" t="n">
         <v>8285</v>
       </c>
-      <c r="H5" s="24">
+      <c r="H5" s="25">
         <f>(E5/C5-1)*100</f>
         <v/>
       </c>
-      <c r="I5" s="24">
+      <c r="I5" s="25">
         <f>(G5/F5-1)*100</f>
         <v/>
       </c>
@@ -71499,29 +71719,29 @@
           <t>Vanderbilt</t>
         </is>
       </c>
-      <c r="B6" s="18" t="n">
+      <c r="B6" s="19" t="n">
         <v>13575</v>
       </c>
-      <c r="C6" s="18" t="n">
+      <c r="C6" s="19" t="n">
         <v>13456</v>
       </c>
-      <c r="D6" s="18" t="n">
+      <c r="D6" s="19" t="n">
         <v>13710</v>
       </c>
-      <c r="E6" s="18" t="n">
+      <c r="E6" s="19" t="n">
         <v>13456</v>
       </c>
-      <c r="F6" s="18" t="n">
+      <c r="F6" s="19" t="n">
         <v>13710</v>
       </c>
-      <c r="G6" s="18" t="n">
+      <c r="G6" s="19" t="n">
         <v>13710</v>
       </c>
-      <c r="H6" s="24">
+      <c r="H6" s="25">
         <f>(E6/C6-1)*100</f>
         <v/>
       </c>
-      <c r="I6" s="24">
+      <c r="I6" s="25">
         <f>(G6/F6-1)*100</f>
         <v/>
       </c>
@@ -71537,29 +71757,29 @@
           <t>Northwestern</t>
         </is>
       </c>
-      <c r="B7" s="18" t="n">
+      <c r="B7" s="19" t="n">
         <v>23431</v>
       </c>
-      <c r="C7" s="18" t="n">
+      <c r="C7" s="19" t="n">
         <v>22801</v>
       </c>
-      <c r="D7" s="18" t="n">
+      <c r="D7" s="19" t="n">
         <v>22732</v>
       </c>
-      <c r="E7" s="18" t="n">
+      <c r="E7" s="19" t="n">
         <v>23203</v>
       </c>
-      <c r="F7" s="18" t="n">
+      <c r="F7" s="19" t="n">
         <v>23161</v>
       </c>
-      <c r="G7" s="18" t="n">
+      <c r="G7" s="19" t="n">
         <v>23000</v>
       </c>
-      <c r="H7" s="24">
+      <c r="H7" s="25">
         <f>(E7/C7-1)*100</f>
         <v/>
       </c>
-      <c r="I7" s="24">
+      <c r="I7" s="25">
         <f>(G7/F7-1)*100</f>
         <v/>
       </c>
@@ -71575,21 +71795,21 @@
           <t>Princeton</t>
         </is>
       </c>
-      <c r="B8" s="18" t="n">
+      <c r="B8" s="19" t="n">
         <v>9050</v>
       </c>
-      <c r="C8" s="18" t="n"/>
-      <c r="D8" s="18" t="n"/>
-      <c r="E8" s="18" t="n">
+      <c r="C8" s="19" t="n"/>
+      <c r="D8" s="19" t="n"/>
+      <c r="E8" s="19" t="n">
         <v>8922</v>
       </c>
-      <c r="F8" s="18" t="n">
+      <c r="F8" s="19" t="n">
         <v>8842</v>
       </c>
-      <c r="G8" s="18" t="n">
+      <c r="G8" s="19" t="n">
         <v>8778</v>
       </c>
-      <c r="I8" s="24">
+      <c r="I8" s="25">
         <f>(G8/F8-1)*100</f>
         <v/>
       </c>
@@ -71605,29 +71825,29 @@
           <t>Harvard</t>
         </is>
       </c>
-      <c r="B9" s="18" t="n">
+      <c r="B9" s="19" t="n">
         <v>21189</v>
       </c>
-      <c r="C9" s="18" t="n">
+      <c r="C9" s="19" t="n">
         <v>21278</v>
       </c>
-      <c r="D9" s="18" t="n">
+      <c r="D9" s="19" t="n">
         <v>21613</v>
       </c>
-      <c r="E9" s="18" t="n">
+      <c r="E9" s="19" t="n">
         <v>30386</v>
       </c>
-      <c r="F9" s="18" t="n">
+      <c r="F9" s="19" t="n">
         <v>30631</v>
       </c>
-      <c r="G9" s="18" t="n">
+      <c r="G9" s="19" t="n">
         <v>21400</v>
       </c>
-      <c r="H9" s="24">
+      <c r="H9" s="25">
         <f>(E9/C9-1)*100</f>
         <v/>
       </c>
-      <c r="I9" s="24">
+      <c r="I9" s="25">
         <f>(G9/F9-1)*100</f>
         <v/>
       </c>
@@ -71643,29 +71863,29 @@
           <t>Yale</t>
         </is>
       </c>
-      <c r="B10" s="18" t="n">
+      <c r="B10" s="19" t="n">
         <v>15564</v>
       </c>
-      <c r="C10" s="18" t="n">
+      <c r="C10" s="19" t="n">
         <v>15081</v>
       </c>
-      <c r="D10" s="18" t="n">
+      <c r="D10" s="19" t="n">
         <v>14806</v>
       </c>
-      <c r="E10" s="18" t="n">
+      <c r="E10" s="19" t="n">
         <v>15081</v>
       </c>
-      <c r="F10" s="18" t="n">
+      <c r="F10" s="19" t="n">
         <v>14776</v>
       </c>
-      <c r="G10" s="18" t="n">
+      <c r="G10" s="19" t="n">
         <v>14751</v>
       </c>
-      <c r="H10" s="24">
+      <c r="H10" s="25">
         <f>(E10/C10-1)*100</f>
         <v/>
       </c>
-      <c r="I10" s="24">
+      <c r="I10" s="25">
         <f>(G10/F10-1)*100</f>
         <v/>
       </c>
@@ -71681,29 +71901,29 @@
           <t>Chicago</t>
         </is>
       </c>
-      <c r="B11" s="18" t="n">
+      <c r="B11" s="19" t="n">
         <v>16221</v>
       </c>
-      <c r="C11" s="18" t="n">
+      <c r="C11" s="19" t="n">
         <v>15763</v>
       </c>
-      <c r="D11" s="18" t="n">
+      <c r="D11" s="19" t="n">
         <v>15946</v>
       </c>
-      <c r="E11" s="18" t="n">
+      <c r="E11" s="19" t="n">
         <v>18339</v>
       </c>
-      <c r="F11" s="18" t="n">
+      <c r="F11" s="19" t="n">
         <v>18339</v>
       </c>
-      <c r="G11" s="18" t="n">
+      <c r="G11" s="19" t="n">
         <v>18058</v>
       </c>
-      <c r="H11" s="24">
+      <c r="H11" s="25">
         <f>(E11/C11-1)*100</f>
         <v/>
       </c>
-      <c r="I11" s="24">
+      <c r="I11" s="25">
         <f>(G11/F11-1)*100</f>
         <v/>
       </c>
@@ -71719,29 +71939,29 @@
           <t>Duke</t>
         </is>
       </c>
-      <c r="B12" s="18" t="n">
+      <c r="B12" s="19" t="n">
         <v>17499</v>
       </c>
-      <c r="C12" s="18" t="n">
+      <c r="C12" s="19" t="n">
         <v>17112</v>
       </c>
-      <c r="D12" s="18" t="n">
+      <c r="D12" s="19" t="n">
         <v>18024</v>
       </c>
-      <c r="E12" s="18" t="n">
+      <c r="E12" s="19" t="n">
         <v>17112</v>
       </c>
-      <c r="F12" s="18" t="n">
+      <c r="F12" s="19" t="n">
         <v>18023</v>
       </c>
-      <c r="G12" s="18" t="n">
+      <c r="G12" s="19" t="n">
         <v>18009</v>
       </c>
-      <c r="H12" s="24">
+      <c r="H12" s="25">
         <f>(E12/C12-1)*100</f>
         <v/>
       </c>
-      <c r="I12" s="24">
+      <c r="I12" s="25">
         <f>(G12/F12-1)*100</f>
         <v/>
       </c>
@@ -71757,29 +71977,29 @@
           <t>Emory</t>
         </is>
       </c>
-      <c r="B13" s="18" t="n">
+      <c r="B13" s="19" t="n">
         <v>15179</v>
       </c>
-      <c r="C13" s="18" t="n">
+      <c r="C13" s="19" t="n">
         <v>15046</v>
       </c>
-      <c r="D13" s="18" t="n">
+      <c r="D13" s="19" t="n">
         <v>14852</v>
       </c>
-      <c r="E13" s="18" t="n">
+      <c r="E13" s="19" t="n">
         <v>15046</v>
       </c>
-      <c r="F13" s="18" t="n">
+      <c r="F13" s="19" t="n">
         <v>14841</v>
       </c>
-      <c r="G13" s="18" t="n">
+      <c r="G13" s="19" t="n">
         <v>16000</v>
       </c>
-      <c r="H13" s="24">
+      <c r="H13" s="25">
         <f>(E13/C13-1)*100</f>
         <v/>
       </c>
-      <c r="I13" s="24">
+      <c r="I13" s="25">
         <f>(G13/F13-1)*100</f>
         <v/>
       </c>
@@ -71795,29 +72015,29 @@
           <t>Penn</t>
         </is>
       </c>
-      <c r="B14" s="18" t="n">
+      <c r="B14" s="19" t="n">
         <v>24023</v>
       </c>
-      <c r="C14" s="18" t="n">
+      <c r="C14" s="19" t="n">
         <v>23790</v>
       </c>
-      <c r="D14" s="18" t="n">
+      <c r="D14" s="19" t="n">
         <v>23374</v>
       </c>
-      <c r="E14" s="18" t="n">
+      <c r="E14" s="19" t="n">
         <v>28711</v>
       </c>
-      <c r="F14" s="18" t="n">
+      <c r="F14" s="19" t="n">
         <v>28201</v>
       </c>
-      <c r="G14" s="18" t="n">
+      <c r="G14" s="19" t="n">
         <v>23374</v>
       </c>
-      <c r="H14" s="24">
+      <c r="H14" s="25">
         <f>(E14/C14-1)*100</f>
         <v/>
       </c>
-      <c r="I14" s="24">
+      <c r="I14" s="25">
         <f>(G14/F14-1)*100</f>
         <v/>
       </c>
@@ -71833,29 +72053,29 @@
           <t>Stanford</t>
         </is>
       </c>
-      <c r="B15" s="18" t="n">
+      <c r="B15" s="19" t="n">
         <v>18625</v>
       </c>
-      <c r="C15" s="18" t="n">
+      <c r="C15" s="19" t="n">
         <v>18446</v>
       </c>
-      <c r="D15" s="18" t="n">
+      <c r="D15" s="19" t="n">
         <v>18283</v>
       </c>
-      <c r="E15" s="18" t="n">
+      <c r="E15" s="19" t="n">
         <v>18446</v>
       </c>
-      <c r="F15" s="18" t="n">
+      <c r="F15" s="19" t="n">
         <v>18283</v>
       </c>
-      <c r="G15" s="18" t="n">
+      <c r="G15" s="19" t="n">
         <v>17529</v>
       </c>
-      <c r="H15" s="24">
+      <c r="H15" s="25">
         <f>(E15/C15-1)*100</f>
         <v/>
       </c>
-      <c r="I15" s="24">
+      <c r="I15" s="25">
         <f>(G15/F15-1)*100</f>
         <v/>
       </c>
@@ -71871,22 +72091,22 @@
           <t>Northeastern</t>
         </is>
       </c>
-      <c r="B16" s="18" t="n">
+      <c r="B16" s="19" t="n">
         <v>39774</v>
       </c>
-      <c r="C16" s="18" t="n">
+      <c r="C16" s="19" t="n">
         <v>38760</v>
       </c>
-      <c r="D16" s="18" t="n">
+      <c r="D16" s="19" t="n">
         <v>36806</v>
       </c>
-      <c r="E16" s="18" t="n">
+      <c r="E16" s="19" t="n">
         <v>31159</v>
       </c>
-      <c r="F16" s="18" t="n">
+      <c r="F16" s="19" t="n">
         <v>30013</v>
       </c>
-      <c r="H16" s="24">
+      <c r="H16" s="25">
         <f>(E16/C16-1)*100</f>
         <v/>
       </c>
@@ -71902,22 +72122,22 @@
           <t>Boston University</t>
         </is>
       </c>
-      <c r="B17" s="18" t="n">
+      <c r="B17" s="19" t="n">
         <v>37737</v>
       </c>
-      <c r="C17" s="18" t="n">
+      <c r="C17" s="19" t="n">
         <v>36624</v>
       </c>
-      <c r="D17" s="18" t="n">
+      <c r="D17" s="19" t="n">
         <v>36714</v>
       </c>
-      <c r="E17" s="18" t="n">
+      <c r="E17" s="19" t="n">
         <v>36624</v>
       </c>
-      <c r="F17" s="18" t="n">
+      <c r="F17" s="19" t="n">
         <v>36714</v>
       </c>
-      <c r="H17" s="24">
+      <c r="H17" s="25">
         <f>(E17/C17-1)*100</f>
         <v/>
       </c>
@@ -71933,22 +72153,22 @@
           <t>MIT</t>
         </is>
       </c>
-      <c r="B18" s="18" t="n">
+      <c r="B18" s="19" t="n">
         <v>11886</v>
       </c>
-      <c r="C18" s="18" t="n">
+      <c r="C18" s="19" t="n">
         <v>11920</v>
       </c>
-      <c r="D18" s="18" t="n">
+      <c r="D18" s="19" t="n">
         <v>11858</v>
       </c>
-      <c r="E18" s="18" t="n">
+      <c r="E18" s="19" t="n">
         <v>11920</v>
       </c>
-      <c r="F18" s="18" t="n">
+      <c r="F18" s="19" t="n">
         <v>11858</v>
       </c>
-      <c r="H18" s="24">
+      <c r="H18" s="25">
         <f>(E18/C18-1)*100</f>
         <v/>
       </c>
@@ -72038,7 +72258,7 @@
           <t>Salaries and wages</t>
         </is>
       </c>
-      <c r="C5" s="18" t="n">
+      <c r="C5" s="19" t="n">
         <v>515800000</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
@@ -72063,7 +72283,7 @@
           <t>Total operating expenses</t>
         </is>
       </c>
-      <c r="C6" s="18" t="n">
+      <c r="C6" s="19" t="n">
         <v>1087937000</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
@@ -72088,7 +72308,7 @@
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="C7" s="18" t="n">
+      <c r="C7" s="19" t="n">
         <v>82255000</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
@@ -72113,7 +72333,7 @@
           <t>Interest</t>
         </is>
       </c>
-      <c r="C8" s="18" t="n">
+      <c r="C8" s="19" t="n">
         <v>45396000</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
@@ -72138,7 +72358,7 @@
           <t>Salaries and wages</t>
         </is>
       </c>
-      <c r="C9" s="18" t="n">
+      <c r="C9" s="19" t="n">
         <v>804000000</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
@@ -72163,7 +72383,7 @@
           <t>Total operating expenses</t>
         </is>
       </c>
-      <c r="C10" s="18" t="n">
+      <c r="C10" s="19" t="n">
         <v>1799663000</v>
       </c>
       <c r="D10" s="4" t="inlineStr">
@@ -72188,7 +72408,7 @@
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="C11" s="18" t="n">
+      <c r="C11" s="19" t="n">
         <v>116913000</v>
       </c>
       <c r="D11" s="4" t="inlineStr">
@@ -72213,7 +72433,7 @@
           <t>Interest</t>
         </is>
       </c>
-      <c r="C12" s="18" t="n">
+      <c r="C12" s="19" t="n">
         <v>30063000</v>
       </c>
       <c r="D12" s="4" t="inlineStr">
@@ -72238,7 +72458,7 @@
           <t>Salaries and wages</t>
         </is>
       </c>
-      <c r="C13" s="18" t="n"/>
+      <c r="C13" s="19" t="n"/>
       <c r="D13" s="4" t="inlineStr">
         <is>
           <t>Not separately reported. 'Salaries, wages, and benefits  1,997,951  1,832,098' (thousands), FY25 report PDF p.11 (printed p.9); note 16 (PDF p.34) also combined.</t>
@@ -72261,7 +72481,7 @@
           <t>Total operating expenses</t>
         </is>
       </c>
-      <c r="C14" s="18" t="n">
+      <c r="C14" s="19" t="n">
         <v>3607255000</v>
       </c>
       <c r="D14" s="4" t="inlineStr">
@@ -72286,7 +72506,7 @@
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="C15" s="18" t="n">
+      <c r="C15" s="19" t="n">
         <v>216713000</v>
       </c>
       <c r="D15" s="4" t="inlineStr">
@@ -72311,7 +72531,7 @@
           <t>Interest</t>
         </is>
       </c>
-      <c r="C16" s="18" t="n">
+      <c r="C16" s="19" t="n">
         <v>99478000</v>
       </c>
       <c r="D16" s="4" t="inlineStr">
@@ -72336,7 +72556,7 @@
           <t>Salaries and wages</t>
         </is>
       </c>
-      <c r="C17" s="18" t="n">
+      <c r="C17" s="19" t="n">
         <v>1162823000</v>
       </c>
       <c r="D17" s="4" t="inlineStr">
@@ -72361,7 +72581,7 @@
           <t>Total operating expenses</t>
         </is>
       </c>
-      <c r="C18" s="18" t="n">
+      <c r="C18" s="19" t="n">
         <v>2744548000</v>
       </c>
       <c r="D18" s="4" t="inlineStr">
@@ -72386,7 +72606,7 @@
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="C19" s="18" t="n">
+      <c r="C19" s="19" t="n">
         <v>231467000</v>
       </c>
       <c r="D19" s="4" t="inlineStr">
@@ -72411,7 +72631,7 @@
           <t>Interest</t>
         </is>
       </c>
-      <c r="C20" s="18" t="n">
+      <c r="C20" s="19" t="n">
         <v>221826000</v>
       </c>
       <c r="D20" s="4" t="inlineStr">
@@ -72436,7 +72656,7 @@
           <t>Salaries and wages</t>
         </is>
       </c>
-      <c r="C21" s="18" t="n"/>
+      <c r="C21" s="19" t="n"/>
       <c r="D21" s="4" t="inlineStr">
         <is>
           <t>NOT EXTRACTED: the Harvard Financial Report PDFs could not be retrieved (finance.harvard.edu returns Akamai 'Access Denied' 403 to curl with a browser User-Agent, and WebFetch reports the host blocked by the network egress proxy). No number was taken from a search snippet or memory.</t>
@@ -72459,7 +72679,7 @@
           <t>Total operating expenses</t>
         </is>
       </c>
-      <c r="C22" s="18" t="n"/>
+      <c r="C22" s="19" t="n"/>
       <c r="D22" s="4" t="inlineStr">
         <is>
           <t>NOT EXTRACTED: the Harvard Financial Report PDFs could not be retrieved (finance.harvard.edu returns Akamai 'Access Denied' 403 to curl with a browser User-Agent, and WebFetch reports the host blocked by the network egress proxy). No number was taken from a search snippet or memory.</t>
@@ -72482,7 +72702,7 @@
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="C23" s="18" t="n"/>
+      <c r="C23" s="19" t="n"/>
       <c r="D23" s="4" t="inlineStr">
         <is>
           <t>NOT EXTRACTED: the Harvard Financial Report PDFs could not be retrieved (finance.harvard.edu returns Akamai 'Access Denied' 403 to curl with a browser User-Agent, and WebFetch reports the host blocked by the network egress proxy). No number was taken from a search snippet or memory.</t>
@@ -72505,7 +72725,7 @@
           <t>Interest</t>
         </is>
       </c>
-      <c r="C24" s="18" t="n"/>
+      <c r="C24" s="19" t="n"/>
       <c r="D24" s="4" t="inlineStr">
         <is>
           <t>NOT EXTRACTED: the Harvard Financial Report PDFs could not be retrieved (finance.harvard.edu returns Akamai 'Access Denied' 403 to curl with a browser User-Agent, and WebFetch reports the host blocked by the network egress proxy). No number was taken from a search snippet or memory.</t>
@@ -72528,7 +72748,7 @@
           <t>Salaries and wages</t>
         </is>
       </c>
-      <c r="C25" s="18" t="n">
+      <c r="C25" s="19" t="n">
         <v>2737371000</v>
       </c>
       <c r="D25" s="4" t="inlineStr">
@@ -72553,7 +72773,7 @@
           <t>Total operating expenses</t>
         </is>
       </c>
-      <c r="C26" s="18" t="n">
+      <c r="C26" s="19" t="n">
         <v>5807911000</v>
       </c>
       <c r="D26" s="4" t="inlineStr">
@@ -72578,7 +72798,7 @@
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="C27" s="18" t="n"/>
+      <c r="C27" s="19" t="n"/>
       <c r="D27" s="4" t="inlineStr">
         <is>
           <t>Not separate on the face. Combined row: 'Depreciation, amortization and interest 504,923 - 504,923 470,601' (PDF p24). Note 8: 'Depreciation expense included in operating expenses amounted to $344.8 million and $328.9 million in 2025 and 2024' (PDF p48, printed p.46).</t>
@@ -72601,7 +72821,7 @@
           <t>Interest</t>
         </is>
       </c>
-      <c r="C28" s="18" t="n"/>
+      <c r="C28" s="19" t="n"/>
       <c r="D28" s="4" t="inlineStr">
         <is>
           <t>Not separate on the face (combined row above). Note 10: 'Total interest expense incurred on indebtedness was $108.3 million and $111.3 million in 2025 and 2024, respectively. Interest capitalized to land, buildings and equipment totaled $14.4 million and $9.9 million ... Amortization expense related to bond issue costs included in operating expenses amounted to $3.0 million and $3.7 million' (PDF p52). Note 6: financing lease 'Interest on lease liabilities Depreciation, amortization and interest 12,877 6,213' (PDF p46).</t>
@@ -72624,7 +72844,7 @@
           <t>Salaries and wages</t>
         </is>
       </c>
-      <c r="C29" s="18" t="n">
+      <c r="C29" s="19" t="n">
         <v>3678678000</v>
       </c>
       <c r="D29" s="4" t="inlineStr">
@@ -72649,7 +72869,7 @@
           <t>Total operating expenses</t>
         </is>
       </c>
-      <c r="C30" s="18" t="n">
+      <c r="C30" s="19" t="n">
         <v>8283042000</v>
       </c>
       <c r="D30" s="4" t="inlineStr">
@@ -72674,7 +72894,7 @@
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="C31" s="18" t="n">
+      <c r="C31" s="19" t="n">
         <v>401386000</v>
       </c>
       <c r="D31" s="4" t="inlineStr">
@@ -72699,7 +72919,7 @@
           <t>Interest</t>
         </is>
       </c>
-      <c r="C32" s="18" t="n">
+      <c r="C32" s="19" t="n">
         <v>215170000</v>
       </c>
       <c r="D32" s="4" t="inlineStr">
@@ -72724,7 +72944,7 @@
           <t>Salaries and wages</t>
         </is>
       </c>
-      <c r="C33" s="18" t="n">
+      <c r="C33" s="19" t="n">
         <v>5041664000</v>
       </c>
       <c r="D33" s="4" t="inlineStr">
@@ -72749,7 +72969,7 @@
           <t>Total operating expenses</t>
         </is>
       </c>
-      <c r="C34" s="18" t="n">
+      <c r="C34" s="19" t="n">
         <v>10953208000</v>
       </c>
       <c r="D34" s="4" t="inlineStr">
@@ -72774,7 +72994,7 @@
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="C35" s="18" t="n">
+      <c r="C35" s="19" t="n">
         <v>471677000</v>
       </c>
       <c r="D35" s="4" t="inlineStr">
@@ -72799,7 +73019,7 @@
           <t>Interest</t>
         </is>
       </c>
-      <c r="C36" s="18" t="n">
+      <c r="C36" s="19" t="n">
         <v>161512000</v>
       </c>
       <c r="D36" s="4" t="inlineStr">
@@ -72824,7 +73044,7 @@
           <t>Salaries and wages</t>
         </is>
       </c>
-      <c r="C37" s="18" t="n">
+      <c r="C37" s="19" t="n">
         <v>5265449000</v>
       </c>
       <c r="D37" s="4" t="inlineStr">
@@ -72849,7 +73069,7 @@
           <t>Total operating expenses</t>
         </is>
       </c>
-      <c r="C38" s="18" t="n">
+      <c r="C38" s="19" t="n">
         <v>10577959000</v>
       </c>
       <c r="D38" s="4" t="inlineStr">
@@ -72874,7 +73094,7 @@
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="C39" s="18" t="n">
+      <c r="C39" s="19" t="n">
         <v>379158000</v>
       </c>
       <c r="D39" s="4" t="inlineStr">
@@ -72899,7 +73119,7 @@
           <t>Interest</t>
         </is>
       </c>
-      <c r="C40" s="18" t="n">
+      <c r="C40" s="19" t="n">
         <v>113892000</v>
       </c>
       <c r="D40" s="4" t="inlineStr">
@@ -72924,7 +73144,7 @@
           <t>Salaries and wages</t>
         </is>
       </c>
-      <c r="C41" s="18" t="n"/>
+      <c r="C41" s="19" t="n"/>
       <c r="D41" s="4" t="inlineStr">
         <is>
           <t>NOT DISCLOSED. Statement of Activities (Expenses) shows only 'Compensation and benefits 9,019,270' (in thousands, 2025 column), combined; no separate salaries and wages or benefits line anywhere in the statements or notes (searched full text for 'salar' and 'wages'). FY25 report, printed p.2 (PDF p.6).</t>
@@ -72947,7 +73167,7 @@
           <t>Total operating expenses</t>
         </is>
       </c>
-      <c r="C42" s="18" t="n">
+      <c r="C42" s="19" t="n">
         <v>16445321000</v>
       </c>
       <c r="D42" s="4" t="inlineStr">
@@ -72972,7 +73192,7 @@
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="C43" s="18" t="n">
+      <c r="C43" s="19" t="n">
         <v>686510000</v>
       </c>
       <c r="D43" s="4" t="inlineStr">
@@ -72997,7 +73217,7 @@
           <t>Interest</t>
         </is>
       </c>
-      <c r="C44" s="18" t="n">
+      <c r="C44" s="19" t="n">
         <v>133923000</v>
       </c>
       <c r="D44" s="4" t="inlineStr">
@@ -73022,7 +73242,7 @@
           <t>Salaries and wages</t>
         </is>
       </c>
-      <c r="C45" s="18" t="n"/>
+      <c r="C45" s="19" t="n"/>
       <c r="D45" s="4" t="inlineStr">
         <is>
           <t>Not separately reported. Statement of activities row: 'Salaries and benefits  11,647,045  10,757,678' (thousands), FY25 report PDF p.15. Note (p.55) also shows only 'SALARIES AND BENEFITS'.</t>
@@ -73045,7 +73265,7 @@
           <t>Total operating expenses</t>
         </is>
       </c>
-      <c r="C46" s="18" t="n">
+      <c r="C46" s="19" t="n">
         <v>18935447000</v>
       </c>
       <c r="D46" s="4" t="inlineStr">
@@ -73070,7 +73290,7 @@
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="C47" s="18" t="n">
+      <c r="C47" s="19" t="n">
         <v>930917000</v>
       </c>
       <c r="D47" s="4" t="inlineStr">
@@ -73095,7 +73315,7 @@
           <t>Interest</t>
         </is>
       </c>
-      <c r="C48" s="18" t="n">
+      <c r="C48" s="19" t="n">
         <v>278763000</v>
       </c>
       <c r="D48" s="4" t="inlineStr">
@@ -73120,7 +73340,7 @@
           <t>Salaries and wages</t>
         </is>
       </c>
-      <c r="C49" s="18" t="n"/>
+      <c r="C49" s="19" t="n"/>
       <c r="D49" s="4" t="inlineStr">
         <is>
           <t>Not separately reported. Only 'Salary and benefits  1,341,049' (thousands) on the Consolidated Statement of Activities, 2025 column, and Note 14 total row 'Total $1,341,049 $846,088 $151,250 $49,862 $2,388,249'. FY25 report PDF p6 (printed p4) and PDF p28 (printed p26).</t>
@@ -73143,7 +73363,7 @@
           <t>Total operating expenses</t>
         </is>
       </c>
-      <c r="C50" s="18" t="n">
+      <c r="C50" s="19" t="n">
         <v>2388249000</v>
       </c>
       <c r="D50" s="4" t="inlineStr">
@@ -73168,7 +73388,7 @@
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="C51" s="18" t="n">
+      <c r="C51" s="19" t="n">
         <v>151250000</v>
       </c>
       <c r="D51" s="4" t="inlineStr">
@@ -73193,7 +73413,7 @@
           <t>Interest</t>
         </is>
       </c>
-      <c r="C52" s="18" t="n">
+      <c r="C52" s="19" t="n">
         <v>49862000</v>
       </c>
       <c r="D52" s="4" t="inlineStr">
@@ -73218,7 +73438,7 @@
           <t>Salaries and wages</t>
         </is>
       </c>
-      <c r="C53" s="18" t="n">
+      <c r="C53" s="19" t="n">
         <v>1238476000</v>
       </c>
       <c r="D53" s="4" t="inlineStr">
@@ -73243,7 +73463,7 @@
           <t>Total operating expenses</t>
         </is>
       </c>
-      <c r="C54" s="18" t="n">
+      <c r="C54" s="19" t="n">
         <v>2719848000</v>
       </c>
       <c r="D54" s="4" t="inlineStr">
@@ -73268,7 +73488,7 @@
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="C55" s="18" t="n">
+      <c r="C55" s="19" t="n">
         <v>160697000</v>
       </c>
       <c r="D55" s="4" t="inlineStr">
@@ -73293,7 +73513,7 @@
           <t>Interest</t>
         </is>
       </c>
-      <c r="C56" s="18" t="n">
+      <c r="C56" s="19" t="n">
         <v>81689000</v>
       </c>
       <c r="D56" s="4" t="inlineStr">
@@ -73318,7 +73538,7 @@
           <t>Salaries and wages</t>
         </is>
       </c>
-      <c r="C57" s="18" t="n">
+      <c r="C57" s="19" t="n">
         <v>2090862000</v>
       </c>
       <c r="D57" s="4" t="inlineStr">
@@ -73343,7 +73563,7 @@
           <t>Total operating expenses</t>
         </is>
       </c>
-      <c r="C58" s="18" t="n">
+      <c r="C58" s="19" t="n">
         <v>5117184000</v>
       </c>
       <c r="D58" s="4" t="inlineStr">
@@ -73368,7 +73588,7 @@
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="C59" s="18" t="n">
+      <c r="C59" s="19" t="n">
         <v>289575000</v>
       </c>
       <c r="D59" s="4" t="inlineStr">
@@ -73393,7 +73613,7 @@
           <t>Interest</t>
         </is>
       </c>
-      <c r="C60" s="18" t="n">
+      <c r="C60" s="19" t="n">
         <v>170489000</v>
       </c>
       <c r="D60" s="4" t="inlineStr">
@@ -73425,7 +73645,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -73488,7 +73708,7 @@
           <t>6,273 rows in the June 2026 file -&gt; 1,527 institutions (584 public, 943 private) after CONTROL, CCBASIC 15-23, CCUGPROF 5-15, net price and 10-year earnings present. The original release had 1,557.</t>
         </is>
       </c>
-      <c r="E4" s="26" t="inlineStr">
+      <c r="E4" s="27" t="inlineStr">
         <is>
           <t>Pass</t>
         </is>
@@ -73513,7 +73733,7 @@
           <t>Northeastern 33rd of 1,527 (29th of 943 private; ties with its 'Northeastern University Oakland' row at $92,538). Vanderbilt 38th, Boston University 77th, MIT 1st. Earlier release: 38th / 53rd / 75th / 2nd.</t>
         </is>
       </c>
-      <c r="E5" s="26" t="inlineStr">
+      <c r="E5" s="27" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -73538,7 +73758,7 @@
           <t>No. Net price is now AY2023-24 (IPEDS 2024-25 collection). 10-year earnings are the pooled AY2009-10 / 2010-11 entry cohorts measured CY2020-21 in 2022 dollars; the last 10-year refresh was June 13, 2024 and no later cohort exists. Scorecard was updated June 10, 2026 for IPEDS and FSA items.</t>
         </is>
       </c>
-      <c r="E6" s="26" t="inlineStr">
+      <c r="E6" s="27" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -73563,7 +73783,7 @@
           <t>OLS on private institutions: slope 0.924, intercept $34,026, r 0.47, R-squared 0.22. Weak fit: 'better deal / worse deal' is directional.</t>
         </is>
       </c>
-      <c r="E7" s="26" t="inlineStr">
+      <c r="E7" s="27" t="inlineStr">
         <is>
           <t>Pass / caveat</t>
         </is>
@@ -73588,7 +73808,7 @@
           <t>The field is measured 10 years after entry (enrollment). Slide says 'after entry'.</t>
         </is>
       </c>
-      <c r="E8" s="26" t="inlineStr">
+      <c r="E8" s="27" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -73613,7 +73833,7 @@
           <t>One institution reports a negative net price (Colegio Universitario de San Juan, -$778): counted in statistics, falls left of the axis. Three institutions exceed $56K net price (axis now to $60K). Cal Maritime is now Cal Poly Maritime Academy; University of the Sciences (merged into Saint Joseph's University in 2022) drops out. MIT net price is now $20,111 (the old file's $5,084 looked like an outlier).</t>
         </is>
       </c>
-      <c r="E9" s="26" t="inlineStr">
+      <c r="E9" s="27" t="inlineStr">
         <is>
           <t>Handled</t>
         </is>
@@ -73638,7 +73858,7 @@
           <t>The 2015-2024 reports all ask 'aware of and understand the financial challenges confronting my institution'. 'Realistic about' was only the 2013-2014 wording. Slide statement corrected.</t>
         </is>
       </c>
-      <c r="E10" s="26" t="inlineStr">
+      <c r="E10" s="27" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -73663,7 +73883,7 @@
           <t>2015 faculty 33 -&gt; 32; 2020 31/87/93 -&gt; 34/84/90 (the original used a private-nonprofit sub-column); 2022 28/91/91 -&gt; 53/90/91 (the 2022 chart on p.28 has misaligned rows; the detail tables give 53/90/91); 2024 44/91/95 -&gt; 39/79/88 (the original used the private-nonprofit column). 2023 and the other rows match.</t>
         </is>
       </c>
-      <c r="E11" s="26" t="inlineStr">
+      <c r="E11" s="27" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -73688,7 +73908,7 @@
           <t>Different item: 'Faculty members understand the financial challenges my institution faces when they participate in college-wide budget discussions.' Values 27 and 32 are correct for that item; marked with an asterisk.</t>
         </is>
       </c>
-      <c r="E12" s="26" t="inlineStr">
+      <c r="E12" s="27" t="inlineStr">
         <is>
           <t>Caveat</t>
         </is>
@@ -73713,7 +73933,7 @@
           <t>The three-group item was not asked. Trustees-only statement: 74% (2025, n=169, +/-7%) and 79% (2026, n=213, +/-6%). Plotted as separate open markers. No faculty or senior-administrator values exist for these years.</t>
         </is>
       </c>
-      <c r="E13" s="26" t="inlineStr">
+      <c r="E13" s="27" t="inlineStr">
         <is>
           <t>Info</t>
         </is>
@@ -73738,7 +73958,7 @@
           <t>Fielded by Gallup in the earlier editions and by Hanover Research from 2021 (n=133 in 2021; 273-416 earlier; 169-238 for 2022-2026). No margin of error is stated for 2015-2022 (6-7% for 2023-2026). Year-to-year moves of a few points are within sampling error.</t>
         </is>
       </c>
-      <c r="E14" s="26" t="inlineStr">
+      <c r="E14" s="27" t="inlineStr">
         <is>
           <t>Caveat</t>
         </is>
@@ -73763,7 +73983,7 @@
           <t>Business officers rating other groups (Sr. Administrators includes their own peers); not faculty's own view.</t>
         </is>
       </c>
-      <c r="E15" s="26" t="inlineStr">
+      <c r="E15" s="27" t="inlineStr">
         <is>
           <t>Fixed (labeled)</t>
         </is>
@@ -73788,7 +74008,7 @@
           <t>The original values equal audited total operating expenses to the dollar for every school checked (Rice, Vanderbilt, Northwestern, Princeton, Yale, Chicago, Duke, Emory, Penn, Stanford), and equal the IPEDS FY23 'total expenses' field for Rice, Vanderbilt, Northwestern, Princeton, Harvard, Duke and Penn. Depreciation, amortization and interest were never removed although the axis says they were. FY25 now follows the axis; FY23 restated is 5-15% lower (S3_FY23_Recalc).</t>
         </is>
       </c>
-      <c r="E16" s="27" t="inlineStr">
+      <c r="E16" s="28" t="inlineStr">
         <is>
           <t>Finding / fixed</t>
         </is>
@@ -73810,10 +74030,10 @@
       </c>
       <c r="D17" s="4" t="inlineStr">
         <is>
-          <t>Exactly 72.800% of each school's audited combined salaries and benefits: an undisclosed assumption. Schools that report both lines run 74.8%-81.4%, so 72.8% understates S&amp;W by 3-10%. Northwestern is now actual (Form 990 ties to the audited line); Penn and Stanford are flagged estimates using their own Form 990 shares.</t>
-        </is>
-      </c>
-      <c r="E17" s="27" t="inlineStr">
+          <t>Exactly 72.800% of each school's audited combined salaries and benefits: an undisclosed assumption. Schools that report both lines run 74.8%-81.4%, so 72.8% understates S&amp;W by 3-10%. Northwestern is now actual (Form 990 ties to the audited line); Penn and Stanford are flagged estimates.</t>
+        </is>
+      </c>
+      <c r="E17" s="28" t="inlineStr">
         <is>
           <t>Finding / fixed</t>
         </is>
@@ -73835,12 +74055,12 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Northeastern, Northwestern, Penn, Stanford, Vanderbilt combine salaries and benefits. Northeastern and Northwestern use Form 990 S&amp;W; Vanderbilt uses the MD&amp;A expense chart; Penn and Stanford are estimated (grey markers). Sensitivity in S3_Sensitivity C: using the median share of the three hospital-consolidated schools with audited splits (about 81%) instead of each school's own 990 share moves Penn by about +6% and Stanford by about +1%.</t>
-        </is>
-      </c>
-      <c r="E18" s="26" t="inlineStr">
-        <is>
-          <t>Handled / caveat</t>
+          <t>Northeastern, Northwestern, Penn, Stanford, Vanderbilt combine salaries and benefits. Northeastern and Northwestern use Form 990 S&amp;W; Vanderbilt uses the MD&amp;A expense chart. Penn and Stanford (grey markers) use S&amp;W = combined / 1.35, a 35% fringe benefit rate assumed per Northeastern's direction (74.1% S&amp;W share).</t>
+        </is>
+      </c>
+      <c r="E18" s="27" t="inlineStr">
+        <is>
+          <t>Decided / caveat</t>
         </is>
       </c>
     </row>
@@ -73855,17 +74075,17 @@
       </c>
       <c r="C19" s="4" t="inlineStr">
         <is>
-          <t>Student counts</t>
+          <t>35% fringe rate vs observed rates</t>
         </is>
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>One instrument for all: Common Data Set 2024-25 B1 total all students (fall 2024). The original mixed fall 2021 (Rice), fall 2022 (Vanderbilt), degree-seeking counts (Harvard, Penn) and round estimates (Emory, Northwestern). CDS differs materially from IPEDS for Northeastern (+24%), Chicago (-14%), Penn (-17%) and Harvard (-30%).</t>
-        </is>
-      </c>
-      <c r="E19" s="26" t="inlineStr">
-        <is>
-          <t>Handled / caveat</t>
+          <t>Schools that report both lines have fringe rates (benefits / S&amp;W) of 22.8% to 33.8% (Chicago 22.8%, Duke 23.6%, Emory 23.9%, Rice 23.9%, Princeton 30.3%, BU 31.5%, Yale 31.5%, MIT 33.8%). 35% is above all of them, so the Penn and Stanford estimates lean low: using each school's own Form 990 S&amp;W share instead would raise S&amp;W per student by about 4% (Penn) and 8% (Stanford) (S3_Sensitivity C). Neither changes the ranking of Penn or Stanford or any conclusion about Northeastern.</t>
+        </is>
+      </c>
+      <c r="E19" s="27" t="inlineStr">
+        <is>
+          <t>Caveat</t>
         </is>
       </c>
     </row>
@@ -73880,17 +74100,17 @@
       </c>
       <c r="C20" s="4" t="inlineStr">
         <is>
-          <t>Northeastern student count is the key sensitivity</t>
+          <t>Student counts</t>
         </is>
       </c>
       <c r="D20" s="4" t="inlineStr">
         <is>
-          <t>CDS 39,774 -&gt; S&amp;W per student $26.3K; IPEDS-style 32,553 -&gt; $32.1K; Facts and Figures 48,812 -&gt; $21.4K. Northeastern is lowest in the peer set on all three (S3_Sensitivity A, B). Confirm the official count with University Decision Support.</t>
+          <t>One instrument for all: Common Data Set 2024-25 B1 total all students (fall 2024). The original mixed fall 2021 (Rice), fall 2022 (Vanderbilt), degree-seeking counts (Harvard, Penn) and round estimates (Emory, Northwestern). CDS differs materially from IPEDS for Northeastern (+24%), Chicago (-14%), Penn (-17%) and Harvard (-30%).</t>
         </is>
       </c>
       <c r="E20" s="27" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Handled / caveat</t>
         </is>
       </c>
     </row>
@@ -73905,17 +74125,17 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>Headcount vs FTE</t>
+          <t>Northeastern student count is the key sensitivity</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>Northeastern and BU headcounts include large graduate, online and co-op populations (BU reports 29.6K FTE against 37.7K headcount), so S&amp;W per headcount student understates S&amp;W per FTE student for both.</t>
-        </is>
-      </c>
-      <c r="E21" s="26" t="inlineStr">
-        <is>
-          <t>Caveat</t>
+          <t>CDS 39,774 (used, per Northeastern's direction) -&gt; S&amp;W per student $26.3K; IPEDS-style 32,553 -&gt; $32.1K; Facts and Figures 48,812 -&gt; $21.4K. Northeastern is lowest in the peer set on all three (S3_Sensitivity A, B).</t>
+        </is>
+      </c>
+      <c r="E21" s="27" t="inlineStr">
+        <is>
+          <t>Decided</t>
         </is>
       </c>
     </row>
@@ -73930,15 +74150,15 @@
       </c>
       <c r="C22" s="4" t="inlineStr">
         <is>
-          <t>Northeastern S&amp;W scope</t>
+          <t>Headcount vs FTE</t>
         </is>
       </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>Form 990 (university) lines 5-10 are 96.8% of the audited combined line; S&amp;W may be understated by about 3% against the consolidated core expenses.</t>
-        </is>
-      </c>
-      <c r="E22" s="26" t="inlineStr">
+          <t>Northeastern and BU headcounts include large graduate, online and co-op populations (BU reports 29.6K FTE against 37.7K headcount), so S&amp;W per headcount student understates S&amp;W per FTE student for both.</t>
+        </is>
+      </c>
+      <c r="E22" s="27" t="inlineStr">
         <is>
           <t>Caveat</t>
         </is>
@@ -73955,17 +74175,17 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>FY23 to FY24 comparability</t>
+          <t>Northeastern S&amp;W scope</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Duke's FY24 includes the July 1, 2023 physician-practice acquisition (S&amp;W +29.5%); FY25 is unaffected. Rice's FY25 scholarship presentation changed (total and core not strictly comparable with FY24). Emory FY25 includes three months of Houston Healthcare. Northeastern FY25 includes two weeks of Marymount Manhattan College.</t>
-        </is>
-      </c>
-      <c r="E23" s="26" t="inlineStr">
-        <is>
-          <t>Info</t>
+          <t>Form 990 (university) lines 5-10 are 96.8% of the audited combined line; S&amp;W may be understated by about 3% against the consolidated core expenses.</t>
+        </is>
+      </c>
+      <c r="E23" s="27" t="inlineStr">
+        <is>
+          <t>Caveat</t>
         </is>
       </c>
     </row>
@@ -73980,17 +74200,17 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>Entities inside the numbers</t>
+          <t>FY23 to FY24 comparability</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Consolidated: hospitals at Chicago, Duke, Emory, Penn, Stanford; Lincoln Laboratory (MIT), Plasma Physics Laboratory (Princeton), SLAC (Stanford). Not consolidated: Northwestern Medicine, VUMC, Yale New Haven Hospital, Boston Medical Center, Argonne, Fermilab. Footnoted on the slide.</t>
-        </is>
-      </c>
-      <c r="E24" s="26" t="inlineStr">
-        <is>
-          <t>Handled</t>
+          <t>Duke's FY24 includes the July 1, 2023 physician-practice acquisition (S&amp;W +29.5%); FY25 is unaffected. Rice's FY25 scholarship presentation changed (total and core not strictly comparable with FY24). Emory FY25 includes three months of Houston Healthcare. Northeastern FY25 includes two weeks of Marymount Manhattan College.</t>
+        </is>
+      </c>
+      <c r="E24" s="27" t="inlineStr">
+        <is>
+          <t>Info</t>
         </is>
       </c>
     </row>
@@ -74005,17 +74225,17 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Arithmetic</t>
+          <t>Entities inside the numbers</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>For every school, core = total - depreciation - amortization - interest (formula), S&amp;W per student = x * y (column Q = 0), and the natural-classification lines sum to total operating expenses in every year (as reported by the extraction). Key rows for Northeastern, BU and MIT re-checked against the PDFs.</t>
-        </is>
-      </c>
-      <c r="E25" s="26" t="inlineStr">
-        <is>
-          <t>Pass</t>
+          <t>Consolidated: hospitals at Chicago, Duke, Emory, Penn, Stanford; Lincoln Laboratory (MIT), Plasma Physics Laboratory (Princeton), SLAC (Stanford). Not consolidated: Northwestern Medicine, VUMC, Yale New Haven Hospital, Boston Medical Center, Argonne, Fermilab. Footnoted on the slide.</t>
+        </is>
+      </c>
+      <c r="E25" s="27" t="inlineStr">
+        <is>
+          <t>Handled</t>
         </is>
       </c>
     </row>
@@ -74030,17 +74250,17 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Harvard</t>
+          <t>Arithmetic</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>The FY25 Financial Report could not be reached (finance.harvard.edu denies automated access). Harvard is not on the FY25 chart; CDS fall 2024 enrollment (21,189) is recorded.</t>
+          <t>For every school, core = total - depreciation - amortization - interest (formula), S&amp;W per student = x * y (column Q = 0), and the natural-classification lines sum to total operating expenses in every year (as reported by the extraction). Key rows for Northeastern, BU and MIT re-checked against the PDFs.</t>
         </is>
       </c>
       <c r="E26" s="27" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -74055,15 +74275,40 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
+          <t>Harvard</t>
+        </is>
+      </c>
+      <c r="D27" s="4" t="inlineStr">
+        <is>
+          <t>The FY25 Financial Report could not be reached (finance.harvard.edu denies automated access). Harvard is not on the FY25 chart; CDS fall 2024 enrollment (21,189) is recorded.</t>
+        </is>
+      </c>
+      <c r="E27" s="28" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="B28" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C28" s="4" t="inlineStr">
+        <is>
           <t>Original chart construction</t>
         </is>
       </c>
-      <c r="D27" s="4" t="inlineStr">
+      <c r="D28" s="4" t="inlineStr">
         <is>
           <t>The original plotted only the eight iso-lines; logos were hand-placed pictures, so positions did not come from data, and Stanford's x-value exceeded the axis maximum. Rebuilt with real data points.</t>
         </is>
       </c>
-      <c r="E27" s="26" t="inlineStr">
+      <c r="E28" s="27" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>

</xml_diff>

<commit_message>
Add Harvard to slide 3 from its FY25 audited financial report
Harvard: S&W $2,759M, total operating expenses $6,794M less depreciation $459M and interest $263M = core $6,073M; 21,189 students (CDS) = $130K S&W per student, 45% S&W share.
Workbook: Harvard row with live formulas, evidence, sensitivity E (Extension School), checks. Removed the pending draft tag and note.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCNX7EgSWHMHv9UtVBoXog
</commit_message>
<xml_diff>
--- a/nu-peer-slides/NU_peer_slides_backup.xlsx
+++ b/nu-peer-slides/NU_peer_slides_backup.xlsx
@@ -601,7 +601,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>What is still open (Harvard FY25 report; Northeastern headcount confirmation; Penn / Stanford salaries and wages).</t>
+          <t>What is still open (optional: Penn / Stanford consolidated salaries and wages; Princeton CDS; Harvard FY23 report for calibration).</t>
         </is>
       </c>
     </row>
@@ -662,17 +662,17 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Harvard FY25 Financial Report (and FY23 for calibration)</t>
+          <t>Harvard FY23 Financial Report (optional)</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>finance.harvard.edu denies automated access; the PDFs are public.</t>
+          <t>Only needed to add Harvard to the FY23 recalculation sheet; the FY25 chart does not depend on it.</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Download the FY25 Harvard Financial Report from finance.harvard.edu (Financial Reports) in a browser and upload; I will add Harvard to the chart.</t>
+          <t>Upload the FY23 or FY24 Harvard Financial Report if you want the calibration row.</t>
         </is>
       </c>
     </row>
@@ -69332,17 +69332,58 @@
           <t>June 30, 2025</t>
         </is>
       </c>
-      <c r="D9" s="13" t="inlineStr">
-        <is>
-          <t>pending</t>
-        </is>
+      <c r="C9" s="19" t="n">
+        <v>2758560000</v>
+      </c>
+      <c r="D9" s="9" t="inlineStr">
+        <is>
+          <t>audited line</t>
+        </is>
+      </c>
+      <c r="E9" s="19">
+        <f>C9+755895000</f>
+        <v/>
+      </c>
+      <c r="H9" s="19" t="n">
+        <v>6794371000</v>
+      </c>
+      <c r="I9" s="19" t="n">
+        <v>459031000</v>
+      </c>
+      <c r="K9" s="19" t="n">
+        <v>262546000</v>
+      </c>
+      <c r="L9" s="19">
+        <f>H9-I9-J9-K9</f>
+        <v/>
       </c>
       <c r="M9" s="19" t="n">
         <v>21189</v>
       </c>
+      <c r="N9" s="11">
+        <f>C9/M9</f>
+        <v/>
+      </c>
+      <c r="O9" s="11">
+        <f>L9/M9</f>
+        <v/>
+      </c>
+      <c r="P9" s="20">
+        <f>C9/L9</f>
+        <v/>
+      </c>
+      <c r="Q9" s="21">
+        <f>O9*P9-N9</f>
+        <v/>
+      </c>
+      <c r="R9" s="9" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
       <c r="S9" s="4" t="inlineStr">
         <is>
-          <t>PENDING: Harvard's finance site denies automated access; FY25 Financial Report PDF needed.</t>
+          <t>Separate S&amp;W and benefits lines in the FY25 audited Financial Report (supplied by Northeastern; Statement of Changes in Net Assets, PDF p.18). Depreciation and interest are separate operating lines; nine natural-classification lines sum to total operating expenses. No hospital consolidated. CDS students exclude the Harvard Extension School although expenses include it (S3_Sensitivity E).</t>
         </is>
       </c>
     </row>
@@ -69955,7 +69996,7 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>Median (13 schools with data)</t>
+          <t>Median (14 schools)</t>
         </is>
       </c>
       <c r="N20" s="8">
@@ -70004,7 +70045,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J43"/>
+  <dimension ref="A1:J52"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -70202,11 +70243,11 @@
         <v/>
       </c>
       <c r="F12" s="16">
-        <f>RANK(D12,D$12:D$24,1)</f>
+        <f>RANK(D12,D$12:D$25,1)</f>
         <v/>
       </c>
       <c r="G12" s="16">
-        <f>RANK(E12,E$12:E$24,1)</f>
+        <f>RANK(E12,E$12:E$25,1)</f>
         <v/>
       </c>
       <c r="H12" s="25">
@@ -70236,11 +70277,11 @@
         <v/>
       </c>
       <c r="F13" s="16">
-        <f>RANK(D13,D$12:D$24,1)</f>
+        <f>RANK(D13,D$12:D$25,1)</f>
         <v/>
       </c>
       <c r="G13" s="16">
-        <f>RANK(E13,E$12:E$24,1)</f>
+        <f>RANK(E13,E$12:E$25,1)</f>
         <v/>
       </c>
       <c r="H13" s="25">
@@ -70270,11 +70311,11 @@
         <v/>
       </c>
       <c r="F14" s="16">
-        <f>RANK(D14,D$12:D$24,1)</f>
+        <f>RANK(D14,D$12:D$25,1)</f>
         <v/>
       </c>
       <c r="G14" s="16">
-        <f>RANK(E14,E$12:E$24,1)</f>
+        <f>RANK(E14,E$12:E$25,1)</f>
         <v/>
       </c>
       <c r="H14" s="25">
@@ -70304,11 +70345,11 @@
         <v/>
       </c>
       <c r="F15" s="16">
-        <f>RANK(D15,D$12:D$24,1)</f>
+        <f>RANK(D15,D$12:D$25,1)</f>
         <v/>
       </c>
       <c r="G15" s="16">
-        <f>RANK(E15,E$12:E$24,1)</f>
+        <f>RANK(E15,E$12:E$25,1)</f>
         <v/>
       </c>
       <c r="H15" s="25">
@@ -70319,30 +70360,30 @@
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>Yale</t>
+          <t>Harvard</t>
         </is>
       </c>
       <c r="B16" s="19">
-        <f>S3_FY25!M10</f>
+        <f>S3_FY25!M9</f>
         <v/>
       </c>
       <c r="C16" s="19" t="n">
-        <v>15081</v>
+        <v>30386</v>
       </c>
       <c r="D16" s="11">
-        <f>S3_FY25!C10/B16</f>
+        <f>S3_FY25!C9/B16</f>
         <v/>
       </c>
       <c r="E16" s="11">
-        <f>S3_FY25!C10/C16</f>
+        <f>S3_FY25!C9/C16</f>
         <v/>
       </c>
       <c r="F16" s="16">
-        <f>RANK(D16,D$12:D$24,1)</f>
+        <f>RANK(D16,D$12:D$25,1)</f>
         <v/>
       </c>
       <c r="G16" s="16">
-        <f>RANK(E16,E$12:E$24,1)</f>
+        <f>RANK(E16,E$12:E$25,1)</f>
         <v/>
       </c>
       <c r="H16" s="25">
@@ -70353,30 +70394,30 @@
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Yale</t>
         </is>
       </c>
       <c r="B17" s="19">
-        <f>S3_FY25!M11</f>
+        <f>S3_FY25!M10</f>
         <v/>
       </c>
       <c r="C17" s="19" t="n">
-        <v>18339</v>
+        <v>15081</v>
       </c>
       <c r="D17" s="11">
-        <f>S3_FY25!C11/B17</f>
+        <f>S3_FY25!C10/B17</f>
         <v/>
       </c>
       <c r="E17" s="11">
-        <f>S3_FY25!C11/C17</f>
+        <f>S3_FY25!C10/C17</f>
         <v/>
       </c>
       <c r="F17" s="16">
-        <f>RANK(D17,D$12:D$24,1)</f>
+        <f>RANK(D17,D$12:D$25,1)</f>
         <v/>
       </c>
       <c r="G17" s="16">
-        <f>RANK(E17,E$12:E$24,1)</f>
+        <f>RANK(E17,E$12:E$25,1)</f>
         <v/>
       </c>
       <c r="H17" s="25">
@@ -70387,30 +70428,30 @@
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>Duke</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="B18" s="19">
-        <f>S3_FY25!M12</f>
+        <f>S3_FY25!M11</f>
         <v/>
       </c>
       <c r="C18" s="19" t="n">
-        <v>17112</v>
+        <v>18339</v>
       </c>
       <c r="D18" s="11">
-        <f>S3_FY25!C12/B18</f>
+        <f>S3_FY25!C11/B18</f>
         <v/>
       </c>
       <c r="E18" s="11">
-        <f>S3_FY25!C12/C18</f>
+        <f>S3_FY25!C11/C18</f>
         <v/>
       </c>
       <c r="F18" s="16">
-        <f>RANK(D18,D$12:D$24,1)</f>
+        <f>RANK(D18,D$12:D$25,1)</f>
         <v/>
       </c>
       <c r="G18" s="16">
-        <f>RANK(E18,E$12:E$24,1)</f>
+        <f>RANK(E18,E$12:E$25,1)</f>
         <v/>
       </c>
       <c r="H18" s="25">
@@ -70421,30 +70462,30 @@
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>Emory</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="B19" s="19">
-        <f>S3_FY25!M13</f>
+        <f>S3_FY25!M12</f>
         <v/>
       </c>
       <c r="C19" s="19" t="n">
-        <v>15046</v>
+        <v>17112</v>
       </c>
       <c r="D19" s="11">
-        <f>S3_FY25!C13/B19</f>
+        <f>S3_FY25!C12/B19</f>
         <v/>
       </c>
       <c r="E19" s="11">
-        <f>S3_FY25!C13/C19</f>
+        <f>S3_FY25!C12/C19</f>
         <v/>
       </c>
       <c r="F19" s="16">
-        <f>RANK(D19,D$12:D$24,1)</f>
+        <f>RANK(D19,D$12:D$25,1)</f>
         <v/>
       </c>
       <c r="G19" s="16">
-        <f>RANK(E19,E$12:E$24,1)</f>
+        <f>RANK(E19,E$12:E$25,1)</f>
         <v/>
       </c>
       <c r="H19" s="25">
@@ -70455,30 +70496,30 @@
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Penn</t>
+          <t>Emory</t>
         </is>
       </c>
       <c r="B20" s="19">
-        <f>S3_FY25!M14</f>
+        <f>S3_FY25!M13</f>
         <v/>
       </c>
       <c r="C20" s="19" t="n">
-        <v>28711</v>
+        <v>15046</v>
       </c>
       <c r="D20" s="11">
-        <f>S3_FY25!C14/B20</f>
+        <f>S3_FY25!C13/B20</f>
         <v/>
       </c>
       <c r="E20" s="11">
-        <f>S3_FY25!C14/C20</f>
+        <f>S3_FY25!C13/C20</f>
         <v/>
       </c>
       <c r="F20" s="16">
-        <f>RANK(D20,D$12:D$24,1)</f>
+        <f>RANK(D20,D$12:D$25,1)</f>
         <v/>
       </c>
       <c r="G20" s="16">
-        <f>RANK(E20,E$12:E$24,1)</f>
+        <f>RANK(E20,E$12:E$25,1)</f>
         <v/>
       </c>
       <c r="H20" s="25">
@@ -70489,30 +70530,30 @@
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>Stanford</t>
+          <t>Penn</t>
         </is>
       </c>
       <c r="B21" s="19">
-        <f>S3_FY25!M15</f>
+        <f>S3_FY25!M14</f>
         <v/>
       </c>
       <c r="C21" s="19" t="n">
-        <v>18446</v>
+        <v>28711</v>
       </c>
       <c r="D21" s="11">
-        <f>S3_FY25!C15/B21</f>
+        <f>S3_FY25!C14/B21</f>
         <v/>
       </c>
       <c r="E21" s="11">
-        <f>S3_FY25!C15/C21</f>
+        <f>S3_FY25!C14/C21</f>
         <v/>
       </c>
       <c r="F21" s="16">
-        <f>RANK(D21,D$12:D$24,1)</f>
+        <f>RANK(D21,D$12:D$25,1)</f>
         <v/>
       </c>
       <c r="G21" s="16">
-        <f>RANK(E21,E$12:E$24,1)</f>
+        <f>RANK(E21,E$12:E$25,1)</f>
         <v/>
       </c>
       <c r="H21" s="25">
@@ -70523,30 +70564,30 @@
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Northeastern</t>
+          <t>Stanford</t>
         </is>
       </c>
       <c r="B22" s="19">
-        <f>S3_FY25!M16</f>
+        <f>S3_FY25!M15</f>
         <v/>
       </c>
       <c r="C22" s="19" t="n">
-        <v>31159</v>
+        <v>18446</v>
       </c>
       <c r="D22" s="11">
-        <f>S3_FY25!C16/B22</f>
+        <f>S3_FY25!C15/B22</f>
         <v/>
       </c>
       <c r="E22" s="11">
-        <f>S3_FY25!C16/C22</f>
+        <f>S3_FY25!C15/C22</f>
         <v/>
       </c>
       <c r="F22" s="16">
-        <f>RANK(D22,D$12:D$24,1)</f>
+        <f>RANK(D22,D$12:D$25,1)</f>
         <v/>
       </c>
       <c r="G22" s="16">
-        <f>RANK(E22,E$12:E$24,1)</f>
+        <f>RANK(E22,E$12:E$25,1)</f>
         <v/>
       </c>
       <c r="H22" s="25">
@@ -70557,30 +70598,30 @@
     <row r="23">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>Boston University</t>
+          <t>Northeastern</t>
         </is>
       </c>
       <c r="B23" s="19">
-        <f>S3_FY25!M17</f>
+        <f>S3_FY25!M16</f>
         <v/>
       </c>
       <c r="C23" s="19" t="n">
-        <v>36624</v>
+        <v>31159</v>
       </c>
       <c r="D23" s="11">
-        <f>S3_FY25!C17/B23</f>
+        <f>S3_FY25!C16/B23</f>
         <v/>
       </c>
       <c r="E23" s="11">
-        <f>S3_FY25!C17/C23</f>
+        <f>S3_FY25!C16/C23</f>
         <v/>
       </c>
       <c r="F23" s="16">
-        <f>RANK(D23,D$12:D$24,1)</f>
+        <f>RANK(D23,D$12:D$25,1)</f>
         <v/>
       </c>
       <c r="G23" s="16">
-        <f>RANK(E23,E$12:E$24,1)</f>
+        <f>RANK(E23,E$12:E$25,1)</f>
         <v/>
       </c>
       <c r="H23" s="25">
@@ -70591,30 +70632,30 @@
     <row r="24">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>Boston University</t>
         </is>
       </c>
       <c r="B24" s="19">
-        <f>S3_FY25!M18</f>
+        <f>S3_FY25!M17</f>
         <v/>
       </c>
       <c r="C24" s="19" t="n">
-        <v>11920</v>
+        <v>36624</v>
       </c>
       <c r="D24" s="11">
-        <f>S3_FY25!C18/B24</f>
+        <f>S3_FY25!C17/B24</f>
         <v/>
       </c>
       <c r="E24" s="11">
-        <f>S3_FY25!C18/C24</f>
+        <f>S3_FY25!C17/C24</f>
         <v/>
       </c>
       <c r="F24" s="16">
-        <f>RANK(D24,D$12:D$24,1)</f>
+        <f>RANK(D24,D$12:D$25,1)</f>
         <v/>
       </c>
       <c r="G24" s="16">
-        <f>RANK(E24,E$12:E$24,1)</f>
+        <f>RANK(E24,E$12:E$25,1)</f>
         <v/>
       </c>
       <c r="H24" s="25">
@@ -70622,115 +70663,107 @@
         <v/>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" s="3" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="B25" s="19">
+        <f>S3_FY25!M18</f>
+        <v/>
+      </c>
+      <c r="C25" s="19" t="n">
+        <v>11920</v>
+      </c>
+      <c r="D25" s="11">
+        <f>S3_FY25!C18/B25</f>
+        <v/>
+      </c>
+      <c r="E25" s="11">
+        <f>S3_FY25!C18/C25</f>
+        <v/>
+      </c>
+      <c r="F25" s="16">
+        <f>RANK(D25,D$12:D$25,1)</f>
+        <v/>
+      </c>
+      <c r="G25" s="16">
+        <f>RANK(E25,E$12:E$25,1)</f>
+        <v/>
+      </c>
+      <c r="H25" s="25">
+        <f>(C25/B25-1)*100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="3" t="inlineStr">
         <is>
           <t>C. Penn and Stanford estimated S&amp;W under alternative assumptions</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="B28" s="5" t="inlineStr">
+      <c r="B29" s="5" t="inlineStr">
         <is>
           <t>Salaries + benefits ($)</t>
         </is>
       </c>
-      <c r="C28" s="5" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>Fringe rate used (input on S3_FY25)</t>
         </is>
       </c>
-      <c r="D28" s="5" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>S&amp;W per student, used</t>
         </is>
       </c>
-      <c r="E28" s="5" t="inlineStr">
+      <c r="E29" s="5" t="inlineStr">
         <is>
           <t>Alt 1: own Form 990 S&amp;W share</t>
         </is>
       </c>
-      <c r="F28" s="5" t="inlineStr">
+      <c r="F29" s="5" t="inlineStr">
         <is>
           <t>S&amp;W per student, Alt 1</t>
         </is>
       </c>
-      <c r="G28" s="5" t="inlineStr">
+      <c r="G29" s="5" t="inlineStr">
         <is>
           <t>Alt 1 vs used (%)</t>
         </is>
       </c>
-      <c r="H28" s="5" t="inlineStr">
+      <c r="H29" s="5" t="inlineStr">
         <is>
           <t>Alt 2: original slide 72.8%</t>
         </is>
       </c>
-      <c r="I28" s="5" t="inlineStr">
+      <c r="I29" s="5" t="inlineStr">
         <is>
           <t>S&amp;W per student, Alt 2</t>
         </is>
       </c>
-      <c r="J28" s="5" t="inlineStr">
+      <c r="J29" s="5" t="inlineStr">
         <is>
           <t>Alt 2 vs used (%)</t>
         </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="9" t="inlineStr">
-        <is>
-          <t>Penn</t>
-        </is>
-      </c>
-      <c r="B29" s="19">
-        <f>S3_FY25!E14</f>
-        <v/>
-      </c>
-      <c r="C29" s="15">
-        <f>S3_FY25!E3</f>
-        <v/>
-      </c>
-      <c r="D29" s="11">
-        <f>B29/(1+C29)/S3_FY25!M14</f>
-        <v/>
-      </c>
-      <c r="E29" s="20">
-        <f>S3_FY25!F14/S3_FY25!G14</f>
-        <v/>
-      </c>
-      <c r="F29" s="11">
-        <f>B29*E29/S3_FY25!M14</f>
-        <v/>
-      </c>
-      <c r="G29" s="25">
-        <f>(F29/D29-1)*100</f>
-        <v/>
-      </c>
-      <c r="H29" s="20" t="n">
-        <v>0.728</v>
-      </c>
-      <c r="I29" s="11">
-        <f>B29*H29/S3_FY25!M14</f>
-        <v/>
-      </c>
-      <c r="J29" s="25">
-        <f>(I29/D29-1)*100</f>
-        <v/>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="9" t="inlineStr">
         <is>
-          <t>Stanford</t>
+          <t>Penn</t>
         </is>
       </c>
       <c r="B30" s="19">
-        <f>S3_FY25!E15</f>
+        <f>S3_FY25!E14</f>
         <v/>
       </c>
       <c r="C30" s="15">
@@ -70738,15 +70771,15 @@
         <v/>
       </c>
       <c r="D30" s="11">
-        <f>B30/(1+C30)/S3_FY25!M15</f>
+        <f>B30/(1+C30)/S3_FY25!M14</f>
         <v/>
       </c>
       <c r="E30" s="20">
-        <f>S3_FY25!F15/S3_FY25!G15</f>
+        <f>S3_FY25!F14/S3_FY25!G14</f>
         <v/>
       </c>
       <c r="F30" s="11">
-        <f>B30*E30/S3_FY25!M15</f>
+        <f>B30*E30/S3_FY25!M14</f>
         <v/>
       </c>
       <c r="G30" s="25">
@@ -70757,7 +70790,7 @@
         <v>0.728</v>
       </c>
       <c r="I30" s="11">
-        <f>B30*H30/S3_FY25!M15</f>
+        <f>B30*H30/S3_FY25!M14</f>
         <v/>
       </c>
       <c r="J30" s="25">
@@ -70765,66 +70798,89 @@
         <v/>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="3" t="inlineStr">
+    <row r="31">
+      <c r="A31" s="9" t="inlineStr">
+        <is>
+          <t>Stanford</t>
+        </is>
+      </c>
+      <c r="B31" s="19">
+        <f>S3_FY25!E15</f>
+        <v/>
+      </c>
+      <c r="C31" s="15">
+        <f>S3_FY25!E3</f>
+        <v/>
+      </c>
+      <c r="D31" s="11">
+        <f>B31/(1+C31)/S3_FY25!M15</f>
+        <v/>
+      </c>
+      <c r="E31" s="20">
+        <f>S3_FY25!F15/S3_FY25!G15</f>
+        <v/>
+      </c>
+      <c r="F31" s="11">
+        <f>B31*E31/S3_FY25!M15</f>
+        <v/>
+      </c>
+      <c r="G31" s="25">
+        <f>(F31/D31-1)*100</f>
+        <v/>
+      </c>
+      <c r="H31" s="20" t="n">
+        <v>0.728</v>
+      </c>
+      <c r="I31" s="11">
+        <f>B31*H31/S3_FY25!M15</f>
+        <v/>
+      </c>
+      <c r="J31" s="25">
+        <f>(I31/D31-1)*100</f>
+        <v/>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>D. Fringe benefit rates (benefits / S&amp;W) observed where audited statements report both lines</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="5" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="5" t="inlineStr">
         <is>
           <t>Institution</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B34" s="5" t="inlineStr">
         <is>
           <t>S&amp;W ($)</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>Benefits ($)</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>Fringe rate</t>
         </is>
-      </c>
-    </row>
-    <row r="34">
-      <c r="A34" s="9" t="inlineStr">
-        <is>
-          <t>Rice</t>
-        </is>
-      </c>
-      <c r="B34" s="19">
-        <f>S3_FY25!C5</f>
-        <v/>
-      </c>
-      <c r="C34" s="19">
-        <f>S3_FY25!E5-S3_FY25!C5</f>
-        <v/>
-      </c>
-      <c r="D34" s="20">
-        <f>C34/B34</f>
-        <v/>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="9" t="inlineStr">
         <is>
-          <t>Princeton</t>
+          <t>Rice</t>
         </is>
       </c>
       <c r="B35" s="19">
-        <f>S3_FY25!C8</f>
+        <f>S3_FY25!C5</f>
         <v/>
       </c>
       <c r="C35" s="19">
-        <f>S3_FY25!E8-S3_FY25!C8</f>
+        <f>S3_FY25!E5-S3_FY25!C5</f>
         <v/>
       </c>
       <c r="D35" s="20">
@@ -70835,15 +70891,15 @@
     <row r="36">
       <c r="A36" s="9" t="inlineStr">
         <is>
-          <t>Yale</t>
+          <t>Princeton</t>
         </is>
       </c>
       <c r="B36" s="19">
-        <f>S3_FY25!C10</f>
+        <f>S3_FY25!C8</f>
         <v/>
       </c>
       <c r="C36" s="19">
-        <f>S3_FY25!E10-S3_FY25!C10</f>
+        <f>S3_FY25!E8-S3_FY25!C8</f>
         <v/>
       </c>
       <c r="D36" s="20">
@@ -70854,15 +70910,15 @@
     <row r="37">
       <c r="A37" s="9" t="inlineStr">
         <is>
-          <t>Chicago</t>
+          <t>Harvard</t>
         </is>
       </c>
       <c r="B37" s="19">
-        <f>S3_FY25!C11</f>
+        <f>S3_FY25!C9</f>
         <v/>
       </c>
       <c r="C37" s="19">
-        <f>S3_FY25!E11-S3_FY25!C11</f>
+        <f>S3_FY25!E9-S3_FY25!C9</f>
         <v/>
       </c>
       <c r="D37" s="20">
@@ -70873,15 +70929,15 @@
     <row r="38">
       <c r="A38" s="9" t="inlineStr">
         <is>
-          <t>Duke</t>
+          <t>Yale</t>
         </is>
       </c>
       <c r="B38" s="19">
-        <f>S3_FY25!C12</f>
+        <f>S3_FY25!C10</f>
         <v/>
       </c>
       <c r="C38" s="19">
-        <f>S3_FY25!E12-S3_FY25!C12</f>
+        <f>S3_FY25!E10-S3_FY25!C10</f>
         <v/>
       </c>
       <c r="D38" s="20">
@@ -70892,15 +70948,15 @@
     <row r="39">
       <c r="A39" s="9" t="inlineStr">
         <is>
-          <t>Emory</t>
+          <t>Chicago</t>
         </is>
       </c>
       <c r="B39" s="19">
-        <f>S3_FY25!C13</f>
+        <f>S3_FY25!C11</f>
         <v/>
       </c>
       <c r="C39" s="19">
-        <f>S3_FY25!E13-S3_FY25!C13</f>
+        <f>S3_FY25!E11-S3_FY25!C11</f>
         <v/>
       </c>
       <c r="D39" s="20">
@@ -70911,15 +70967,15 @@
     <row r="40">
       <c r="A40" s="9" t="inlineStr">
         <is>
-          <t>Boston University</t>
+          <t>Duke</t>
         </is>
       </c>
       <c r="B40" s="19">
-        <f>S3_FY25!C17</f>
+        <f>S3_FY25!C12</f>
         <v/>
       </c>
       <c r="C40" s="19">
-        <f>S3_FY25!E17-S3_FY25!C17</f>
+        <f>S3_FY25!E12-S3_FY25!C12</f>
         <v/>
       </c>
       <c r="D40" s="20">
@@ -70930,15 +70986,15 @@
     <row r="41">
       <c r="A41" s="9" t="inlineStr">
         <is>
-          <t>MIT</t>
+          <t>Emory</t>
         </is>
       </c>
       <c r="B41" s="19">
-        <f>S3_FY25!C18</f>
+        <f>S3_FY25!C13</f>
         <v/>
       </c>
       <c r="C41" s="19">
-        <f>S3_FY25!E18-S3_FY25!C18</f>
+        <f>S3_FY25!E13-S3_FY25!C13</f>
         <v/>
       </c>
       <c r="D41" s="20">
@@ -70947,28 +71003,176 @@
       </c>
     </row>
     <row r="42">
-      <c r="A42" s="3" t="inlineStr">
+      <c r="A42" s="9" t="inlineStr">
+        <is>
+          <t>Boston University</t>
+        </is>
+      </c>
+      <c r="B42" s="19">
+        <f>S3_FY25!C17</f>
+        <v/>
+      </c>
+      <c r="C42" s="19">
+        <f>S3_FY25!E17-S3_FY25!C17</f>
+        <v/>
+      </c>
+      <c r="D42" s="20">
+        <f>C42/B42</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="9" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="B43" s="19">
+        <f>S3_FY25!C18</f>
+        <v/>
+      </c>
+      <c r="C43" s="19">
+        <f>S3_FY25!E18-S3_FY25!C18</f>
+        <v/>
+      </c>
+      <c r="D43" s="20">
+        <f>C43/B43</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="3" t="inlineStr">
         <is>
           <t>Minimum / median / maximum</t>
         </is>
       </c>
-      <c r="B42" s="23">
-        <f>MIN(D34:D41)</f>
-        <v/>
-      </c>
-      <c r="C42" s="23">
-        <f>MEDIAN(D34:D41)</f>
-        <v/>
-      </c>
-      <c r="D42" s="23">
-        <f>MAX(D34:D41)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="43">
-      <c r="A43" s="17" t="inlineStr">
+      <c r="B44" s="23">
+        <f>MIN(D35:D43)</f>
+        <v/>
+      </c>
+      <c r="C44" s="23">
+        <f>MEDIAN(D35:D43)</f>
+        <v/>
+      </c>
+      <c r="D44" s="23">
+        <f>MAX(D35:D43)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="17" t="inlineStr">
         <is>
           <t>The 35% assumption sits above every observed rate, so the Penn and Stanford estimates lean low relative to peers (Alt 1 gives higher S&amp;W per student).</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="3" t="inlineStr">
+        <is>
+          <t>E. Harvard S&amp;W per student by student-count basis (CDS excludes the Harvard Extension School; expenses include it)</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>Basis</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>Students</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>S&amp;W per student</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>Core opex per student</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="9" t="inlineStr">
+        <is>
+          <t>Common Data Set 2024-25 (used on slide)</t>
+        </is>
+      </c>
+      <c r="B49" s="19" t="n">
+        <v>21189</v>
+      </c>
+      <c r="C49" s="11">
+        <f>S3_FY25!C9/B49</f>
+        <v/>
+      </c>
+      <c r="D49" s="11">
+        <f>S3_FY25!L9/B49</f>
+        <v/>
+      </c>
+      <c r="E49" s="9" t="inlineStr">
+        <is>
+          <t>B1 grand total all students, degree schools only; matches the FY25 report's own 'approximately 7,000 undergraduate and 14,000 graduate students'</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="9" t="inlineStr">
+        <is>
+          <t>Harvard OIRA Fact Book fall 2023 degree students incl. Extension</t>
+        </is>
+      </c>
+      <c r="B50" s="19" t="n">
+        <v>24596</v>
+      </c>
+      <c r="C50" s="11">
+        <f>S3_FY25!C9/B50</f>
+        <v/>
+      </c>
+      <c r="D50" s="11">
+        <f>S3_FY25!L9/B50</f>
+        <v/>
+      </c>
+      <c r="E50" s="9" t="inlineStr">
+        <is>
+          <t>Fact Book 2023-24 enrollment page: 24,596 degree students (includes 3,595 Extension degree candidates); fall 2024 not used because not opened</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="9" t="inlineStr">
+        <is>
+          <t>IPEDS fall 2023 total</t>
+        </is>
+      </c>
+      <c r="B51" s="19" t="n">
+        <v>30386</v>
+      </c>
+      <c r="C51" s="11">
+        <f>S3_FY25!C9/B51</f>
+        <v/>
+      </c>
+      <c r="D51" s="11">
+        <f>S3_FY25!L9/B51</f>
+        <v/>
+      </c>
+      <c r="E51" s="9" t="inlineStr">
+        <is>
+          <t>Includes non-degree and Extension students; broadest count</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="17" t="inlineStr">
+        <is>
+          <t>Harvard stays well above Northeastern ($26K) on every basis.</t>
         </is>
       </c>
     </row>
@@ -71286,7 +71490,7 @@
       </c>
       <c r="D9" s="22" t="inlineStr">
         <is>
-          <t>Harvard FY23 report not reached</t>
+          <t>FY23 not in the FY25 report (FY24 comparative: S&amp;W 2,631,642,000)</t>
         </is>
       </c>
       <c r="M9" s="19" t="n">
@@ -72656,15 +72860,17 @@
           <t>Salaries and wages</t>
         </is>
       </c>
-      <c r="C21" s="19" t="n"/>
+      <c r="C21" s="19" t="n">
+        <v>2758560000</v>
+      </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>NOT EXTRACTED: the Harvard Financial Report PDFs could not be retrieved (finance.harvard.edu returns Akamai 'Access Denied' 403 to curl with a browser User-Agent, and WebFetch reports the host blocked by the network egress proxy). No number was taken from a search snippet or memory.</t>
+          <t>'Salaries and wages 2,758,560' (Consolidated Statements of Changes in Net Assets with General Operating Account Detail, operating expenses; $ thousands; columns: without donor restrictions, with donor restrictions, 2025 total, 2024 total). Statement of changes in net assets, PDF p.18 (printed p.17). Same figure in Note 17 natural classification, PDF p.43 (printed p.42).</t>
         </is>
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>FY25 Harvard University Financial Report (located, NOT retrieved: 403): https://finance.harvard.edu/sites/g/files/omnuum12671/files/2025-10/fy25-financial-report.pdf; FY25 Financial Overview from the VP for Finance and the Treasurer (located, NOT retrieved: 403): https://finance.harvard.edu/sites/g/files/omnuum12671/files/2025-10/fy25-financial-overview.pdf</t>
+          <t>Harvard University Financial Report, Fiscal Year 2025 (audited consolidated financial statements with unqualified opinion; supplied by Brett Sweet, file fy25-financial-report.pdf, 46 pages): https://finance.harvard.edu/sites/g/files/omnuum12671/files/2025-10/fy25-financial-report.pdf</t>
         </is>
       </c>
     </row>
@@ -72679,15 +72885,17 @@
           <t>Total operating expenses</t>
         </is>
       </c>
-      <c r="C22" s="19" t="n"/>
+      <c r="C22" s="19" t="n">
+        <v>6794371000</v>
+      </c>
       <c r="D22" s="4" t="inlineStr">
         <is>
-          <t>NOT EXTRACTED: the Harvard Financial Report PDFs could not be retrieved (finance.harvard.edu returns Akamai 'Access Denied' 403 to curl with a browser User-Agent, and WebFetch reports the host blocked by the network egress proxy). No number was taken from a search snippet or memory.</t>
+          <t>'TOTAL OPERATING EXPENSES 6,794,371' (Statement of changes in net assets, PDF p.18 (printed p.17)). The nine natural-classification lines (salaries and wages, employee benefits, services purchased, depreciation, space and occupancy, supplies and equipment, interest, scholarships and other student awards, other expenses) sum to 6,794,371; Note 17 total also 6,794,371 (PDF p.43 (printed p.42)).</t>
         </is>
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>FY25 Harvard University Financial Report (located, NOT retrieved: 403): https://finance.harvard.edu/sites/g/files/omnuum12671/files/2025-10/fy25-financial-report.pdf; FY25 Financial Overview from the VP for Finance and the Treasurer (located, NOT retrieved: 403): https://finance.harvard.edu/sites/g/files/omnuum12671/files/2025-10/fy25-financial-overview.pdf</t>
+          <t>Harvard University Financial Report, Fiscal Year 2025 (audited consolidated financial statements with unqualified opinion; supplied by Brett Sweet, file fy25-financial-report.pdf, 46 pages): https://finance.harvard.edu/sites/g/files/omnuum12671/files/2025-10/fy25-financial-report.pdf</t>
         </is>
       </c>
     </row>
@@ -72702,15 +72910,17 @@
           <t>Depreciation</t>
         </is>
       </c>
-      <c r="C23" s="19" t="n"/>
+      <c r="C23" s="19" t="n">
+        <v>459031000</v>
+      </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>NOT EXTRACTED: the Harvard Financial Report PDFs could not be retrieved (finance.harvard.edu returns Akamai 'Access Denied' 403 to curl with a browser User-Agent, and WebFetch reports the host blocked by the network egress proxy). No number was taken from a search snippet or memory.</t>
+          <t>'Depreciation (Note 7) 459,031' (Statement of changes in net assets, PDF p.18 (printed p.17)); Note 17: 'Depreciation ... 459,031'.</t>
         </is>
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>FY25 Harvard University Financial Report (located, NOT retrieved: 403): https://finance.harvard.edu/sites/g/files/omnuum12671/files/2025-10/fy25-financial-report.pdf; FY25 Financial Overview from the VP for Finance and the Treasurer (located, NOT retrieved: 403): https://finance.harvard.edu/sites/g/files/omnuum12671/files/2025-10/fy25-financial-overview.pdf</t>
+          <t>Harvard University Financial Report, Fiscal Year 2025 (audited consolidated financial statements with unqualified opinion; supplied by Brett Sweet, file fy25-financial-report.pdf, 46 pages): https://finance.harvard.edu/sites/g/files/omnuum12671/files/2025-10/fy25-financial-report.pdf</t>
         </is>
       </c>
     </row>
@@ -72725,15 +72935,17 @@
           <t>Interest</t>
         </is>
       </c>
-      <c r="C24" s="19" t="n"/>
+      <c r="C24" s="19" t="n">
+        <v>262546000</v>
+      </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>NOT EXTRACTED: the Harvard Financial Report PDFs could not be retrieved (finance.harvard.edu returns Akamai 'Access Denied' 403 to curl with a browser User-Agent, and WebFetch reports the host blocked by the network egress proxy). No number was taken from a search snippet or memory.</t>
+          <t>'Interest (Note 10) 262,546' (Statement of changes in net assets, PDF p.18 (printed p.17)); Note 17: 'Interest ... 262,546'.</t>
         </is>
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>FY25 Harvard University Financial Report (located, NOT retrieved: 403): https://finance.harvard.edu/sites/g/files/omnuum12671/files/2025-10/fy25-financial-report.pdf; FY25 Financial Overview from the VP for Finance and the Treasurer (located, NOT retrieved: 403): https://finance.harvard.edu/sites/g/files/omnuum12671/files/2025-10/fy25-financial-overview.pdf</t>
+          <t>Harvard University Financial Report, Fiscal Year 2025 (audited consolidated financial statements with unqualified opinion; supplied by Brett Sweet, file fy25-financial-report.pdf, 46 pages): https://finance.harvard.edu/sites/g/files/omnuum12671/files/2025-10/fy25-financial-report.pdf</t>
         </is>
       </c>
     </row>
@@ -73645,7 +73857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E28"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -74080,7 +74292,7 @@
       </c>
       <c r="D19" s="4" t="inlineStr">
         <is>
-          <t>Schools that report both lines have fringe rates (benefits / S&amp;W) of 22.8% to 33.8% (Chicago 22.8%, Duke 23.6%, Emory 23.9%, Rice 23.9%, Princeton 30.3%, BU 31.5%, Yale 31.5%, MIT 33.8%). 35% is above all of them, so the Penn and Stanford estimates lean low: using each school's own Form 990 S&amp;W share instead would raise S&amp;W per student by about 4% (Penn) and 8% (Stanford) (S3_Sensitivity C). Neither changes the ranking of Penn or Stanford or any conclusion about Northeastern.</t>
+          <t>Schools that report both lines have fringe rates (benefits / S&amp;W) of 22.8% to 33.8% (Chicago 22.8%, Duke 23.6%, Emory 23.9%, Rice 23.9%, Harvard 27.4%, Princeton 30.3%, BU 31.5%, Yale 31.5%, MIT 33.8%). 35% is above all of them, so the Penn and Stanford estimates lean low: using each school's own Form 990 S&amp;W share instead would raise S&amp;W per student by about 4% (Penn) and 8% (Stanford) (S3_Sensitivity C). Neither changes the ranking of Penn or Stanford or any conclusion about Northeastern.</t>
         </is>
       </c>
       <c r="E19" s="27" t="inlineStr">
@@ -74280,12 +74492,12 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>The FY25 Financial Report could not be reached (finance.harvard.edu denies automated access). Harvard is not on the FY25 chart; CDS fall 2024 enrollment (21,189) is recorded.</t>
-        </is>
-      </c>
-      <c r="E27" s="28" t="inlineStr">
-        <is>
-          <t>Open</t>
+          <t>Added from the FY25 audited Financial Report supplied by Northeastern (finance.harvard.edu blocks automated access). S&amp;W $2,758.6M and benefits $755.9M are separate lines (benefits 27.4% of S&amp;W); total operating expenses $6,794.4M - depreciation $459.0M - interest $262.5M = core $6,072.8M; the nine natural-classification lines sum to the total in FY25 and FY24 (Note 17). S&amp;W share 45.4%; 21,189 students -&gt; $130K S&amp;W per student, next to Princeton ($128K) with a lower S&amp;W share. No hospital consolidated.</t>
+        </is>
+      </c>
+      <c r="E27" s="27" t="inlineStr">
+        <is>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -74300,15 +74512,65 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
+          <t>Harvard student count</t>
+        </is>
+      </c>
+      <c r="D28" s="4" t="inlineStr">
+        <is>
+          <t>CDS (21,189) matches the FY25 report's own 'approximately 7,000 undergraduate and 14,000 graduate students' but excludes the Harvard Extension School, whose costs are in the expenses (Division of Continuing Education). With Extension degree students (24,596 in fall 2023) S&amp;W per student would be about $112K; with IPEDS 30,386, $91K (S3_Sensitivity E). No effect on Northeastern's ranking.</t>
+        </is>
+      </c>
+      <c r="E28" s="27" t="inlineStr">
+        <is>
+          <t>Caveat</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="B29" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C29" s="4" t="inlineStr">
+        <is>
+          <t>Harvard FY23 calibration</t>
+        </is>
+      </c>
+      <c r="D29" s="4" t="inlineStr">
+        <is>
+          <t>FY23 statements not supplied, so Harvard is not on S3_FY23_Recalc. Sanity check only: FY24 core opex on the stated definition ($5,760M) is 2.6% below the original slide's FY23 'core opex' ($5,912M), consistent with the original using total operating expenses.</t>
+        </is>
+      </c>
+      <c r="E29" s="27" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="B30" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C30" s="4" t="inlineStr">
+        <is>
           <t>Original chart construction</t>
         </is>
       </c>
-      <c r="D28" s="4" t="inlineStr">
+      <c r="D30" s="4" t="inlineStr">
         <is>
           <t>The original plotted only the eight iso-lines; logos were hand-placed pictures, so positions did not come from data, and Stanford's x-value exceeded the axis maximum. Rebuilt with real data points.</t>
         </is>
       </c>
-      <c r="E28" s="27" t="inlineStr">
+      <c r="E30" s="27" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>

</xml_diff>

<commit_message>
Harvard: add Extension School students (24,819) and FY23 from the uploaded report
Students = CDS fall 2024 (21,189) + Extension School degree students (3,630, Harvard OIRA Fact Book) because expenses include Continuing Education: $111K S&W per student.
FY23 audited figures tie to the original slide's S&W to the dollar; its 'core' equals total operating expenses (12.0% too high vs the stated definition).
Slide 3 label placement hint for Harvard; render check re-done.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCNX7EgSWHMHv9UtVBoXog
</commit_message>
<xml_diff>
--- a/nu-peer-slides/NU_peer_slides_backup.xlsx
+++ b/nu-peer-slides/NU_peer_slides_backup.xlsx
@@ -601,7 +601,7 @@
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>What is still open (optional: Penn / Stanford consolidated salaries and wages; Princeton CDS; Harvard FY23 report for calibration).</t>
+          <t>What is still open (optional: Penn / Stanford consolidated salaries and wages; Princeton CDS).</t>
         </is>
       </c>
     </row>
@@ -616,7 +616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -662,17 +662,17 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>Harvard FY23 Financial Report (optional)</t>
+          <t>Penn and Stanford salaries and wages (optional)</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>Only needed to add Harvard to the FY23 recalculation sheet; the FY25 chart does not depend on it.</t>
+          <t>Estimated at combined salaries+benefits / 1.35 (35% fringe rate, per Northeastern). Audited statements combine the two lines; Form 990s cover a narrower scope.</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>Upload the FY23 or FY24 Harvard Financial Report if you want the calibration row.</t>
+          <t>If either finance office can supply consolidated S&amp;W, replace the grey estimate.</t>
         </is>
       </c>
     </row>
@@ -684,17 +684,17 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>Penn and Stanford salaries and wages (optional)</t>
+          <t>Princeton Common Data Set 2024-25 (optional)</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>Estimated at combined salaries+benefits / 1.35 (35% fringe rate, per Northeastern). Audited statements combine the two lines; Form 990s cover a narrower scope.</t>
+          <t>ir.princeton.edu is behind a bot challenge; the Treasurer's report count (9,050) is used.</t>
         </is>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
-          <t>If either finance office can supply consolidated S&amp;W, replace the grey estimate.</t>
+          <t>Upload the CDS PDF if you want the same instrument as the other schools.</t>
         </is>
       </c>
     </row>
@@ -706,37 +706,15 @@
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>Princeton Common Data Set 2024-25 (optional)</t>
+          <t>IPEDS fall 2024 enrollment and FY24 finance files</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>ir.princeton.edu is behind a bot challenge; the Treasurer's report count (9,050) is used.</t>
+          <t>Not yet posted on the IPEDS data center.</t>
         </is>
       </c>
       <c r="D6" s="4" t="inlineStr">
-        <is>
-          <t>Upload the CDS PDF if you want the same instrument as the other schools.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>IPEDS fall 2024 enrollment and FY24 finance files</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>Not yet posted on the IPEDS data center.</t>
-        </is>
-      </c>
-      <c r="D7" s="4" t="inlineStr">
         <is>
           <t>Re-check when posted.</t>
         </is>
@@ -69358,7 +69336,7 @@
         <v/>
       </c>
       <c r="M9" s="19" t="n">
-        <v>21189</v>
+        <v>24819</v>
       </c>
       <c r="N9" s="11">
         <f>C9/M9</f>
@@ -69383,7 +69361,7 @@
       </c>
       <c r="S9" s="4" t="inlineStr">
         <is>
-          <t>Separate S&amp;W and benefits lines in the FY25 audited Financial Report (supplied by Northeastern; Statement of Changes in Net Assets, PDF p.18). Depreciation and interest are separate operating lines; nine natural-classification lines sum to total operating expenses. No hospital consolidated. CDS students exclude the Harvard Extension School although expenses include it (S3_Sensitivity E).</t>
+          <t>Separate S&amp;W and benefits lines in the FY25 audited Financial Report (supplied by Northeastern; Statement of Changes in Net Assets, PDF p.18). Depreciation and interest are separate operating lines; nine natural-classification lines sum to total operating expenses. No hospital consolidated. Students = CDS 21,189 + Extension School degree students 3,630 (Fact Book, fall 2024) = 24,819, because expenses include the Division of Continuing Education (S3_Sensitivity E).</t>
         </is>
       </c>
     </row>
@@ -70045,7 +70023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J52"/>
+  <dimension ref="A1:J53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -70187,7 +70165,7 @@
       </c>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>CDS fall 2024</t>
+          <t>Students used (CDS fall 2024; Harvard + Extension)</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
@@ -70197,7 +70175,7 @@
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>S&amp;W per student (CDS)</t>
+          <t>S&amp;W per student (used)</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -71069,7 +71047,7 @@
     <row r="47">
       <c r="A47" s="3" t="inlineStr">
         <is>
-          <t>E. Harvard S&amp;W per student by student-count basis (CDS excludes the Harvard Extension School; expenses include it)</t>
+          <t>E. Harvard S&amp;W per student by student-count basis (CDS excludes the Harvard Extension School; the expenses include it)</t>
         </is>
       </c>
     </row>
@@ -71103,11 +71081,12 @@
     <row r="49">
       <c r="A49" s="9" t="inlineStr">
         <is>
-          <t>Common Data Set 2024-25 (used on slide)</t>
-        </is>
-      </c>
-      <c r="B49" s="19" t="n">
-        <v>21189</v>
+          <t>CDS 2024-25 + Extension School degree students, fall 2024 (USED on slide)</t>
+        </is>
+      </c>
+      <c r="B49" s="19">
+        <f>21189+3630</f>
+        <v/>
       </c>
       <c r="C49" s="11">
         <f>S3_FY25!C9/B49</f>
@@ -71119,18 +71098,18 @@
       </c>
       <c r="E49" s="9" t="inlineStr">
         <is>
-          <t>B1 grand total all students, degree schools only; matches the FY25 report's own 'approximately 7,000 undergraduate and 14,000 graduate students'</t>
+          <t>CDS B1 grand total 21,189 (degree schools only) + Extension undergraduate 621 + graduate 3,009 (Harvard OIRA Fact Book 2025-26, 'as of October 15 of the academic year')</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="9" t="inlineStr">
         <is>
-          <t>Harvard OIRA Fact Book fall 2023 degree students incl. Extension</t>
+          <t>Fact Book University total degree headcount, fall 2024</t>
         </is>
       </c>
       <c r="B50" s="19" t="n">
-        <v>24596</v>
+        <v>24519</v>
       </c>
       <c r="C50" s="11">
         <f>S3_FY25!C9/B50</f>
@@ -71142,18 +71121,18 @@
       </c>
       <c r="E50" s="9" t="inlineStr">
         <is>
-          <t>Fact Book 2023-24 enrollment page: 24,596 degree students (includes 3,595 Extension degree candidates); fall 2024 not used because not opened</t>
+          <t>Distinct students; some Extension students are also registered in another school, so this is 300 below the sum above</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="9" t="inlineStr">
         <is>
-          <t>IPEDS fall 2023 total</t>
+          <t>CDS 2024-25 only (excludes Extension School)</t>
         </is>
       </c>
       <c r="B51" s="19" t="n">
-        <v>30386</v>
+        <v>21189</v>
       </c>
       <c r="C51" s="11">
         <f>S3_FY25!C9/B51</f>
@@ -71165,12 +71144,35 @@
       </c>
       <c r="E51" s="9" t="inlineStr">
         <is>
-          <t>Includes non-degree and Extension students; broadest count</t>
+          <t>The count used in the first FY25 draft; expenses include Continuing Education, so S&amp;W per student is overstated on this basis</t>
         </is>
       </c>
     </row>
     <row r="52">
-      <c r="A52" s="17" t="inlineStr">
+      <c r="A52" s="9" t="inlineStr">
+        <is>
+          <t>IPEDS fall 2023 total</t>
+        </is>
+      </c>
+      <c r="B52" s="19" t="n">
+        <v>30386</v>
+      </c>
+      <c r="C52" s="11">
+        <f>S3_FY25!C9/B52</f>
+        <v/>
+      </c>
+      <c r="D52" s="11">
+        <f>S3_FY25!L9/B52</f>
+        <v/>
+      </c>
+      <c r="E52" s="9" t="inlineStr">
+        <is>
+          <t>Adds non-degree Extension course takers (not in the Fact Book); fall 2024 IPEDS not yet posted</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="17" t="inlineStr">
         <is>
           <t>Harvard stays well above Northeastern ($26K) on every basis.</t>
         </is>
@@ -71488,10 +71490,30 @@
       <c r="C9" s="19" t="n">
         <v>5911797000</v>
       </c>
-      <c r="D9" s="22" t="inlineStr">
-        <is>
-          <t>FY23 not in the FY25 report (FY24 comparative: S&amp;W 2,631,642,000)</t>
-        </is>
+      <c r="D9" s="19" t="n">
+        <v>2421076000</v>
+      </c>
+      <c r="E9" s="19" t="n">
+        <v>5911797000</v>
+      </c>
+      <c r="F9" s="19" t="n">
+        <v>633399000</v>
+      </c>
+      <c r="G9" s="19">
+        <f>E9-F9</f>
+        <v/>
+      </c>
+      <c r="H9" s="25">
+        <f>(C9/E9-1)*100</f>
+        <v/>
+      </c>
+      <c r="I9" s="25">
+        <f>(C9/G9-1)*100</f>
+        <v/>
+      </c>
+      <c r="J9" s="25">
+        <f>(B9/D9-1)*100</f>
+        <v/>
       </c>
       <c r="M9" s="19" t="n">
         <v>5911797000</v>
@@ -72385,7 +72407,7 @@
     <row r="20">
       <c r="A20" s="17" t="inlineStr">
         <is>
-          <t>Reading it: Harvard (CDS excludes Extension School), Penn (CDS counts degree-seeking traditional programs only), Chicago (CDS ~12-14% below IPEDS) and Northeastern (CDS ~24% ABOVE IPEDS) do not match IPEDS; the original slide mixed fall 2021 (Rice), fall 2022 (Vanderbilt), degree-seeking counts (Harvard, Penn) and round estimates (Emory 16,000, Northwestern 23,000).</t>
+          <t>Reading it: Harvard (CDS excludes Extension School; the slide adds it back), Penn (CDS counts degree-seeking traditional programs only), Chicago (CDS ~12-14% below IPEDS) and Northeastern (CDS ~24% ABOVE IPEDS) do not match IPEDS; the original slide mixed fall 2021 (Rice), fall 2022 (Vanderbilt), degree-seeking counts (Harvard, Penn) and round estimates (Emory 16,000, Northwestern 23,000).</t>
         </is>
       </c>
     </row>
@@ -72870,7 +72892,7 @@
       </c>
       <c r="E21" s="4" t="inlineStr">
         <is>
-          <t>Harvard University Financial Report, Fiscal Year 2025 (audited consolidated financial statements with unqualified opinion; supplied by Brett Sweet, file fy25-financial-report.pdf, 46 pages): https://finance.harvard.edu/sites/g/files/omnuum12671/files/2025-10/fy25-financial-report.pdf</t>
+          <t>Harvard University Financial Report, Fiscal Year 2025 (audited consolidated financial statements with unqualified opinion; supplied by Brett Sweet, file fy25-financial-report.pdf, 46 pages): https://finance.harvard.edu/sites/g/files/omnuum12671/files/2025-10/fy25-financial-report.pdf; Harvard University Financial Report, Fiscal Year 2023 (audited consolidated financial statements; supplied by Brett Sweet, file fy23_harvard_financial_report.pdf, 47 pages): https://finance.harvard.edu/ (Financial Reports; FY23 report)</t>
         </is>
       </c>
     </row>
@@ -72895,7 +72917,7 @@
       </c>
       <c r="E22" s="4" t="inlineStr">
         <is>
-          <t>Harvard University Financial Report, Fiscal Year 2025 (audited consolidated financial statements with unqualified opinion; supplied by Brett Sweet, file fy25-financial-report.pdf, 46 pages): https://finance.harvard.edu/sites/g/files/omnuum12671/files/2025-10/fy25-financial-report.pdf</t>
+          <t>Harvard University Financial Report, Fiscal Year 2025 (audited consolidated financial statements with unqualified opinion; supplied by Brett Sweet, file fy25-financial-report.pdf, 46 pages): https://finance.harvard.edu/sites/g/files/omnuum12671/files/2025-10/fy25-financial-report.pdf; Harvard University Financial Report, Fiscal Year 2023 (audited consolidated financial statements; supplied by Brett Sweet, file fy23_harvard_financial_report.pdf, 47 pages): https://finance.harvard.edu/ (Financial Reports; FY23 report)</t>
         </is>
       </c>
     </row>
@@ -72920,7 +72942,7 @@
       </c>
       <c r="E23" s="4" t="inlineStr">
         <is>
-          <t>Harvard University Financial Report, Fiscal Year 2025 (audited consolidated financial statements with unqualified opinion; supplied by Brett Sweet, file fy25-financial-report.pdf, 46 pages): https://finance.harvard.edu/sites/g/files/omnuum12671/files/2025-10/fy25-financial-report.pdf</t>
+          <t>Harvard University Financial Report, Fiscal Year 2025 (audited consolidated financial statements with unqualified opinion; supplied by Brett Sweet, file fy25-financial-report.pdf, 46 pages): https://finance.harvard.edu/sites/g/files/omnuum12671/files/2025-10/fy25-financial-report.pdf; Harvard University Financial Report, Fiscal Year 2023 (audited consolidated financial statements; supplied by Brett Sweet, file fy23_harvard_financial_report.pdf, 47 pages): https://finance.harvard.edu/ (Financial Reports; FY23 report)</t>
         </is>
       </c>
     </row>
@@ -72945,7 +72967,7 @@
       </c>
       <c r="E24" s="4" t="inlineStr">
         <is>
-          <t>Harvard University Financial Report, Fiscal Year 2025 (audited consolidated financial statements with unqualified opinion; supplied by Brett Sweet, file fy25-financial-report.pdf, 46 pages): https://finance.harvard.edu/sites/g/files/omnuum12671/files/2025-10/fy25-financial-report.pdf</t>
+          <t>Harvard University Financial Report, Fiscal Year 2025 (audited consolidated financial statements with unqualified opinion; supplied by Brett Sweet, file fy25-financial-report.pdf, 46 pages): https://finance.harvard.edu/sites/g/files/omnuum12671/files/2025-10/fy25-financial-report.pdf; Harvard University Financial Report, Fiscal Year 2023 (audited consolidated financial statements; supplied by Brett Sweet, file fy23_harvard_financial_report.pdf, 47 pages): https://finance.harvard.edu/ (Financial Reports; FY23 report)</t>
         </is>
       </c>
     </row>
@@ -74217,7 +74239,7 @@
       </c>
       <c r="D16" s="4" t="inlineStr">
         <is>
-          <t>The original values equal audited total operating expenses to the dollar for every school checked (Rice, Vanderbilt, Northwestern, Princeton, Yale, Chicago, Duke, Emory, Penn, Stanford), and equal the IPEDS FY23 'total expenses' field for Rice, Vanderbilt, Northwestern, Princeton, Harvard, Duke and Penn. Depreciation, amortization and interest were never removed although the axis says they were. FY25 now follows the axis; FY23 restated is 5-15% lower (S3_FY23_Recalc).</t>
+          <t>The original values equal audited total operating expenses to the dollar for every school checked (Rice, Vanderbilt, Northwestern, Princeton, Harvard, Yale, Chicago, Duke, Emory, Penn, Stanford), and equal the IPEDS FY23 'total expenses' field for Rice, Vanderbilt, Northwestern, Princeton, Harvard, Duke and Penn. Depreciation, amortization and interest were never removed although the axis says they were. FY25 now follows the axis; FY23 restated is 5-15% lower (S3_FY23_Recalc).</t>
         </is>
       </c>
       <c r="E16" s="28" t="inlineStr">
@@ -74492,7 +74514,7 @@
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Added from the FY25 audited Financial Report supplied by Northeastern (finance.harvard.edu blocks automated access). S&amp;W $2,758.6M and benefits $755.9M are separate lines (benefits 27.4% of S&amp;W); total operating expenses $6,794.4M - depreciation $459.0M - interest $262.5M = core $6,072.8M; the nine natural-classification lines sum to the total in FY25 and FY24 (Note 17). S&amp;W share 45.4%; 21,189 students -&gt; $130K S&amp;W per student, next to Princeton ($128K) with a lower S&amp;W share. No hospital consolidated.</t>
+          <t>Added from the FY25 audited Financial Report supplied by Northeastern (finance.harvard.edu blocks automated access). S&amp;W $2,758.6M and benefits $755.9M are separate lines (benefits 27.4% of S&amp;W); total operating expenses $6,794.4M - depreciation $459.0M - interest $262.5M = core $6,072.8M; the nine natural-classification lines sum to the total in FY25 and FY24 (Note 17). S&amp;W share 45.4%; 24,819 students (CDS + Extension School degree students) -&gt; $111K S&amp;W per student, below Princeton ($128K) with a lower S&amp;W share. No hospital consolidated.</t>
         </is>
       </c>
       <c r="E27" s="27" t="inlineStr">
@@ -74517,12 +74539,12 @@
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>CDS (21,189) matches the FY25 report's own 'approximately 7,000 undergraduate and 14,000 graduate students' but excludes the Harvard Extension School, whose costs are in the expenses (Division of Continuing Education). With Extension degree students (24,596 in fall 2023) S&amp;W per student would be about $112K; with IPEDS 30,386, $91K (S3_Sensitivity E). No effect on Northeastern's ranking.</t>
+          <t>Expenses include the Division of Continuing Education (Harvard Extension School) but the Common Data Set excludes it. Students on the slide = CDS 21,189 + Extension degree students 3,630 (621 undergraduate + 3,009 graduate, Harvard OIRA Fact Book 2025-26, fall 2024) = 24,819 -&gt; $111K S&amp;W per student. Alternatives (S3_Sensitivity E): CDS only 21,189 -&gt; $130K; Fact Book distinct total 24,519 -&gt; $113K; IPEDS fall 2023 30,386 (adds non-degree course takers) -&gt; $91K. Harvard's own report: 'approximately 7,000 undergraduate and 14,000 graduate students' (Note 1). No effect on Northeastern's ranking.</t>
         </is>
       </c>
       <c r="E28" s="27" t="inlineStr">
         <is>
-          <t>Caveat</t>
+          <t>Handled / caveat</t>
         </is>
       </c>
     </row>
@@ -74542,12 +74564,12 @@
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>FY23 statements not supplied, so Harvard is not on S3_FY23_Recalc. Sanity check only: FY24 core opex on the stated definition ($5,760M) is 2.6% below the original slide's FY23 'core opex' ($5,912M), consistent with the original using total operating expenses.</t>
+          <t>FY23 Financial Report (supplied by Northeastern): original slide S&amp;W $2,421,076K equals the audited FY23 salaries and wages line to the dollar; the original 'core opex' $5,911,797K equals audited FY23 total operating expenses to the dollar. On the stated definition FY23 core is $5,278,398K (total less depreciation $424,809K and interest $208,590K), so the original x value was 12.0% too high. Same finding as for the other schools. Original 21,400 students = the report's 'approximately 7,200 undergraduate and 14,200 graduate' (Note 1). S&amp;W grew 13.9% FY23 to FY25 ($2,421M to $2,759M).</t>
         </is>
       </c>
       <c r="E29" s="27" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Pass / finding</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Slide 3: y axis 20-70%, larger markers, health-system schools in blue; slide 1: royal-blue private markers, smaller public markers with hairline border
Slide 3: iso-lines drawn to the plot edges and labelled along the top; Chicago, Duke, Emory royal blue, Penn and Stanford (estimated S&W) lighter blue, with a legend row.
Slide 1: private markers royal blue, public markers one size smaller with a 0.25 pt black outline.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCNX7EgSWHMHv9UtVBoXog
</commit_message>
<xml_diff>
--- a/nu-peer-slides/NU_peer_slides_backup.xlsx
+++ b/nu-peer-slides/NU_peer_slides_backup.xlsx
@@ -672,7 +672,7 @@
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
-          <t>If either finance office can supply consolidated S&amp;W, replace the grey estimate.</t>
+          <t>If either finance office can supply consolidated S&amp;W, replace the light-blue estimate.</t>
         </is>
       </c>
     </row>
@@ -74289,7 +74289,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Northeastern, Northwestern, Penn, Stanford, Vanderbilt combine salaries and benefits. Northeastern and Northwestern use Form 990 S&amp;W; Vanderbilt uses the MD&amp;A expense chart. Penn and Stanford (grey markers) use S&amp;W = combined / 1.35, a 35% fringe benefit rate assumed per Northeastern's direction (74.1% S&amp;W share).</t>
+          <t>Northeastern, Northwestern, Penn, Stanford, Vanderbilt combine salaries and benefits. Northeastern and Northwestern use Form 990 S&amp;W; Vanderbilt uses the MD&amp;A expense chart. Penn and Stanford (light-blue markers) use S&amp;W = combined / 1.35, a 35% fringe benefit rate assumed per Northeastern's direction (74.1% S&amp;W share).</t>
         </is>
       </c>
       <c r="E18" s="27" t="inlineStr">

</xml_diff>

<commit_message>
Northeastern S&W tied to the audited salary-and-benefits line; check of the $1.3B claim added
Audited FY25 'Salary and benefits' $1,341.0M includes benefits. S&W = audited line x 80.54% S&W share from the Form 990 = $1,080M ($27.2K per student, 49.4% of core opex; x axis unchanged at $55.0K). Workbook adds compensation per student for all 14 schools and the numerator sensitivity for Northeastern.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCNX7EgSWHMHv9UtVBoXog
</commit_message>
<xml_diff>
--- a/nu-peer-slides/NU_peer_slides_backup.xlsx
+++ b/nu-peer-slides/NU_peer_slides_backup.xlsx
@@ -69780,12 +69780,12 @@
         </is>
       </c>
       <c r="C16" s="19">
-        <f>F16</f>
+        <f>E16*F16/G16</f>
         <v/>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>Form 990 (96.8% of audited combined)</t>
+          <t>audited combined x Form 990 S&amp;W share (80.5%)</t>
         </is>
       </c>
       <c r="E16" s="19" t="n">
@@ -69836,7 +69836,7 @@
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>Audited statements show 'Salary and benefits' combined ($1,341.0M). S&amp;W from Form 990 lines 5+6+7 (990 lines 5-10 are 96.8% of the audited combined line). Interest ($49.9M) is below the debt-note figure ($60.0M).</t>
+          <t>Audited statements show 'Salary and benefits' combined ($1,341.0M). S&amp;W = audited combined x the Form 990 S&amp;W share (lines 5+6+7 / lines 5-10 = 80.54%), because the 990 covers only 96.8% of the audited line; as filed the 990 S&amp;W is $1,045.1M (column F). See S3_Sensitivity G. Interest ($49.9M) is below the debt-note figure ($60.0M).</t>
         </is>
       </c>
     </row>
@@ -70023,7 +70023,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J53"/>
+  <dimension ref="A1:J84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -71175,6 +71175,607 @@
       <c r="A53" s="17" t="inlineStr">
         <is>
           <t>Harvard stays well above Northeastern ($26K) on every basis.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
+        <is>
+          <t>F. Salaries + benefits (combined compensation) per student: the like-for-like basis for the audited 'salary and benefits' line</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="5" t="inlineStr">
+        <is>
+          <t>Institution</t>
+        </is>
+      </c>
+      <c r="B56" s="5" t="inlineStr">
+        <is>
+          <t>Salaries + benefits ($)</t>
+        </is>
+      </c>
+      <c r="C56" s="5" t="inlineStr">
+        <is>
+          <t>Students used</t>
+        </is>
+      </c>
+      <c r="D56" s="5" t="inlineStr">
+        <is>
+          <t>Compensation per student</t>
+        </is>
+      </c>
+      <c r="E56" s="5" t="inlineStr">
+        <is>
+          <t>Rank low-to-high</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="9" t="inlineStr">
+        <is>
+          <t>Rice</t>
+        </is>
+      </c>
+      <c r="B57" s="19">
+        <f>S3_FY25!E5</f>
+        <v/>
+      </c>
+      <c r="C57" s="19">
+        <f>S3_FY25!M5</f>
+        <v/>
+      </c>
+      <c r="D57" s="11">
+        <f>B57/C57</f>
+        <v/>
+      </c>
+      <c r="E57" s="16">
+        <f>RANK(D57,D$57:D$70,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="9" t="inlineStr">
+        <is>
+          <t>Vanderbilt</t>
+        </is>
+      </c>
+      <c r="B58" s="19">
+        <f>S3_FY25!E6</f>
+        <v/>
+      </c>
+      <c r="C58" s="19">
+        <f>S3_FY25!M6</f>
+        <v/>
+      </c>
+      <c r="D58" s="11">
+        <f>B58/C58</f>
+        <v/>
+      </c>
+      <c r="E58" s="16">
+        <f>RANK(D58,D$57:D$70,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="9" t="inlineStr">
+        <is>
+          <t>Northwestern</t>
+        </is>
+      </c>
+      <c r="B59" s="19">
+        <f>S3_FY25!E7</f>
+        <v/>
+      </c>
+      <c r="C59" s="19">
+        <f>S3_FY25!M7</f>
+        <v/>
+      </c>
+      <c r="D59" s="11">
+        <f>B59/C59</f>
+        <v/>
+      </c>
+      <c r="E59" s="16">
+        <f>RANK(D59,D$57:D$70,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="9" t="inlineStr">
+        <is>
+          <t>Princeton</t>
+        </is>
+      </c>
+      <c r="B60" s="19">
+        <f>S3_FY25!E8</f>
+        <v/>
+      </c>
+      <c r="C60" s="19">
+        <f>S3_FY25!M8</f>
+        <v/>
+      </c>
+      <c r="D60" s="11">
+        <f>B60/C60</f>
+        <v/>
+      </c>
+      <c r="E60" s="16">
+        <f>RANK(D60,D$57:D$70,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="9" t="inlineStr">
+        <is>
+          <t>Harvard</t>
+        </is>
+      </c>
+      <c r="B61" s="19">
+        <f>S3_FY25!E9</f>
+        <v/>
+      </c>
+      <c r="C61" s="19">
+        <f>S3_FY25!M9</f>
+        <v/>
+      </c>
+      <c r="D61" s="11">
+        <f>B61/C61</f>
+        <v/>
+      </c>
+      <c r="E61" s="16">
+        <f>RANK(D61,D$57:D$70,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="9" t="inlineStr">
+        <is>
+          <t>Yale</t>
+        </is>
+      </c>
+      <c r="B62" s="19">
+        <f>S3_FY25!E10</f>
+        <v/>
+      </c>
+      <c r="C62" s="19">
+        <f>S3_FY25!M10</f>
+        <v/>
+      </c>
+      <c r="D62" s="11">
+        <f>B62/C62</f>
+        <v/>
+      </c>
+      <c r="E62" s="16">
+        <f>RANK(D62,D$57:D$70,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="9" t="inlineStr">
+        <is>
+          <t>Chicago</t>
+        </is>
+      </c>
+      <c r="B63" s="19">
+        <f>S3_FY25!E11</f>
+        <v/>
+      </c>
+      <c r="C63" s="19">
+        <f>S3_FY25!M11</f>
+        <v/>
+      </c>
+      <c r="D63" s="11">
+        <f>B63/C63</f>
+        <v/>
+      </c>
+      <c r="E63" s="16">
+        <f>RANK(D63,D$57:D$70,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="9" t="inlineStr">
+        <is>
+          <t>Duke</t>
+        </is>
+      </c>
+      <c r="B64" s="19">
+        <f>S3_FY25!E12</f>
+        <v/>
+      </c>
+      <c r="C64" s="19">
+        <f>S3_FY25!M12</f>
+        <v/>
+      </c>
+      <c r="D64" s="11">
+        <f>B64/C64</f>
+        <v/>
+      </c>
+      <c r="E64" s="16">
+        <f>RANK(D64,D$57:D$70,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="9" t="inlineStr">
+        <is>
+          <t>Emory</t>
+        </is>
+      </c>
+      <c r="B65" s="19">
+        <f>S3_FY25!E13</f>
+        <v/>
+      </c>
+      <c r="C65" s="19">
+        <f>S3_FY25!M13</f>
+        <v/>
+      </c>
+      <c r="D65" s="11">
+        <f>B65/C65</f>
+        <v/>
+      </c>
+      <c r="E65" s="16">
+        <f>RANK(D65,D$57:D$70,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="9" t="inlineStr">
+        <is>
+          <t>Penn</t>
+        </is>
+      </c>
+      <c r="B66" s="19">
+        <f>S3_FY25!E14</f>
+        <v/>
+      </c>
+      <c r="C66" s="19">
+        <f>S3_FY25!M14</f>
+        <v/>
+      </c>
+      <c r="D66" s="11">
+        <f>B66/C66</f>
+        <v/>
+      </c>
+      <c r="E66" s="16">
+        <f>RANK(D66,D$57:D$70,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="9" t="inlineStr">
+        <is>
+          <t>Stanford</t>
+        </is>
+      </c>
+      <c r="B67" s="19">
+        <f>S3_FY25!E15</f>
+        <v/>
+      </c>
+      <c r="C67" s="19">
+        <f>S3_FY25!M15</f>
+        <v/>
+      </c>
+      <c r="D67" s="11">
+        <f>B67/C67</f>
+        <v/>
+      </c>
+      <c r="E67" s="16">
+        <f>RANK(D67,D$57:D$70,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" s="9" t="inlineStr">
+        <is>
+          <t>Northeastern</t>
+        </is>
+      </c>
+      <c r="B68" s="19">
+        <f>S3_FY25!E16</f>
+        <v/>
+      </c>
+      <c r="C68" s="19">
+        <f>S3_FY25!M16</f>
+        <v/>
+      </c>
+      <c r="D68" s="11">
+        <f>B68/C68</f>
+        <v/>
+      </c>
+      <c r="E68" s="16">
+        <f>RANK(D68,D$57:D$70,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="9" t="inlineStr">
+        <is>
+          <t>Boston University</t>
+        </is>
+      </c>
+      <c r="B69" s="19">
+        <f>S3_FY25!E17</f>
+        <v/>
+      </c>
+      <c r="C69" s="19">
+        <f>S3_FY25!M17</f>
+        <v/>
+      </c>
+      <c r="D69" s="11">
+        <f>B69/C69</f>
+        <v/>
+      </c>
+      <c r="E69" s="16">
+        <f>RANK(D69,D$57:D$70,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="9" t="inlineStr">
+        <is>
+          <t>MIT</t>
+        </is>
+      </c>
+      <c r="B70" s="19">
+        <f>S3_FY25!E18</f>
+        <v/>
+      </c>
+      <c r="C70" s="19">
+        <f>S3_FY25!M18</f>
+        <v/>
+      </c>
+      <c r="D70" s="11">
+        <f>B70/C70</f>
+        <v/>
+      </c>
+      <c r="E70" s="16">
+        <f>RANK(D70,D$57:D$70,1)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" s="17" t="inlineStr">
+        <is>
+          <t>Northeastern is lowest on compensation per student as well ($33.7K vs Boston University $43.1K). Penn and Stanford combined figures are audited; only their S&amp;W split is estimated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="3" t="inlineStr">
+        <is>
+          <t>G. Northeastern: which numerator? (check of the '$1.3 billion / about 40,000 students' expectation)</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>Basis</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr">
+        <is>
+          <t>Amount ($)</t>
+        </is>
+      </c>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
+          <t>Per student (CDS 39,774)</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>Share of core operating expenses</t>
+        </is>
+      </c>
+      <c r="E75" s="5" t="inlineStr">
+        <is>
+          <t>Students x per-student (check)</t>
+        </is>
+      </c>
+      <c r="F75" s="5" t="inlineStr">
+        <is>
+          <t>Comparable with peers' S&amp;W?</t>
+        </is>
+      </c>
+      <c r="G75" s="5" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="9" t="inlineStr">
+        <is>
+          <t>Audited 'Salary and benefits' x Form 990 S&amp;W share (USED on slide)</t>
+        </is>
+      </c>
+      <c r="B76" s="19">
+        <f>S3_FY25!C16</f>
+        <v/>
+      </c>
+      <c r="C76" s="11">
+        <f>B76/S3_FY25!M16</f>
+        <v/>
+      </c>
+      <c r="D76" s="20">
+        <f>B76/S3_FY25!L16</f>
+        <v/>
+      </c>
+      <c r="E76" s="19">
+        <f>S3_FY25!M16*C76</f>
+        <v/>
+      </c>
+      <c r="F76" s="9" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="G76" s="9" t="inlineStr">
+        <is>
+          <t>Audited FY25 combined line x 80.54%; same consolidated scope as core operating expenses</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" s="9" t="inlineStr">
+        <is>
+          <t>Form 990 S&amp;W as filed (lines 5+6+7)</t>
+        </is>
+      </c>
+      <c r="B77" s="19">
+        <f>S3_FY25!F16</f>
+        <v/>
+      </c>
+      <c r="C77" s="11">
+        <f>B77/S3_FY25!M16</f>
+        <v/>
+      </c>
+      <c r="D77" s="20">
+        <f>B77/S3_FY25!L16</f>
+        <v/>
+      </c>
+      <c r="E77" s="19">
+        <f>S3_FY25!M16*C77</f>
+        <v/>
+      </c>
+      <c r="F77" s="9" t="inlineStr">
+        <is>
+          <t>Yes, narrower scope</t>
+        </is>
+      </c>
+      <c r="G77" s="9" t="inlineStr">
+        <is>
+          <t>The value used in the first FY25 draft; university-only, 96.8% of the audited line's scope</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" s="9" t="inlineStr">
+        <is>
+          <t>Audited combined line / 1.35 (35% fringe, as for Penn and Stanford)</t>
+        </is>
+      </c>
+      <c r="B78" s="19">
+        <f>S3_FY25!E16/1.35</f>
+        <v/>
+      </c>
+      <c r="C78" s="11">
+        <f>B78/S3_FY25!M16</f>
+        <v/>
+      </c>
+      <c r="D78" s="20">
+        <f>B78/S3_FY25!L16</f>
+        <v/>
+      </c>
+      <c r="E78" s="19">
+        <f>S3_FY25!M16*C78</f>
+        <v/>
+      </c>
+      <c r="F78" s="9" t="inlineStr">
+        <is>
+          <t>Yes (assumption)</t>
+        </is>
+      </c>
+      <c r="G78" s="9" t="inlineStr">
+        <is>
+          <t>Northeastern's own 990 fringe rate is 24.2%, below 35%</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" s="9" t="inlineStr">
+        <is>
+          <t>Audited 'Salary and benefits' (combined)</t>
+        </is>
+      </c>
+      <c r="B79" s="19">
+        <f>S3_FY25!E16</f>
+        <v/>
+      </c>
+      <c r="C79" s="11">
+        <f>B79/S3_FY25!M16</f>
+        <v/>
+      </c>
+      <c r="D79" s="20">
+        <f>B79/S3_FY25!L16</f>
+        <v/>
+      </c>
+      <c r="E79" s="19">
+        <f>S3_FY25!M16*C79</f>
+        <v/>
+      </c>
+      <c r="F79" s="9" t="inlineStr">
+        <is>
+          <t>NO: includes benefits</t>
+        </is>
+      </c>
+      <c r="G79" s="9" t="inlineStr">
+        <is>
+          <t>This is the roughly $1.3 billion; it is salaries AND benefits (about $261M of benefits)</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" s="9" t="inlineStr">
+        <is>
+          <t>Form 990 lines 5-10 (combined, university only)</t>
+        </is>
+      </c>
+      <c r="B80" s="19">
+        <f>S3_FY25!G16</f>
+        <v/>
+      </c>
+      <c r="C80" s="11">
+        <f>B80/S3_FY25!M16</f>
+        <v/>
+      </c>
+      <c r="D80" s="20">
+        <f>B80/S3_FY25!L16</f>
+        <v/>
+      </c>
+      <c r="E80" s="19">
+        <f>S3_FY25!M16*C80</f>
+        <v/>
+      </c>
+      <c r="F80" s="9" t="inlineStr">
+        <is>
+          <t>NO: includes benefits</t>
+        </is>
+      </c>
+      <c r="G80" s="9" t="inlineStr">
+        <is>
+          <t>Also about $1.3 billion; 3.2% below the audited line</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="3" t="inlineStr">
+        <is>
+          <t>Check: 40,000 students x S&amp;W per student used</t>
+        </is>
+      </c>
+      <c r="B82" s="19">
+        <f>40000*C76</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
+          <t>Audited 'Salary and benefits' less that product = implied benefits</t>
+        </is>
+      </c>
+      <c r="B83" s="19">
+        <f>S3_FY25!E16-B82</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="17" t="inlineStr">
+        <is>
+          <t>So 40,000 x $27K is about $1.09 billion of salaries and wages; the roughly $1.3 billion in the statements includes about $0.25 billion of benefits.</t>
         </is>
       </c>
     </row>
@@ -73879,7 +74480,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -74364,7 +74965,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>CDS 39,774 (used, per Northeastern's direction) -&gt; S&amp;W per student $26.3K; IPEDS-style 32,553 -&gt; $32.1K; Facts and Figures 48,812 -&gt; $21.4K. Northeastern is lowest in the peer set on all three (S3_Sensitivity A, B).</t>
+          <t>CDS 39,774 (used, per Northeastern's direction) -&gt; S&amp;W per student $27.2K; IPEDS-style 32,553 -&gt; $33.2K; Facts and Figures 48,812 -&gt; $22.1K. Northeastern is lowest in the peer set on all three (S3_Sensitivity A, B).</t>
         </is>
       </c>
       <c r="E21" s="27" t="inlineStr">
@@ -74414,12 +75015,12 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Form 990 (university) lines 5-10 are 96.8% of the audited combined line; S&amp;W may be understated by about 3% against the consolidated core expenses.</t>
+          <t>Form 990 (university only) lines 5-10 are 96.8% of the audited combined line. To keep S&amp;W on the same consolidated scope as core operating expenses, S&amp;W = audited 'Salary and benefits' $1,341.0M x the 990 S&amp;W share of lines 5-10 (80.54%) = $1,080.1M, which moves the point from $26.3K and 47.8% (990 as filed) to $27.2K and 49.4%. The x value ($55.0K) is unchanged (S3_Sensitivity G).</t>
         </is>
       </c>
       <c r="E23" s="27" t="inlineStr">
         <is>
-          <t>Caveat</t>
+          <t>Handled</t>
         </is>
       </c>
     </row>
@@ -74434,17 +75035,17 @@
       </c>
       <c r="C24" s="4" t="inlineStr">
         <is>
-          <t>FY23 to FY24 comparability</t>
+          <t>Northeastern: '40,000 students x S&amp;W per student = about $1.3 billion'</t>
         </is>
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Duke's FY24 includes the July 1, 2023 physician-practice acquisition (S&amp;W +29.5%); FY25 is unaffected. Rice's FY25 scholarship presentation changed (total and core not strictly comparable with FY24). Emory FY25 includes three months of Houston Healthcare. Northeastern FY25 includes two weeks of Marymount Manhattan College.</t>
-        </is>
-      </c>
-      <c r="E24" s="27" t="inlineStr">
-        <is>
-          <t>Info</t>
+          <t>Does not hold for S&amp;W. The audited statements show one line, 'Salary and benefits' $1,341.0M, which includes benefits (the Form 990 puts benefits at $252M, 24.2% of S&amp;W). 39,774 x $27.2K = $1,080M of S&amp;W. $1,341.0M / 39,774 = $33.7K is salary-plus-benefits per student: not comparable with the peers' S&amp;W, but on that like-for-like basis Northeastern is still lowest (Boston University $43.1K; S3_Sensitivity F, G).</t>
+        </is>
+      </c>
+      <c r="E24" s="28" t="inlineStr">
+        <is>
+          <t>Finding</t>
         </is>
       </c>
     </row>
@@ -74459,17 +75060,17 @@
       </c>
       <c r="C25" s="4" t="inlineStr">
         <is>
-          <t>Entities inside the numbers</t>
+          <t>FY23 to FY24 comparability</t>
         </is>
       </c>
       <c r="D25" s="4" t="inlineStr">
         <is>
-          <t>Consolidated: hospitals at Chicago, Duke, Emory, Penn, Stanford; Lincoln Laboratory (MIT), Plasma Physics Laboratory (Princeton), SLAC (Stanford). Not consolidated: Northwestern Medicine, VUMC, Yale New Haven Hospital, Boston Medical Center, Argonne, Fermilab. Footnoted on the slide.</t>
+          <t>Duke's FY24 includes the July 1, 2023 physician-practice acquisition (S&amp;W +29.5%); FY25 is unaffected. Rice's FY25 scholarship presentation changed (total and core not strictly comparable with FY24). Emory FY25 includes three months of Houston Healthcare. Northeastern FY25 includes two weeks of Marymount Manhattan College.</t>
         </is>
       </c>
       <c r="E25" s="27" t="inlineStr">
         <is>
-          <t>Handled</t>
+          <t>Info</t>
         </is>
       </c>
     </row>
@@ -74484,17 +75085,17 @@
       </c>
       <c r="C26" s="4" t="inlineStr">
         <is>
-          <t>Arithmetic</t>
+          <t>Entities inside the numbers</t>
         </is>
       </c>
       <c r="D26" s="4" t="inlineStr">
         <is>
-          <t>For every school, core = total - depreciation - amortization - interest (formula), S&amp;W per student = x * y (column Q = 0), and the natural-classification lines sum to total operating expenses in every year (as reported by the extraction). Key rows for Northeastern, BU and MIT re-checked against the PDFs.</t>
+          <t>Consolidated: hospitals at Chicago, Duke, Emory, Penn, Stanford; Lincoln Laboratory (MIT), Plasma Physics Laboratory (Princeton), SLAC (Stanford). Not consolidated: Northwestern Medicine, VUMC, Yale New Haven Hospital, Boston Medical Center, Argonne, Fermilab. Footnoted on the slide.</t>
         </is>
       </c>
       <c r="E26" s="27" t="inlineStr">
         <is>
-          <t>Pass</t>
+          <t>Handled</t>
         </is>
       </c>
     </row>
@@ -74509,12 +75110,12 @@
       </c>
       <c r="C27" s="4" t="inlineStr">
         <is>
-          <t>Harvard</t>
+          <t>Arithmetic</t>
         </is>
       </c>
       <c r="D27" s="4" t="inlineStr">
         <is>
-          <t>Added from the FY25 audited Financial Report supplied by Northeastern (finance.harvard.edu blocks automated access). S&amp;W $2,758.6M and benefits $755.9M are separate lines (benefits 27.4% of S&amp;W); total operating expenses $6,794.4M - depreciation $459.0M - interest $262.5M = core $6,072.8M; the nine natural-classification lines sum to the total in FY25 and FY24 (Note 17). S&amp;W share 45.4%; 24,819 students (CDS + Extension School degree students) -&gt; $111K S&amp;W per student, below Princeton ($128K) with a lower S&amp;W share. No hospital consolidated.</t>
+          <t>For every school, core = total - depreciation - amortization - interest (formula), S&amp;W per student = x * y (column Q = 0), and the natural-classification lines sum to total operating expenses in every year (as reported by the extraction). Key rows for Northeastern, BU and MIT re-checked against the PDFs.</t>
         </is>
       </c>
       <c r="E27" s="27" t="inlineStr">
@@ -74534,17 +75135,17 @@
       </c>
       <c r="C28" s="4" t="inlineStr">
         <is>
-          <t>Harvard student count</t>
+          <t>Harvard</t>
         </is>
       </c>
       <c r="D28" s="4" t="inlineStr">
         <is>
-          <t>Expenses include the Division of Continuing Education (Harvard Extension School) but the Common Data Set excludes it. Students on the slide = CDS 21,189 + Extension degree students 3,630 (621 undergraduate + 3,009 graduate, Harvard OIRA Fact Book 2025-26, fall 2024) = 24,819 -&gt; $111K S&amp;W per student. Alternatives (S3_Sensitivity E): CDS only 21,189 -&gt; $130K; Fact Book distinct total 24,519 -&gt; $113K; IPEDS fall 2023 30,386 (adds non-degree course takers) -&gt; $91K. Harvard's own report: 'approximately 7,000 undergraduate and 14,000 graduate students' (Note 1). No effect on Northeastern's ranking.</t>
+          <t>Added from the FY25 audited Financial Report supplied by Northeastern (finance.harvard.edu blocks automated access). S&amp;W $2,758.6M and benefits $755.9M are separate lines (benefits 27.4% of S&amp;W); total operating expenses $6,794.4M - depreciation $459.0M - interest $262.5M = core $6,072.8M; the nine natural-classification lines sum to the total in FY25 and FY24 (Note 17). S&amp;W share 45.4%; 24,819 students (CDS + Extension School degree students) -&gt; $111K S&amp;W per student, below Princeton ($128K) with a lower S&amp;W share. No hospital consolidated.</t>
         </is>
       </c>
       <c r="E28" s="27" t="inlineStr">
         <is>
-          <t>Handled / caveat</t>
+          <t>Pass</t>
         </is>
       </c>
     </row>
@@ -74559,17 +75160,17 @@
       </c>
       <c r="C29" s="4" t="inlineStr">
         <is>
-          <t>Harvard FY23 calibration</t>
+          <t>Harvard student count</t>
         </is>
       </c>
       <c r="D29" s="4" t="inlineStr">
         <is>
-          <t>FY23 Financial Report (supplied by Northeastern): original slide S&amp;W $2,421,076K equals the audited FY23 salaries and wages line to the dollar; the original 'core opex' $5,911,797K equals audited FY23 total operating expenses to the dollar. On the stated definition FY23 core is $5,278,398K (total less depreciation $424,809K and interest $208,590K), so the original x value was 12.0% too high. Same finding as for the other schools. Original 21,400 students = the report's 'approximately 7,200 undergraduate and 14,200 graduate' (Note 1). S&amp;W grew 13.9% FY23 to FY25 ($2,421M to $2,759M).</t>
+          <t>Expenses include the Division of Continuing Education (Harvard Extension School) but the Common Data Set excludes it. Students on the slide = CDS 21,189 + Extension degree students 3,630 (621 undergraduate + 3,009 graduate, Harvard OIRA Fact Book 2025-26, fall 2024) = 24,819 -&gt; $111K S&amp;W per student. Alternatives (S3_Sensitivity E): CDS only 21,189 -&gt; $130K; Fact Book distinct total 24,519 -&gt; $113K; IPEDS fall 2023 30,386 (adds non-degree course takers) -&gt; $91K. Harvard's own report: 'approximately 7,000 undergraduate and 14,000 graduate students' (Note 1). No effect on Northeastern's ranking.</t>
         </is>
       </c>
       <c r="E29" s="27" t="inlineStr">
         <is>
-          <t>Pass / finding</t>
+          <t>Handled / caveat</t>
         </is>
       </c>
     </row>
@@ -74584,15 +75185,40 @@
       </c>
       <c r="C30" s="4" t="inlineStr">
         <is>
+          <t>Harvard FY23 calibration</t>
+        </is>
+      </c>
+      <c r="D30" s="4" t="inlineStr">
+        <is>
+          <t>FY23 Financial Report (supplied by Northeastern): original slide S&amp;W $2,421,076K equals the audited FY23 salaries and wages line to the dollar; the original 'core opex' $5,911,797K equals audited FY23 total operating expenses to the dollar. On the stated definition FY23 core is $5,278,398K (total less depreciation $424,809K and interest $208,590K), so the original x value was 12.0% too high. Same finding as for the other schools. Original 21,400 students = the report's 'approximately 7,200 undergraduate and 14,200 graduate' (Note 1). S&amp;W grew 13.9% FY23 to FY25 ($2,421M to $2,759M).</t>
+        </is>
+      </c>
+      <c r="E30" s="27" t="inlineStr">
+        <is>
+          <t>Pass / finding</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="B31" s="4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="C31" s="4" t="inlineStr">
+        <is>
           <t>Original chart construction</t>
         </is>
       </c>
-      <c r="D30" s="4" t="inlineStr">
+      <c r="D31" s="4" t="inlineStr">
         <is>
           <t>The original plotted only the eight iso-lines; logos were hand-placed pictures, so positions did not come from data, and Stanford's x-value exceeded the axis maximum. Rebuilt with real data points.</t>
         </is>
       </c>
-      <c r="E30" s="27" t="inlineStr">
+      <c r="E31" s="27" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>

</xml_diff>

<commit_message>
Slide 3: y axis 30-60% without gridlines, Northeastern fringe rate 33%, cleaner label layout
Northeastern S&W = audited salary and benefits / 1.33 (33% fringe rate per Northeastern): $1,008M, $25.4K per student, 46.1% of core opex. The Form 990 basis is kept in the workbook for reference. Labels in the crowded left cluster have explicit positions and every label has a non-crossing leader line.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FCNX7EgSWHMHv9UtVBoXog
</commit_message>
<xml_diff>
--- a/nu-peer-slides/NU_peer_slides_backup.xlsx
+++ b/nu-peer-slides/NU_peer_slides_backup.xlsx
@@ -68929,7 +68929,20 @@
       </c>
       <c r="F3" s="17" t="inlineStr">
         <is>
-          <t>&lt;- input: S&amp;W = combined salaries + benefits / (1 + rate). Change it and the estimates, slide-3 inputs and sensitivities update here.</t>
+          <t>&lt;- input (Penn, Stanford): S&amp;W = combined / (1 + rate)</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>Northeastern fringe rate</t>
+        </is>
+      </c>
+      <c r="L3" s="18" t="n">
+        <v>0.33</v>
+      </c>
+      <c r="M3" s="17" t="inlineStr">
+        <is>
+          <t>&lt;- input, per Northeastern</t>
         </is>
       </c>
     </row>
@@ -69780,12 +69793,12 @@
         </is>
       </c>
       <c r="C16" s="19">
-        <f>E16*F16/G16</f>
+        <f>E16/(1+$L$3)</f>
         <v/>
       </c>
       <c r="D16" s="9" t="inlineStr">
         <is>
-          <t>audited combined x Form 990 S&amp;W share (80.5%)</t>
+          <t>audited combined / (1 + 33% fringe rate)</t>
         </is>
       </c>
       <c r="E16" s="19" t="n">
@@ -69836,7 +69849,7 @@
       </c>
       <c r="S16" s="4" t="inlineStr">
         <is>
-          <t>Audited statements show 'Salary and benefits' combined ($1,341.0M). S&amp;W = audited combined x the Form 990 S&amp;W share (lines 5+6+7 / lines 5-10 = 80.54%), because the 990 covers only 96.8% of the audited line; as filed the 990 S&amp;W is $1,045.1M (column F). See S3_Sensitivity G. Interest ($49.9M) is below the debt-note figure ($60.0M).</t>
+          <t>Audited statements show 'Salary and benefits' combined ($1,341.0M). S&amp;W = combined / (1 + 33% fringe rate, per Northeastern; input L3). Columns F-G (Form 990, university only, 96.8% of the audited line) are for reference: as filed the 990 shows S&amp;W $1,045.1M. See S3_Sensitivity G. Interest ($49.9M) is below the debt-note figure ($60.0M).</t>
         </is>
       </c>
     </row>
@@ -70023,7 +70036,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J84"/>
+  <dimension ref="A1:J85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -71588,7 +71601,7 @@
     <row r="76">
       <c r="A76" s="9" t="inlineStr">
         <is>
-          <t>Audited 'Salary and benefits' x Form 990 S&amp;W share (USED on slide)</t>
+          <t>Audited 'Salary and benefits' / (1 + 33% fringe rate, per Northeastern) (USED on slide)</t>
         </is>
       </c>
       <c r="B76" s="19">
@@ -71614,18 +71627,18 @@
       </c>
       <c r="G76" s="9" t="inlineStr">
         <is>
-          <t>Audited FY25 combined line x 80.54%; same consolidated scope as core operating expenses</t>
+          <t>Fringe rate provided by Northeastern (S3_FY25 cell L3); same consolidated scope as core operating expenses</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="9" t="inlineStr">
         <is>
-          <t>Form 990 S&amp;W as filed (lines 5+6+7)</t>
+          <t>Audited combined x Form 990 S&amp;W share (80.5%)</t>
         </is>
       </c>
       <c r="B77" s="19">
-        <f>S3_FY25!F16</f>
+        <f>S3_FY25!E16*S3_FY25!F16/S3_FY25!G16</f>
         <v/>
       </c>
       <c r="C77" s="11">
@@ -71642,23 +71655,23 @@
       </c>
       <c r="F77" s="9" t="inlineStr">
         <is>
-          <t>Yes, narrower scope</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="G77" s="9" t="inlineStr">
         <is>
-          <t>The value used in the first FY25 draft; university-only, 96.8% of the audited line's scope</t>
+          <t>Implied fringe rate 24.2% from the Form 990; used in the previous draft</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="9" t="inlineStr">
         <is>
-          <t>Audited combined line / 1.35 (35% fringe, as for Penn and Stanford)</t>
+          <t>Form 990 S&amp;W as filed (lines 5+6+7)</t>
         </is>
       </c>
       <c r="B78" s="19">
-        <f>S3_FY25!E16/1.35</f>
+        <f>S3_FY25!F16</f>
         <v/>
       </c>
       <c r="C78" s="11">
@@ -71675,23 +71688,23 @@
       </c>
       <c r="F78" s="9" t="inlineStr">
         <is>
-          <t>Yes (assumption)</t>
+          <t>Yes, narrower scope</t>
         </is>
       </c>
       <c r="G78" s="9" t="inlineStr">
         <is>
-          <t>Northeastern's own 990 fringe rate is 24.2%, below 35%</t>
+          <t>University only; 96.8% of the audited line's scope; used in the first FY25 draft</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="9" t="inlineStr">
         <is>
-          <t>Audited 'Salary and benefits' (combined)</t>
+          <t>Audited combined line / 1.35 (35% fringe, as for Penn and Stanford)</t>
         </is>
       </c>
       <c r="B79" s="19">
-        <f>S3_FY25!E16</f>
+        <f>S3_FY25!E16/1.35</f>
         <v/>
       </c>
       <c r="C79" s="11">
@@ -71708,23 +71721,23 @@
       </c>
       <c r="F79" s="9" t="inlineStr">
         <is>
-          <t>NO: includes benefits</t>
+          <t>Yes (assumption)</t>
         </is>
       </c>
       <c r="G79" s="9" t="inlineStr">
         <is>
-          <t>This is the roughly $1.3 billion; it is salaries AND benefits (about $261M of benefits)</t>
+          <t>Northeastern's rate is 33%, so this leans low</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="9" t="inlineStr">
         <is>
-          <t>Form 990 lines 5-10 (combined, university only)</t>
+          <t>Audited 'Salary and benefits' (combined)</t>
         </is>
       </c>
       <c r="B80" s="19">
-        <f>S3_FY25!G16</f>
+        <f>S3_FY25!E16</f>
         <v/>
       </c>
       <c r="C80" s="11">
@@ -71746,36 +71759,69 @@
       </c>
       <c r="G80" s="9" t="inlineStr">
         <is>
+          <t>This is the roughly $1.3 billion; it is salaries AND benefits (about $333M of benefits at a 33% fringe rate)</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="9" t="inlineStr">
+        <is>
+          <t>Form 990 lines 5-10 (combined, university only)</t>
+        </is>
+      </c>
+      <c r="B81" s="19">
+        <f>S3_FY25!G16</f>
+        <v/>
+      </c>
+      <c r="C81" s="11">
+        <f>B81/S3_FY25!M16</f>
+        <v/>
+      </c>
+      <c r="D81" s="20">
+        <f>B81/S3_FY25!L16</f>
+        <v/>
+      </c>
+      <c r="E81" s="19">
+        <f>S3_FY25!M16*C81</f>
+        <v/>
+      </c>
+      <c r="F81" s="9" t="inlineStr">
+        <is>
+          <t>NO: includes benefits</t>
+        </is>
+      </c>
+      <c r="G81" s="9" t="inlineStr">
+        <is>
           <t>Also about $1.3 billion; 3.2% below the audited line</t>
         </is>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="3" t="inlineStr">
-        <is>
-          <t>Check: 40,000 students x S&amp;W per student used</t>
-        </is>
-      </c>
-      <c r="B82" s="19">
-        <f>40000*C76</f>
-        <v/>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="3" t="inlineStr">
         <is>
+          <t>Check: 40,000 students x S&amp;W per student used</t>
+        </is>
+      </c>
+      <c r="B83" s="19">
+        <f>40000*C76</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
+        <is>
           <t>Audited 'Salary and benefits' less that product = implied benefits</t>
         </is>
       </c>
-      <c r="B83" s="19">
-        <f>S3_FY25!E16-B82</f>
-        <v/>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="17" t="inlineStr">
-        <is>
-          <t>So 40,000 x $27K is about $1.09 billion of salaries and wages; the roughly $1.3 billion in the statements includes about $0.25 billion of benefits.</t>
+      <c r="B84" s="19">
+        <f>S3_FY25!E16-B83</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="17" t="inlineStr">
+        <is>
+          <t>So 40,000 x $25K is about $1.0 billion of salaries and wages; the roughly $1.3 billion in the statements includes about $0.3 billion of benefits.</t>
         </is>
       </c>
     </row>
@@ -74890,7 +74936,7 @@
       </c>
       <c r="D18" s="4" t="inlineStr">
         <is>
-          <t>Northeastern, Northwestern, Penn, Stanford, Vanderbilt combine salaries and benefits. Northeastern and Northwestern use Form 990 S&amp;W; Vanderbilt uses the MD&amp;A expense chart. Penn and Stanford (light-blue markers) use S&amp;W = combined / 1.35, a 35% fringe benefit rate assumed per Northeastern's direction (74.1% S&amp;W share).</t>
+          <t>Northeastern, Northwestern, Penn, Stanford, Vanderbilt combine salaries and benefits. Northeastern uses its 33% fringe benefit rate (S&amp;W = combined / 1.33, per Northeastern); Northwestern uses Form 990 S&amp;W; Vanderbilt uses the MD&amp;A expense chart. Penn and Stanford (light-blue markers) use S&amp;W = combined / 1.35, a 35% fringe benefit rate assumed per Northeastern's direction (74.1% S&amp;W share).</t>
         </is>
       </c>
       <c r="E18" s="27" t="inlineStr">
@@ -74965,7 +75011,7 @@
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>CDS 39,774 (used, per Northeastern's direction) -&gt; S&amp;W per student $27.2K; IPEDS-style 32,553 -&gt; $33.2K; Facts and Figures 48,812 -&gt; $22.1K. Northeastern is lowest in the peer set on all three (S3_Sensitivity A, B).</t>
+          <t>CDS 39,774 (used, per Northeastern's direction) -&gt; S&amp;W per student $25.4K; IPEDS-style 32,553 -&gt; $31.0K; Facts and Figures 48,812 -&gt; $20.7K. Northeastern is lowest in the peer set on all three (S3_Sensitivity A, B).</t>
         </is>
       </c>
       <c r="E21" s="27" t="inlineStr">
@@ -75010,17 +75056,17 @@
       </c>
       <c r="C23" s="4" t="inlineStr">
         <is>
-          <t>Northeastern S&amp;W scope</t>
+          <t>Northeastern S&amp;W basis</t>
         </is>
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>Form 990 (university only) lines 5-10 are 96.8% of the audited combined line. To keep S&amp;W on the same consolidated scope as core operating expenses, S&amp;W = audited 'Salary and benefits' $1,341.0M x the 990 S&amp;W share of lines 5-10 (80.54%) = $1,080.1M, which moves the point from $26.3K and 47.8% (990 as filed) to $27.2K and 49.4%. The x value ($55.0K) is unchanged (S3_Sensitivity G).</t>
+          <t>Northeastern's fringe benefit rate is 33% (per Northeastern), so S&amp;W = audited 'Salary and benefits' $1,341.0M / 1.33 = $1,008.3M ($25.4K per student, 46.1% of core operating expenses); benefits are the remaining $332.7M. The x value ($55.0K) is unchanged. For reference, the Form 990 (university only, 96.8% of the audited line) shows S&amp;W $1,045.1M and a 24.2% fringe rate on lines 5-10; the earlier drafts used the 990 as filed ($26.3K, 47.8%) and then scaled to the audited line ($27.2K, 49.4%) (S3_Sensitivity G).</t>
         </is>
       </c>
       <c r="E23" s="27" t="inlineStr">
         <is>
-          <t>Handled</t>
+          <t>Decided</t>
         </is>
       </c>
     </row>
@@ -75040,7 +75086,7 @@
       </c>
       <c r="D24" s="4" t="inlineStr">
         <is>
-          <t>Does not hold for S&amp;W. The audited statements show one line, 'Salary and benefits' $1,341.0M, which includes benefits (the Form 990 puts benefits at $252M, 24.2% of S&amp;W). 39,774 x $27.2K = $1,080M of S&amp;W. $1,341.0M / 39,774 = $33.7K is salary-plus-benefits per student: not comparable with the peers' S&amp;W, but on that like-for-like basis Northeastern is still lowest (Boston University $43.1K; S3_Sensitivity F, G).</t>
+          <t>Does not hold for S&amp;W. The audited statements show one line, 'Salary and benefits' $1,341.0M, which includes benefits. At Northeastern's 33% fringe rate S&amp;W is $1,008M and benefits $333M: 39,774 x $25.4K = $1,008M. $1,341.0M / 39,774 = $33.7K is salary-plus-benefits per student: not comparable with the peers' S&amp;W, but on that like-for-like basis Northeastern is still lowest (Boston University $43.1K; S3_Sensitivity F, G).</t>
         </is>
       </c>
       <c r="E24" s="28" t="inlineStr">

</xml_diff>